<commit_message>
data: extend VIX history to 2026-08-04 and refresh m30 sample
</commit_message>
<xml_diff>
--- a/04_结果/示例审批/两基金_m30新版式示例_公式说明版.xlsx
+++ b/04_结果/示例审批/两基金_m30新版式示例_公式说明版.xlsx
@@ -2106,14 +2106,14 @@
         <v/>
       </c>
       <c r="V14" s="5" t="n">
-        <v/>
+        <v>16.5</v>
       </c>
       <c r="W14" s="5">
         <f>IF(COUNT(V14:V15)=2,(V14/V15-1)*100,"")</f>
         <v/>
       </c>
       <c r="X14" s="5" t="n">
-        <v/>
+        <v>4.0353</v>
       </c>
       <c r="Y14" s="5" t="inlineStr"/>
       <c r="Z14" s="5" t="inlineStr"/>
@@ -2207,14 +2207,14 @@
         <v/>
       </c>
       <c r="V15" s="5" t="n">
-        <v/>
+        <v>15.86</v>
       </c>
       <c r="W15" s="5">
         <f>IF(COUNT(V15:V16)=2,(V15/V16-1)*100,"")</f>
         <v/>
       </c>
       <c r="X15" s="5" t="n">
-        <v/>
+        <v>-0.8129999999999999</v>
       </c>
       <c r="Y15" s="5">
         <f>IF(AND(X15&gt;$Y$11,C15&lt;=$Y$12),C14,"")</f>
@@ -2326,14 +2326,14 @@
         <v/>
       </c>
       <c r="V16" s="5" t="n">
-        <v/>
+        <v>15.99</v>
       </c>
       <c r="W16" s="5">
         <f>IF(COUNT(V16:V17)=2,(V16/V17-1)*100,"")</f>
         <v/>
       </c>
       <c r="X16" s="5" t="n">
-        <v/>
+        <v>-6.4365</v>
       </c>
       <c r="Y16" s="5">
         <f>IF(AND(X16&gt;$Y$11,C16&lt;=$Y$12),C15,"")</f>
@@ -2445,14 +2445,14 @@
         <v/>
       </c>
       <c r="V17" s="5" t="n">
-        <v/>
+        <v>17.09</v>
       </c>
       <c r="W17" s="5">
         <f>IF(COUNT(V17:V18)=2,(V17/V18-1)*100,"")</f>
         <v/>
       </c>
       <c r="X17" s="5" t="n">
-        <v/>
+        <v>-17.2798</v>
       </c>
       <c r="Y17" s="5">
         <f>IF(AND(X17&gt;$Y$11,C17&lt;=$Y$12),C16,"")</f>
@@ -2564,14 +2564,14 @@
         <v/>
       </c>
       <c r="V18" s="5" t="n">
-        <v/>
+        <v>20.66</v>
       </c>
       <c r="W18" s="5">
         <f>IF(COUNT(V18:V19)=2,(V18/V19-1)*100,"")</f>
         <v/>
       </c>
       <c r="X18" s="5" t="n">
-        <v/>
+        <v>13.4541</v>
       </c>
       <c r="Y18" s="5">
         <f>IF(AND(X18&gt;$Y$11,C18&lt;=$Y$12),C17,"")</f>
@@ -2683,14 +2683,14 @@
         <v/>
       </c>
       <c r="V19" s="5" t="n">
-        <v/>
+        <v>18.21</v>
       </c>
       <c r="W19" s="5">
         <f>IF(COUNT(V19:V20)=2,(V19/V20-1)*100,"")</f>
         <v/>
       </c>
       <c r="X19" s="5" t="n">
-        <v/>
+        <v>-2.4638</v>
       </c>
       <c r="Y19" s="5">
         <f>IF(AND(X19&gt;$Y$11,C19&lt;=$Y$12),C18,"")</f>
@@ -2802,14 +2802,14 @@
         <v/>
       </c>
       <c r="V20" s="5" t="n">
-        <v/>
+        <v>18.67</v>
       </c>
       <c r="W20" s="5">
         <f>IF(COUNT(V20:V21)=2,(V20/V21-1)*100,"")</f>
         <v/>
       </c>
       <c r="X20" s="5" t="n">
-        <v/>
+        <v>0.4844</v>
       </c>
       <c r="Y20" s="5">
         <f>IF(AND(X20&gt;$Y$11,C20&lt;=$Y$12),C19,"")</f>

</xml_diff>

<commit_message>
feat: round returns to 4 decimals with percent display
</commit_message>
<xml_diff>
--- a/04_结果/示例审批/两基金_m30新版式示例_公式说明版.xlsx
+++ b/04_结果/示例审批/两基金_m30新版式示例_公式说明版.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000&quot;%&quot;"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -515,7 +515,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   =IF(COUNT(B15:B16)=2,(B15/B16-1)*100,"")</t>
+          <t xml:space="preserve">   =IF(COUNT(B15:B16)=2,ROUND((B15/B16-1)*100,4),"")</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   所有回报率均以百分比显示并保留4位小数。</t>
+          <t xml:space="preserve">   所有回报率均以百分比显示并保留4位小数（公式 ROUND 到4位，显示格式 0.0000%）。</t>
         </is>
       </c>
     </row>
@@ -3427,11 +3427,11 @@
         <v>194.03</v>
       </c>
       <c r="D15" s="6">
-        <f>IF(COUNT(B15:B16)=2,(B15/B16-1)*100,"")</f>
+        <f>IF(COUNT(B15:B16)=2,ROUND((B15/B16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E15" s="6">
-        <f>IF(COUNT(C15:C16)=2,(C15/C16-1)*100,"")</f>
+        <f>IF(COUNT(C15:C16)=2,ROUND((C15/C16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F15" s="5" t="n">
@@ -3555,42 +3555,42 @@
         <v>112.04</v>
       </c>
       <c r="AT15" s="6">
-        <f>IF(COUNT(J15:J16)=2,(J15/J16-1)*100,"")</f>
+        <f>IF(COUNT(J15:J16)=2,ROUND((J15/J16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU15" s="6">
-        <f>IF(COUNT(O15:O16)=2,(O15/O16-1)*100,"")</f>
+        <f>IF(COUNT(O15:O16)=2,ROUND((O15/O16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV15" s="6">
-        <f>IF(COUNT(T15:T16)=2,(T15/T16-1)*100,"")</f>
+        <f>IF(COUNT(T15:T16)=2,ROUND((T15/T16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW15" s="6">
-        <f>IF(COUNT(Y15:Y16)=2,(Y15/Y16-1)*100,"")</f>
+        <f>IF(COUNT(Y15:Y16)=2,ROUND((Y15/Y16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX15" s="6">
-        <f>IF(COUNT(AD15:AD16)=2,(AD15/AD16-1)*100,"")</f>
+        <f>IF(COUNT(AD15:AD16)=2,ROUND((AD15/AD16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY15" s="6">
-        <f>IF(COUNT(AI15:AI16)=2,(AI15/AI16-1)*100,"")</f>
+        <f>IF(COUNT(AI15:AI16)=2,ROUND((AI15/AI16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ15" s="6">
-        <f>IF(COUNT(AN15:AN16)=2,(AN15/AN16-1)*100,"")</f>
+        <f>IF(COUNT(AN15:AN16)=2,ROUND((AN15/AN16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA15" s="6">
-        <f>IF(COUNT(AS15:AS16)=2,(AS15/AS16-1)*100,"")</f>
+        <f>IF(COUNT(AS15:AS16)=2,ROUND((AS15/AS16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB15" s="5" t="n">
         <v>16.5</v>
       </c>
       <c r="BC15" s="6">
-        <f>IF(COUNT(BB15:BB16)=2,(BB15/BB16-1)*100,"")</f>
+        <f>IF(COUNT(BB15:BB16)=2,ROUND((BB15/BB16-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD15" s="6" t="n">
@@ -3624,11 +3624,11 @@
         <v>187.34</v>
       </c>
       <c r="D16" s="6">
-        <f>IF(COUNT(B16:B17)=2,(B16/B17-1)*100,"")</f>
+        <f>IF(COUNT(B16:B17)=2,ROUND((B16/B17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E16" s="6">
-        <f>IF(COUNT(C16:C17)=2,(C16/C17-1)*100,"")</f>
+        <f>IF(COUNT(C16:C17)=2,ROUND((C16/C17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F16" s="5" t="n">
@@ -3752,42 +3752,42 @@
         <v>111.34</v>
       </c>
       <c r="AT16" s="6">
-        <f>IF(COUNT(J16:J17)=2,(J16/J17-1)*100,"")</f>
+        <f>IF(COUNT(J16:J17)=2,ROUND((J16/J17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU16" s="6">
-        <f>IF(COUNT(O16:O17)=2,(O16/O17-1)*100,"")</f>
+        <f>IF(COUNT(O16:O17)=2,ROUND((O16/O17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV16" s="6">
-        <f>IF(COUNT(T16:T17)=2,(T16/T17-1)*100,"")</f>
+        <f>IF(COUNT(T16:T17)=2,ROUND((T16/T17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW16" s="6">
-        <f>IF(COUNT(Y16:Y17)=2,(Y16/Y17-1)*100,"")</f>
+        <f>IF(COUNT(Y16:Y17)=2,ROUND((Y16/Y17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX16" s="6">
-        <f>IF(COUNT(AD16:AD17)=2,(AD16/AD17-1)*100,"")</f>
+        <f>IF(COUNT(AD16:AD17)=2,ROUND((AD16/AD17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY16" s="6">
-        <f>IF(COUNT(AI16:AI17)=2,(AI16/AI17-1)*100,"")</f>
+        <f>IF(COUNT(AI16:AI17)=2,ROUND((AI16/AI17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ16" s="6">
-        <f>IF(COUNT(AN16:AN17)=2,(AN16/AN17-1)*100,"")</f>
+        <f>IF(COUNT(AN16:AN17)=2,ROUND((AN16/AN17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA16" s="6">
-        <f>IF(COUNT(AS16:AS17)=2,(AS16/AS17-1)*100,"")</f>
+        <f>IF(COUNT(AS16:AS17)=2,ROUND((AS16/AS17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB16" s="5" t="n">
         <v>15.86</v>
       </c>
       <c r="BC16" s="6">
-        <f>IF(COUNT(BB16:BB17)=2,(BB16/BB17-1)*100,"")</f>
+        <f>IF(COUNT(BB16:BB17)=2,ROUND((BB16/BB17-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD16" s="6" t="n">
@@ -3839,11 +3839,11 @@
         <v>182.05</v>
       </c>
       <c r="D17" s="6">
-        <f>IF(COUNT(B17:B18)=2,(B17/B18-1)*100,"")</f>
+        <f>IF(COUNT(B17:B18)=2,ROUND((B17/B18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E17" s="6">
-        <f>IF(COUNT(C17:C18)=2,(C17/C18-1)*100,"")</f>
+        <f>IF(COUNT(C17:C18)=2,ROUND((C17/C18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F17" s="5" t="n">
@@ -3967,42 +3967,42 @@
         <v>108.24</v>
       </c>
       <c r="AT17" s="6">
-        <f>IF(COUNT(J17:J18)=2,(J17/J18-1)*100,"")</f>
+        <f>IF(COUNT(J17:J18)=2,ROUND((J17/J18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU17" s="6">
-        <f>IF(COUNT(O17:O18)=2,(O17/O18-1)*100,"")</f>
+        <f>IF(COUNT(O17:O18)=2,ROUND((O17/O18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV17" s="6">
-        <f>IF(COUNT(T17:T18)=2,(T17/T18-1)*100,"")</f>
+        <f>IF(COUNT(T17:T18)=2,ROUND((T17/T18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW17" s="6">
-        <f>IF(COUNT(Y17:Y18)=2,(Y17/Y18-1)*100,"")</f>
+        <f>IF(COUNT(Y17:Y18)=2,ROUND((Y17/Y18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX17" s="6">
-        <f>IF(COUNT(AD17:AD18)=2,(AD17/AD18-1)*100,"")</f>
+        <f>IF(COUNT(AD17:AD18)=2,ROUND((AD17/AD18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY17" s="6">
-        <f>IF(COUNT(AI17:AI18)=2,(AI17/AI18-1)*100,"")</f>
+        <f>IF(COUNT(AI17:AI18)=2,ROUND((AI17/AI18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ17" s="6">
-        <f>IF(COUNT(AN17:AN18)=2,(AN17/AN18-1)*100,"")</f>
+        <f>IF(COUNT(AN17:AN18)=2,ROUND((AN17/AN18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA17" s="6">
-        <f>IF(COUNT(AS17:AS18)=2,(AS17/AS18-1)*100,"")</f>
+        <f>IF(COUNT(AS17:AS18)=2,ROUND((AS17/AS18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB17" s="5" t="n">
         <v>15.99</v>
       </c>
       <c r="BC17" s="6">
-        <f>IF(COUNT(BB17:BB18)=2,(BB17/BB18-1)*100,"")</f>
+        <f>IF(COUNT(BB17:BB18)=2,ROUND((BB17/BB18-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD17" s="6" t="n">
@@ -4054,11 +4054,11 @@
         <v>179.55</v>
       </c>
       <c r="D18" s="6">
-        <f>IF(COUNT(B18:B19)=2,(B18/B19-1)*100,"")</f>
+        <f>IF(COUNT(B18:B19)=2,ROUND((B18/B19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E18" s="6">
-        <f>IF(COUNT(C18:C19)=2,(C18/C19-1)*100,"")</f>
+        <f>IF(COUNT(C18:C19)=2,ROUND((C18/C19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F18" s="5" t="n">
@@ -4182,42 +4182,42 @@
         <v>106.58</v>
       </c>
       <c r="AT18" s="6">
-        <f>IF(COUNT(J18:J19)=2,(J18/J19-1)*100,"")</f>
+        <f>IF(COUNT(J18:J19)=2,ROUND((J18/J19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU18" s="6">
-        <f>IF(COUNT(O18:O19)=2,(O18/O19-1)*100,"")</f>
+        <f>IF(COUNT(O18:O19)=2,ROUND((O18/O19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV18" s="6">
-        <f>IF(COUNT(T18:T19)=2,(T18/T19-1)*100,"")</f>
+        <f>IF(COUNT(T18:T19)=2,ROUND((T18/T19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW18" s="6">
-        <f>IF(COUNT(Y18:Y19)=2,(Y18/Y19-1)*100,"")</f>
+        <f>IF(COUNT(Y18:Y19)=2,ROUND((Y18/Y19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX18" s="6">
-        <f>IF(COUNT(AD18:AD19)=2,(AD18/AD19-1)*100,"")</f>
+        <f>IF(COUNT(AD18:AD19)=2,ROUND((AD18/AD19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY18" s="6">
-        <f>IF(COUNT(AI18:AI19)=2,(AI18/AI19-1)*100,"")</f>
+        <f>IF(COUNT(AI18:AI19)=2,ROUND((AI18/AI19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ18" s="6">
-        <f>IF(COUNT(AN18:AN19)=2,(AN18/AN19-1)*100,"")</f>
+        <f>IF(COUNT(AN18:AN19)=2,ROUND((AN18/AN19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA18" s="6">
-        <f>IF(COUNT(AS18:AS19)=2,(AS18/AS19-1)*100,"")</f>
+        <f>IF(COUNT(AS18:AS19)=2,ROUND((AS18/AS19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB18" s="5" t="n">
         <v>17.09</v>
       </c>
       <c r="BC18" s="6">
-        <f>IF(COUNT(BB18:BB19)=2,(BB18/BB19-1)*100,"")</f>
+        <f>IF(COUNT(BB18:BB19)=2,ROUND((BB18/BB19-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD18" s="6" t="n">
@@ -4269,11 +4269,11 @@
         <v>173.8</v>
       </c>
       <c r="D19" s="6">
-        <f>IF(COUNT(B19:B20)=2,(B19/B20-1)*100,"")</f>
+        <f>IF(COUNT(B19:B20)=2,ROUND((B19/B20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E19" s="6">
-        <f>IF(COUNT(C19:C20)=2,(C19/C20-1)*100,"")</f>
+        <f>IF(COUNT(C19:C20)=2,ROUND((C19/C20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F19" s="5" t="n">
@@ -4397,42 +4397,42 @@
         <v>109.51</v>
       </c>
       <c r="AT19" s="6">
-        <f>IF(COUNT(J19:J20)=2,(J19/J20-1)*100,"")</f>
+        <f>IF(COUNT(J19:J20)=2,ROUND((J19/J20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU19" s="6">
-        <f>IF(COUNT(O19:O20)=2,(O19/O20-1)*100,"")</f>
+        <f>IF(COUNT(O19:O20)=2,ROUND((O19/O20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV19" s="6">
-        <f>IF(COUNT(T19:T20)=2,(T19/T20-1)*100,"")</f>
+        <f>IF(COUNT(T19:T20)=2,ROUND((T19/T20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW19" s="6">
-        <f>IF(COUNT(Y19:Y20)=2,(Y19/Y20-1)*100,"")</f>
+        <f>IF(COUNT(Y19:Y20)=2,ROUND((Y19/Y20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX19" s="6">
-        <f>IF(COUNT(AD19:AD20)=2,(AD19/AD20-1)*100,"")</f>
+        <f>IF(COUNT(AD19:AD20)=2,ROUND((AD19/AD20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY19" s="6">
-        <f>IF(COUNT(AI19:AI20)=2,(AI19/AI20-1)*100,"")</f>
+        <f>IF(COUNT(AI19:AI20)=2,ROUND((AI19/AI20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ19" s="6">
-        <f>IF(COUNT(AN19:AN20)=2,(AN19/AN20-1)*100,"")</f>
+        <f>IF(COUNT(AN19:AN20)=2,ROUND((AN19/AN20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA19" s="6">
-        <f>IF(COUNT(AS19:AS20)=2,(AS19/AS20-1)*100,"")</f>
+        <f>IF(COUNT(AS19:AS20)=2,ROUND((AS19/AS20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB19" s="5" t="n">
         <v>20.66</v>
       </c>
       <c r="BC19" s="6">
-        <f>IF(COUNT(BB19:BB20)=2,(BB19/BB20-1)*100,"")</f>
+        <f>IF(COUNT(BB19:BB20)=2,ROUND((BB19/BB20-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD19" s="6" t="n">
@@ -4484,11 +4484,11 @@
         <v>179.29</v>
       </c>
       <c r="D20" s="6">
-        <f>IF(COUNT(B20:B21)=2,(B20/B21-1)*100,"")</f>
+        <f>IF(COUNT(B20:B21)=2,ROUND((B20/B21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E20" s="6">
-        <f>IF(COUNT(C20:C21)=2,(C20/C21-1)*100,"")</f>
+        <f>IF(COUNT(C20:C21)=2,ROUND((C20/C21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F20" s="5" t="n">
@@ -4612,42 +4612,42 @@
         <v>109.67</v>
       </c>
       <c r="AT20" s="6">
-        <f>IF(COUNT(J20:J21)=2,(J20/J21-1)*100,"")</f>
+        <f>IF(COUNT(J20:J21)=2,ROUND((J20/J21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU20" s="6">
-        <f>IF(COUNT(O20:O21)=2,(O20/O21-1)*100,"")</f>
+        <f>IF(COUNT(O20:O21)=2,ROUND((O20/O21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV20" s="6">
-        <f>IF(COUNT(T20:T21)=2,(T20/T21-1)*100,"")</f>
+        <f>IF(COUNT(T20:T21)=2,ROUND((T20/T21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW20" s="6">
-        <f>IF(COUNT(Y20:Y21)=2,(Y20/Y21-1)*100,"")</f>
+        <f>IF(COUNT(Y20:Y21)=2,ROUND((Y20/Y21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX20" s="6">
-        <f>IF(COUNT(AD20:AD21)=2,(AD20/AD21-1)*100,"")</f>
+        <f>IF(COUNT(AD20:AD21)=2,ROUND((AD20/AD21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY20" s="6">
-        <f>IF(COUNT(AI20:AI21)=2,(AI20/AI21-1)*100,"")</f>
+        <f>IF(COUNT(AI20:AI21)=2,ROUND((AI20/AI21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ20" s="6">
-        <f>IF(COUNT(AN20:AN21)=2,(AN20/AN21-1)*100,"")</f>
+        <f>IF(COUNT(AN20:AN21)=2,ROUND((AN20/AN21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA20" s="6">
-        <f>IF(COUNT(AS20:AS21)=2,(AS20/AS21-1)*100,"")</f>
+        <f>IF(COUNT(AS20:AS21)=2,ROUND((AS20/AS21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB20" s="5" t="n">
         <v>18.21</v>
       </c>
       <c r="BC20" s="6">
-        <f>IF(COUNT(BB20:BB21)=2,(BB20/BB21-1)*100,"")</f>
+        <f>IF(COUNT(BB20:BB21)=2,ROUND((BB20/BB21-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD20" s="6" t="n">
@@ -4699,11 +4699,11 @@
         <v>178.54</v>
       </c>
       <c r="D21" s="6">
-        <f>IF(COUNT(B21:B22)=2,(B21/B22-1)*100,"")</f>
+        <f>IF(COUNT(B21:B22)=2,ROUND((B21/B22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E21" s="6">
-        <f>IF(COUNT(C21:C22)=2,(C21/C22-1)*100,"")</f>
+        <f>IF(COUNT(C21:C22)=2,ROUND((C21/C22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F21" s="5" t="n">
@@ -4827,42 +4827,42 @@
         <v>107.66</v>
       </c>
       <c r="AT21" s="6">
-        <f>IF(COUNT(J21:J22)=2,(J21/J22-1)*100,"")</f>
+        <f>IF(COUNT(J21:J22)=2,ROUND((J21/J22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU21" s="6">
-        <f>IF(COUNT(O21:O22)=2,(O21/O22-1)*100,"")</f>
+        <f>IF(COUNT(O21:O22)=2,ROUND((O21/O22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV21" s="6">
-        <f>IF(COUNT(T21:T22)=2,(T21/T22-1)*100,"")</f>
+        <f>IF(COUNT(T21:T22)=2,ROUND((T21/T22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW21" s="6">
-        <f>IF(COUNT(Y21:Y22)=2,(Y21/Y22-1)*100,"")</f>
+        <f>IF(COUNT(Y21:Y22)=2,ROUND((Y21/Y22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX21" s="6">
-        <f>IF(COUNT(AD21:AD22)=2,(AD21/AD22-1)*100,"")</f>
+        <f>IF(COUNT(AD21:AD22)=2,ROUND((AD21/AD22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY21" s="6">
-        <f>IF(COUNT(AI21:AI22)=2,(AI21/AI22-1)*100,"")</f>
+        <f>IF(COUNT(AI21:AI22)=2,ROUND((AI21/AI22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ21" s="6">
-        <f>IF(COUNT(AN21:AN22)=2,(AN21/AN22-1)*100,"")</f>
+        <f>IF(COUNT(AN21:AN22)=2,ROUND((AN21/AN22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA21" s="6">
-        <f>IF(COUNT(AS21:AS22)=2,(AS21/AS22-1)*100,"")</f>
+        <f>IF(COUNT(AS21:AS22)=2,ROUND((AS21/AS22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB21" s="5" t="n">
         <v>18.67</v>
       </c>
       <c r="BC21" s="6">
-        <f>IF(COUNT(BB21:BB22)=2,(BB21/BB22-1)*100,"")</f>
+        <f>IF(COUNT(BB21:BB22)=2,ROUND((BB21/BB22-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD21" s="6" t="n">
@@ -4914,11 +4914,11 @@
         <v>178.56</v>
       </c>
       <c r="D22" s="6">
-        <f>IF(COUNT(B22:B23)=2,(B22/B23-1)*100,"")</f>
+        <f>IF(COUNT(B22:B23)=2,ROUND((B22/B23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E22" s="6">
-        <f>IF(COUNT(C22:C23)=2,(C22/C23-1)*100,"")</f>
+        <f>IF(COUNT(C22:C23)=2,ROUND((C22/C23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F22" s="5" t="n">
@@ -5042,42 +5042,42 @@
         <v>106.3</v>
       </c>
       <c r="AT22" s="6">
-        <f>IF(COUNT(J22:J23)=2,(J22/J23-1)*100,"")</f>
+        <f>IF(COUNT(J22:J23)=2,ROUND((J22/J23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU22" s="6">
-        <f>IF(COUNT(O22:O23)=2,(O22/O23-1)*100,"")</f>
+        <f>IF(COUNT(O22:O23)=2,ROUND((O22/O23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV22" s="6">
-        <f>IF(COUNT(T22:T23)=2,(T22/T23-1)*100,"")</f>
+        <f>IF(COUNT(T22:T23)=2,ROUND((T22/T23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW22" s="6">
-        <f>IF(COUNT(Y22:Y23)=2,(Y22/Y23-1)*100,"")</f>
+        <f>IF(COUNT(Y22:Y23)=2,ROUND((Y22/Y23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX22" s="6">
-        <f>IF(COUNT(AD22:AD23)=2,(AD22/AD23-1)*100,"")</f>
+        <f>IF(COUNT(AD22:AD23)=2,ROUND((AD22/AD23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY22" s="6">
-        <f>IF(COUNT(AI22:AI23)=2,(AI22/AI23-1)*100,"")</f>
+        <f>IF(COUNT(AI22:AI23)=2,ROUND((AI22/AI23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ22" s="6">
-        <f>IF(COUNT(AN22:AN23)=2,(AN22/AN23-1)*100,"")</f>
+        <f>IF(COUNT(AN22:AN23)=2,ROUND((AN22/AN23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA22" s="6">
-        <f>IF(COUNT(AS22:AS23)=2,(AS22/AS23-1)*100,"")</f>
+        <f>IF(COUNT(AS22:AS23)=2,ROUND((AS22/AS23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB22" s="5" t="n">
         <v>18.58</v>
       </c>
       <c r="BC22" s="6">
-        <f>IF(COUNT(BB22:BB23)=2,(BB22/BB23-1)*100,"")</f>
+        <f>IF(COUNT(BB22:BB23)=2,ROUND((BB22/BB23-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD22" s="6" t="n">
@@ -5129,11 +5129,11 @@
         <v>178.37</v>
       </c>
       <c r="D23" s="6">
-        <f>IF(COUNT(B23:B24)=2,(B23/B24-1)*100,"")</f>
+        <f>IF(COUNT(B23:B24)=2,ROUND((B23/B24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E23" s="6">
-        <f>IF(COUNT(C23:C24)=2,(C23/C24-1)*100,"")</f>
+        <f>IF(COUNT(C23:C24)=2,ROUND((C23/C24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F23" s="5" t="n">
@@ -5257,42 +5257,42 @@
         <v>105.38</v>
       </c>
       <c r="AT23" s="6">
-        <f>IF(COUNT(J23:J24)=2,(J23/J24-1)*100,"")</f>
+        <f>IF(COUNT(J23:J24)=2,ROUND((J23/J24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU23" s="6">
-        <f>IF(COUNT(O23:O24)=2,(O23/O24-1)*100,"")</f>
+        <f>IF(COUNT(O23:O24)=2,ROUND((O23/O24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV23" s="6">
-        <f>IF(COUNT(T23:T24)=2,(T23/T24-1)*100,"")</f>
+        <f>IF(COUNT(T23:T24)=2,ROUND((T23/T24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW23" s="6">
-        <f>IF(COUNT(Y23:Y24)=2,(Y23/Y24-1)*100,"")</f>
+        <f>IF(COUNT(Y23:Y24)=2,ROUND((Y23/Y24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX23" s="6">
-        <f>IF(COUNT(AD23:AD24)=2,(AD23/AD24-1)*100,"")</f>
+        <f>IF(COUNT(AD23:AD24)=2,ROUND((AD23/AD24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY23" s="6">
-        <f>IF(COUNT(AI23:AI24)=2,(AI23/AI24-1)*100,"")</f>
+        <f>IF(COUNT(AI23:AI24)=2,ROUND((AI23/AI24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ23" s="6">
-        <f>IF(COUNT(AN23:AN24)=2,(AN23/AN24-1)*100,"")</f>
+        <f>IF(COUNT(AN23:AN24)=2,ROUND((AN23/AN24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA23" s="6">
-        <f>IF(COUNT(AS23:AS24)=2,(AS23/AS24-1)*100,"")</f>
+        <f>IF(COUNT(AS23:AS24)=2,ROUND((AS23/AS24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB23" s="5" t="n">
         <v>18.7</v>
       </c>
       <c r="BC23" s="6">
-        <f>IF(COUNT(BB23:BB24)=2,(BB23/BB24-1)*100,"")</f>
+        <f>IF(COUNT(BB23:BB24)=2,ROUND((BB23/BB24-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD23" s="6" t="n">
@@ -5344,11 +5344,11 @@
         <v>182.85</v>
       </c>
       <c r="D24" s="6">
-        <f>IF(COUNT(B24:B25)=2,(B24/B25-1)*100,"")</f>
+        <f>IF(COUNT(B24:B25)=2,ROUND((B24/B25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E24" s="6">
-        <f>IF(COUNT(C24:C25)=2,(C24/C25-1)*100,"")</f>
+        <f>IF(COUNT(C24:C25)=2,ROUND((C24/C25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F24" s="5" t="n">
@@ -5472,42 +5472,42 @@
         <v>109.2</v>
       </c>
       <c r="AT24" s="6">
-        <f>IF(COUNT(J24:J25)=2,(J24/J25-1)*100,"")</f>
+        <f>IF(COUNT(J24:J25)=2,ROUND((J24/J25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU24" s="6">
-        <f>IF(COUNT(O24:O25)=2,(O24/O25-1)*100,"")</f>
+        <f>IF(COUNT(O24:O25)=2,ROUND((O24/O25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV24" s="6">
-        <f>IF(COUNT(T24:T25)=2,(T24/T25-1)*100,"")</f>
+        <f>IF(COUNT(T24:T25)=2,ROUND((T24/T25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW24" s="6">
-        <f>IF(COUNT(Y24:Y25)=2,(Y24/Y25-1)*100,"")</f>
+        <f>IF(COUNT(Y24:Y25)=2,ROUND((Y24/Y25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX24" s="6">
-        <f>IF(COUNT(AD24:AD25)=2,(AD24/AD25-1)*100,"")</f>
+        <f>IF(COUNT(AD24:AD25)=2,ROUND((AD24/AD25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY24" s="6">
-        <f>IF(COUNT(AI24:AI25)=2,(AI24/AI25-1)*100,"")</f>
+        <f>IF(COUNT(AI24:AI25)=2,ROUND((AI24/AI25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ24" s="6">
-        <f>IF(COUNT(AN24:AN25)=2,(AN24/AN25-1)*100,"")</f>
+        <f>IF(COUNT(AN24:AN25)=2,ROUND((AN24/AN25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA24" s="6">
-        <f>IF(COUNT(AS24:AS25)=2,(AS24/AS25-1)*100,"")</f>
+        <f>IF(COUNT(AS24:AS25)=2,ROUND((AS24/AS25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB24" s="5" t="n">
         <v>16.64</v>
       </c>
       <c r="BC24" s="6">
-        <f>IF(COUNT(BB24:BB25)=2,(BB24/BB25-1)*100,"")</f>
+        <f>IF(COUNT(BB24:BB25)=2,ROUND((BB24/BB25-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD24" s="6" t="n">
@@ -5559,11 +5559,11 @@
         <v>183.34</v>
       </c>
       <c r="D25" s="6">
-        <f>IF(COUNT(B25:B26)=2,(B25/B26-1)*100,"")</f>
+        <f>IF(COUNT(B25:B26)=2,ROUND((B25/B26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E25" s="6">
-        <f>IF(COUNT(C25:C26)=2,(C25/C26-1)*100,"")</f>
+        <f>IF(COUNT(C25:C26)=2,ROUND((C25/C26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F25" s="5" t="n">
@@ -5687,42 +5687,42 @@
         <v>110.03</v>
       </c>
       <c r="AT25" s="6">
-        <f>IF(COUNT(J25:J26)=2,(J25/J26-1)*100,"")</f>
+        <f>IF(COUNT(J25:J26)=2,ROUND((J25/J26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU25" s="6">
-        <f>IF(COUNT(O25:O26)=2,(O25/O26-1)*100,"")</f>
+        <f>IF(COUNT(O25:O26)=2,ROUND((O25/O26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV25" s="6">
-        <f>IF(COUNT(T25:T26)=2,(T25/T26-1)*100,"")</f>
+        <f>IF(COUNT(T25:T26)=2,ROUND((T25/T26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW25" s="6">
-        <f>IF(COUNT(Y25:Y26)=2,(Y25/Y26-1)*100,"")</f>
+        <f>IF(COUNT(Y25:Y26)=2,ROUND((Y25/Y26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX25" s="6">
-        <f>IF(COUNT(AD25:AD26)=2,(AD25/AD26-1)*100,"")</f>
+        <f>IF(COUNT(AD25:AD26)=2,ROUND((AD25/AD26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY25" s="6">
-        <f>IF(COUNT(AI25:AI26)=2,(AI25/AI26-1)*100,"")</f>
+        <f>IF(COUNT(AI25:AI26)=2,ROUND((AI25/AI26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ25" s="6">
-        <f>IF(COUNT(AN25:AN26)=2,(AN25/AN26-1)*100,"")</f>
+        <f>IF(COUNT(AN25:AN26)=2,ROUND((AN25/AN26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA25" s="6">
-        <f>IF(COUNT(AS25:AS26)=2,(AS25/AS26-1)*100,"")</f>
+        <f>IF(COUNT(AS25:AS26)=2,ROUND((AS25/AS26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB25" s="5" t="n">
         <v>17.05</v>
       </c>
       <c r="BC25" s="6">
-        <f>IF(COUNT(BB25:BB26)=2,(BB25/BB26-1)*100,"")</f>
+        <f>IF(COUNT(BB25:BB26)=2,ROUND((BB25/BB26-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD25" s="6" t="n">
@@ -5774,11 +5774,11 @@
         <v>180.23</v>
       </c>
       <c r="D26" s="6">
-        <f>IF(COUNT(B26:B27)=2,(B26/B27-1)*100,"")</f>
+        <f>IF(COUNT(B26:B27)=2,ROUND((B26/B27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E26" s="6">
-        <f>IF(COUNT(C26:C27)=2,(C26/C27-1)*100,"")</f>
+        <f>IF(COUNT(C26:C27)=2,ROUND((C26/C27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F26" s="5" t="n">
@@ -5902,42 +5902,42 @@
         <v>110.8</v>
       </c>
       <c r="AT26" s="6">
-        <f>IF(COUNT(J26:J27)=2,(J26/J27-1)*100,"")</f>
+        <f>IF(COUNT(J26:J27)=2,ROUND((J26/J27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU26" s="6">
-        <f>IF(COUNT(O26:O27)=2,(O26/O27-1)*100,"")</f>
+        <f>IF(COUNT(O26:O27)=2,ROUND((O26/O27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV26" s="6">
-        <f>IF(COUNT(T26:T27)=2,(T26/T27-1)*100,"")</f>
+        <f>IF(COUNT(T26:T27)=2,ROUND((T26/T27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW26" s="6">
-        <f>IF(COUNT(Y26:Y27)=2,(Y26/Y27-1)*100,"")</f>
+        <f>IF(COUNT(Y26:Y27)=2,ROUND((Y26/Y27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX26" s="6">
-        <f>IF(COUNT(AD26:AD27)=2,(AD26/AD27-1)*100,"")</f>
+        <f>IF(COUNT(AD26:AD27)=2,ROUND((AD26/AD27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY26" s="6">
-        <f>IF(COUNT(AI26:AI27)=2,(AI26/AI27-1)*100,"")</f>
+        <f>IF(COUNT(AI26:AI27)=2,ROUND((AI26/AI27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ26" s="6">
-        <f>IF(COUNT(AN26:AN27)=2,(AN26/AN27-1)*100,"")</f>
+        <f>IF(COUNT(AN26:AN27)=2,ROUND((AN26/AN27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA26" s="6">
-        <f>IF(COUNT(AS26:AS27)=2,(AS26/AS27-1)*100,"")</f>
+        <f>IF(COUNT(AS26:AS27)=2,ROUND((AS26/AS27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB26" s="5" t="n">
         <v>18.65</v>
       </c>
       <c r="BC26" s="6">
-        <f>IF(COUNT(BB26:BB27)=2,(BB26/BB27-1)*100,"")</f>
+        <f>IF(COUNT(BB26:BB27)=2,ROUND((BB26/BB27-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD26" s="6" t="n">
@@ -5989,11 +5989,11 @@
         <v>180.98</v>
       </c>
       <c r="D27" s="6">
-        <f>IF(COUNT(B27:B28)=2,(B27/B28-1)*100,"")</f>
+        <f>IF(COUNT(B27:B28)=2,ROUND((B27/B28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E27" s="6">
-        <f>IF(COUNT(C27:C28)=2,(C27/C28-1)*100,"")</f>
+        <f>IF(COUNT(C27:C28)=2,ROUND((C27/C28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F27" s="5" t="n">
@@ -6117,42 +6117,42 @@
         <v>110.65</v>
       </c>
       <c r="AT27" s="6">
-        <f>IF(COUNT(J27:J28)=2,(J27/J28-1)*100,"")</f>
+        <f>IF(COUNT(J27:J28)=2,ROUND((J27/J28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU27" s="6">
-        <f>IF(COUNT(O27:O28)=2,(O27/O28-1)*100,"")</f>
+        <f>IF(COUNT(O27:O28)=2,ROUND((O27/O28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV27" s="6">
-        <f>IF(COUNT(T27:T28)=2,(T27/T28-1)*100,"")</f>
+        <f>IF(COUNT(T27:T28)=2,ROUND((T27/T28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW27" s="6">
-        <f>IF(COUNT(Y27:Y28)=2,(Y27/Y28-1)*100,"")</f>
+        <f>IF(COUNT(Y27:Y28)=2,ROUND((Y27/Y28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX27" s="6">
-        <f>IF(COUNT(AD27:AD28)=2,(AD27/AD28-1)*100,"")</f>
+        <f>IF(COUNT(AD27:AD28)=2,ROUND((AD27/AD28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY27" s="6">
-        <f>IF(COUNT(AI27:AI28)=2,(AI27/AI28-1)*100,"")</f>
+        <f>IF(COUNT(AI27:AI28)=2,ROUND((AI27/AI28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ27" s="6">
-        <f>IF(COUNT(AN27:AN28)=2,(AN27/AN28-1)*100,"")</f>
+        <f>IF(COUNT(AN27:AN28)=2,ROUND((AN27/AN28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA27" s="6">
-        <f>IF(COUNT(AS27:AS28)=2,(AS27/AS28-1)*100,"")</f>
+        <f>IF(COUNT(AS27:AS28)=2,ROUND((AS27/AS28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB27" s="5" t="n">
         <v>18.77</v>
       </c>
       <c r="BC27" s="6">
-        <f>IF(COUNT(BB27:BB28)=2,(BB27/BB28-1)*100,"")</f>
+        <f>IF(COUNT(BB27:BB28)=2,ROUND((BB27/BB28-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD27" s="6" t="n">
@@ -6204,11 +6204,11 @@
         <v>184.73</v>
       </c>
       <c r="D28" s="6">
-        <f>IF(COUNT(B28:B29)=2,(B28/B29-1)*100,"")</f>
+        <f>IF(COUNT(B28:B29)=2,ROUND((B28/B29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E28" s="6">
-        <f>IF(COUNT(C28:C29)=2,(C28/C29-1)*100,"")</f>
+        <f>IF(COUNT(C28:C29)=2,ROUND((C28/C29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F28" s="5" t="n">
@@ -6332,42 +6332,42 @@
         <v>112.65</v>
       </c>
       <c r="AT28" s="6">
-        <f>IF(COUNT(J28:J29)=2,(J28/J29-1)*100,"")</f>
+        <f>IF(COUNT(J28:J29)=2,ROUND((J28/J29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU28" s="6">
-        <f>IF(COUNT(O28:O29)=2,(O28/O29-1)*100,"")</f>
+        <f>IF(COUNT(O28:O29)=2,ROUND((O28/O29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV28" s="6">
-        <f>IF(COUNT(T28:T29)=2,(T28/T29-1)*100,"")</f>
+        <f>IF(COUNT(T28:T29)=2,ROUND((T28/T29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW28" s="6">
-        <f>IF(COUNT(Y28:Y29)=2,(Y28/Y29-1)*100,"")</f>
+        <f>IF(COUNT(Y28:Y29)=2,ROUND((Y28/Y29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX28" s="6">
-        <f>IF(COUNT(AD28:AD29)=2,(AD28/AD29-1)*100,"")</f>
+        <f>IF(COUNT(AD28:AD29)=2,ROUND((AD28/AD29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY28" s="6">
-        <f>IF(COUNT(AI28:AI29)=2,(AI28/AI29-1)*100,"")</f>
+        <f>IF(COUNT(AI28:AI29)=2,ROUND((AI28/AI29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ28" s="6">
-        <f>IF(COUNT(AN28:AN29)=2,(AN28/AN29-1)*100,"")</f>
+        <f>IF(COUNT(AN28:AN29)=2,ROUND((AN28/AN29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA28" s="6">
-        <f>IF(COUNT(AS28:AS29)=2,(AS28/AS29-1)*100,"")</f>
+        <f>IF(COUNT(AS28:AS29)=2,ROUND((AS28/AS29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB28" s="5" t="n">
         <v>16.73</v>
       </c>
       <c r="BC28" s="6">
-        <f>IF(COUNT(BB28:BB29)=2,(BB28/BB29-1)*100,"")</f>
+        <f>IF(COUNT(BB28:BB29)=2,ROUND((BB28/BB29-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD28" s="6" t="n">
@@ -6419,11 +6419,11 @@
         <v>186.67</v>
       </c>
       <c r="D29" s="6">
-        <f>IF(COUNT(B29:B30)=2,(B29/B30-1)*100,"")</f>
+        <f>IF(COUNT(B29:B30)=2,ROUND((B29/B30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E29" s="6">
-        <f>IF(COUNT(C29:C30)=2,(C29/C30-1)*100,"")</f>
+        <f>IF(COUNT(C29:C30)=2,ROUND((C29/C30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F29" s="5" t="n">
@@ -6547,42 +6547,42 @@
         <v>113.38</v>
       </c>
       <c r="AT29" s="6">
-        <f>IF(COUNT(J29:J30)=2,(J29/J30-1)*100,"")</f>
+        <f>IF(COUNT(J29:J30)=2,ROUND((J29/J30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU29" s="6">
-        <f>IF(COUNT(O29:O30)=2,(O29/O30-1)*100,"")</f>
+        <f>IF(COUNT(O29:O30)=2,ROUND((O29/O30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV29" s="6">
-        <f>IF(COUNT(T29:T30)=2,(T29/T30-1)*100,"")</f>
+        <f>IF(COUNT(T29:T30)=2,ROUND((T29/T30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW29" s="6">
-        <f>IF(COUNT(Y29:Y30)=2,(Y29/Y30-1)*100,"")</f>
+        <f>IF(COUNT(Y29:Y30)=2,ROUND((Y29/Y30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX29" s="6">
-        <f>IF(COUNT(AD29:AD30)=2,(AD29/AD30-1)*100,"")</f>
+        <f>IF(COUNT(AD29:AD30)=2,ROUND((AD29/AD30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY29" s="6">
-        <f>IF(COUNT(AI29:AI30)=2,(AI29/AI30-1)*100,"")</f>
+        <f>IF(COUNT(AI29:AI30)=2,ROUND((AI29/AI30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ29" s="6">
-        <f>IF(COUNT(AN29:AN30)=2,(AN29/AN30-1)*100,"")</f>
+        <f>IF(COUNT(AN29:AN30)=2,ROUND((AN29/AN30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA29" s="6">
-        <f>IF(COUNT(AS29:AS30)=2,(AS29/AS30-1)*100,"")</f>
+        <f>IF(COUNT(AS29:AS30)=2,ROUND((AS29/AS30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB29" s="5" t="n">
         <v>15.67</v>
       </c>
       <c r="BC29" s="6">
-        <f>IF(COUNT(BB29:BB30)=2,(BB29/BB30-1)*100,"")</f>
+        <f>IF(COUNT(BB29:BB30)=2,ROUND((BB29/BB30-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD29" s="6" t="n">
@@ -6634,11 +6634,11 @@
         <v>185.27</v>
       </c>
       <c r="D30" s="6">
-        <f>IF(COUNT(B30:B31)=2,(B30/B31-1)*100,"")</f>
+        <f>IF(COUNT(B30:B31)=2,ROUND((B30/B31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E30" s="6">
-        <f>IF(COUNT(C30:C31)=2,(C30/C31-1)*100,"")</f>
+        <f>IF(COUNT(C30:C31)=2,ROUND((C30/C31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F30" s="5" t="n">
@@ -6762,42 +6762,42 @@
         <v>111.45</v>
       </c>
       <c r="AT30" s="6">
-        <f>IF(COUNT(J30:J31)=2,(J30/J31-1)*100,"")</f>
+        <f>IF(COUNT(J30:J31)=2,ROUND((J30/J31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU30" s="6">
-        <f>IF(COUNT(O30:O31)=2,(O30/O31-1)*100,"")</f>
+        <f>IF(COUNT(O30:O31)=2,ROUND((O30/O31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV30" s="6">
-        <f>IF(COUNT(T30:T31)=2,(T30/T31-1)*100,"")</f>
+        <f>IF(COUNT(T30:T31)=2,ROUND((T30/T31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW30" s="6">
-        <f>IF(COUNT(Y30:Y31)=2,(Y30/Y31-1)*100,"")</f>
+        <f>IF(COUNT(Y30:Y31)=2,ROUND((Y30/Y31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX30" s="6">
-        <f>IF(COUNT(AD30:AD31)=2,(AD30/AD31-1)*100,"")</f>
+        <f>IF(COUNT(AD30:AD31)=2,ROUND((AD30/AD31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY30" s="6">
-        <f>IF(COUNT(AI30:AI31)=2,(AI30/AI31-1)*100,"")</f>
+        <f>IF(COUNT(AI30:AI31)=2,ROUND((AI30/AI31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ30" s="6">
-        <f>IF(COUNT(AN30:AN31)=2,(AN30/AN31-1)*100,"")</f>
+        <f>IF(COUNT(AN30:AN31)=2,ROUND((AN30/AN31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA30" s="6">
-        <f>IF(COUNT(AS30:AS31)=2,(AS30/AS31-1)*100,"")</f>
+        <f>IF(COUNT(AS30:AS31)=2,ROUND((AS30/AS31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB30" s="5" t="n">
         <v>16.5</v>
       </c>
       <c r="BC30" s="6">
-        <f>IF(COUNT(BB30:BB31)=2,(BB30/BB31-1)*100,"")</f>
+        <f>IF(COUNT(BB30:BB31)=2,ROUND((BB30/BB31-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD30" s="6" t="n">
@@ -6849,11 +6849,11 @@
         <v>183.93</v>
       </c>
       <c r="D31" s="6">
-        <f>IF(COUNT(B31:B32)=2,(B31/B32-1)*100,"")</f>
+        <f>IF(COUNT(B31:B32)=2,ROUND((B31/B32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E31" s="6">
-        <f>IF(COUNT(C31:C32)=2,(C31/C32-1)*100,"")</f>
+        <f>IF(COUNT(C31:C32)=2,ROUND((C31/C32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F31" s="5" t="n">
@@ -6977,42 +6977,42 @@
         <v>111.59</v>
       </c>
       <c r="AT31" s="6">
-        <f>IF(COUNT(J31:J32)=2,(J31/J32-1)*100,"")</f>
+        <f>IF(COUNT(J31:J32)=2,ROUND((J31/J32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU31" s="6">
-        <f>IF(COUNT(O31:O32)=2,(O31/O32-1)*100,"")</f>
+        <f>IF(COUNT(O31:O32)=2,ROUND((O31/O32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV31" s="6">
-        <f>IF(COUNT(T31:T32)=2,(T31/T32-1)*100,"")</f>
+        <f>IF(COUNT(T31:T32)=2,ROUND((T31/T32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW31" s="6">
-        <f>IF(COUNT(Y31:Y32)=2,(Y31/Y32-1)*100,"")</f>
+        <f>IF(COUNT(Y31:Y32)=2,ROUND((Y31/Y32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX31" s="6">
-        <f>IF(COUNT(AD31:AD32)=2,(AD31/AD32-1)*100,"")</f>
+        <f>IF(COUNT(AD31:AD32)=2,ROUND((AD31/AD32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY31" s="6">
-        <f>IF(COUNT(AI31:AI32)=2,(AI31/AI32-1)*100,"")</f>
+        <f>IF(COUNT(AI31:AI32)=2,ROUND((AI31/AI32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ31" s="6">
-        <f>IF(COUNT(AN31:AN32)=2,(AN31/AN32-1)*100,"")</f>
+        <f>IF(COUNT(AN31:AN32)=2,ROUND((AN31/AN32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA31" s="6">
-        <f>IF(COUNT(AS31:AS32)=2,(AS31/AS32-1)*100,"")</f>
+        <f>IF(COUNT(AS31:AS32)=2,ROUND((AS31/AS32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB31" s="5" t="n">
         <v>17.16</v>
       </c>
       <c r="BC31" s="6">
-        <f>IF(COUNT(BB31:BB32)=2,(BB31/BB32-1)*100,"")</f>
+        <f>IF(COUNT(BB31:BB32)=2,ROUND((BB31/BB32-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD31" s="6" t="n">
@@ -7064,11 +7064,11 @@
         <v>186.95</v>
       </c>
       <c r="D32" s="6">
-        <f>IF(COUNT(B32:B33)=2,(B32/B33-1)*100,"")</f>
+        <f>IF(COUNT(B32:B33)=2,ROUND((B32/B33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E32" s="6">
-        <f>IF(COUNT(C32:C33)=2,(C32/C33-1)*100,"")</f>
+        <f>IF(COUNT(C32:C33)=2,ROUND((C32/C33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F32" s="5" t="n">
@@ -7192,42 +7192,42 @@
         <v>111.64</v>
       </c>
       <c r="AT32" s="6">
-        <f>IF(COUNT(J32:J33)=2,(J32/J33-1)*100,"")</f>
+        <f>IF(COUNT(J32:J33)=2,ROUND((J32/J33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU32" s="6">
-        <f>IF(COUNT(O32:O33)=2,(O32/O33-1)*100,"")</f>
+        <f>IF(COUNT(O32:O33)=2,ROUND((O32/O33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV32" s="6">
-        <f>IF(COUNT(T32:T33)=2,(T32/T33-1)*100,"")</f>
+        <f>IF(COUNT(T32:T33)=2,ROUND((T32/T33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW32" s="6">
-        <f>IF(COUNT(Y32:Y33)=2,(Y32/Y33-1)*100,"")</f>
+        <f>IF(COUNT(Y32:Y33)=2,ROUND((Y32/Y33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX32" s="6">
-        <f>IF(COUNT(AD32:AD33)=2,(AD32/AD33-1)*100,"")</f>
+        <f>IF(COUNT(AD32:AD33)=2,ROUND((AD32/AD33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY32" s="6">
-        <f>IF(COUNT(AI32:AI33)=2,(AI32/AI33-1)*100,"")</f>
+        <f>IF(COUNT(AI32:AI33)=2,ROUND((AI32/AI33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ32" s="6">
-        <f>IF(COUNT(AN32:AN33)=2,(AN32/AN33-1)*100,"")</f>
+        <f>IF(COUNT(AN32:AN33)=2,ROUND((AN32/AN33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA32" s="6">
-        <f>IF(COUNT(AS32:AS33)=2,(AS32/AS33-1)*100,"")</f>
+        <f>IF(COUNT(AS32:AS33)=2,ROUND((AS32/AS33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB32" s="5" t="n">
         <v>15.03</v>
       </c>
       <c r="BC32" s="6">
-        <f>IF(COUNT(BB32:BB33)=2,(BB32/BB33-1)*100,"")</f>
+        <f>IF(COUNT(BB32:BB33)=2,ROUND((BB32/BB33-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD32" s="6" t="n">
@@ -7279,11 +7279,11 @@
         <v>185.38</v>
       </c>
       <c r="D33" s="6">
-        <f>IF(COUNT(B33:B34)=2,(B33/B34-1)*100,"")</f>
+        <f>IF(COUNT(B33:B34)=2,ROUND((B33/B34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E33" s="6">
-        <f>IF(COUNT(C33:C34)=2,(C33/C34-1)*100,"")</f>
+        <f>IF(COUNT(C33:C34)=2,ROUND((C33/C34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F33" s="5" t="n">
@@ -7407,42 +7407,42 @@
         <v>110.51</v>
       </c>
       <c r="AT33" s="6">
-        <f>IF(COUNT(J33:J34)=2,(J33/J34-1)*100,"")</f>
+        <f>IF(COUNT(J33:J34)=2,ROUND((J33/J34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU33" s="6">
-        <f>IF(COUNT(O33:O34)=2,(O33/O34-1)*100,"")</f>
+        <f>IF(COUNT(O33:O34)=2,ROUND((O33/O34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV33" s="6">
-        <f>IF(COUNT(T33:T34)=2,(T33/T34-1)*100,"")</f>
+        <f>IF(COUNT(T33:T34)=2,ROUND((T33/T34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW33" s="6">
-        <f>IF(COUNT(Y33:Y34)=2,(Y33/Y34-1)*100,"")</f>
+        <f>IF(COUNT(Y33:Y34)=2,ROUND((Y33/Y34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX33" s="6">
-        <f>IF(COUNT(AD33:AD34)=2,(AD33/AD34-1)*100,"")</f>
+        <f>IF(COUNT(AD33:AD34)=2,ROUND((AD33/AD34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY33" s="6">
-        <f>IF(COUNT(AI33:AI34)=2,(AI33/AI34-1)*100,"")</f>
+        <f>IF(COUNT(AI33:AI34)=2,ROUND((AI33/AI34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ33" s="6">
-        <f>IF(COUNT(AN33:AN34)=2,(AN33/AN34-1)*100,"")</f>
+        <f>IF(COUNT(AN33:AN34)=2,ROUND((AN33/AN34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA33" s="6">
-        <f>IF(COUNT(AS33:AS34)=2,(AS33/AS34-1)*100,"")</f>
+        <f>IF(COUNT(AS33:AS34)=2,ROUND((AS33/AS34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB33" s="5" t="n">
         <v>15.84</v>
       </c>
       <c r="BC33" s="6">
-        <f>IF(COUNT(BB33:BB34)=2,(BB33/BB34-1)*100,"")</f>
+        <f>IF(COUNT(BB33:BB34)=2,ROUND((BB33/BB34-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD33" s="6" t="n">
@@ -7494,11 +7494,11 @@
         <v>182.42</v>
       </c>
       <c r="D34" s="6">
-        <f>IF(COUNT(B34:B35)=2,(B34/B35-1)*100,"")</f>
+        <f>IF(COUNT(B34:B35)=2,ROUND((B34/B35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E34" s="6">
-        <f>IF(COUNT(C34:C35)=2,(C34/C35-1)*100,"")</f>
+        <f>IF(COUNT(C34:C35)=2,ROUND((C34/C35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F34" s="5" t="n">
@@ -7622,42 +7622,42 @@
         <v>109.46</v>
       </c>
       <c r="AT34" s="6">
-        <f>IF(COUNT(J34:J35)=2,(J34/J35-1)*100,"")</f>
+        <f>IF(COUNT(J34:J35)=2,ROUND((J34/J35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU34" s="6">
-        <f>IF(COUNT(O34:O35)=2,(O34/O35-1)*100,"")</f>
+        <f>IF(COUNT(O34:O35)=2,ROUND((O34/O35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV34" s="6">
-        <f>IF(COUNT(T34:T35)=2,(T34/T35-1)*100,"")</f>
+        <f>IF(COUNT(T34:T35)=2,ROUND((T34/T35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW34" s="6">
-        <f>IF(COUNT(Y34:Y35)=2,(Y34/Y35-1)*100,"")</f>
+        <f>IF(COUNT(Y34:Y35)=2,ROUND((Y34/Y35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX34" s="6">
-        <f>IF(COUNT(AD34:AD35)=2,(AD34/AD35-1)*100,"")</f>
+        <f>IF(COUNT(AD34:AD35)=2,ROUND((AD34/AD35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY34" s="6">
-        <f>IF(COUNT(AI34:AI35)=2,(AI34/AI35-1)*100,"")</f>
+        <f>IF(COUNT(AI34:AI35)=2,ROUND((AI34/AI35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ34" s="6">
-        <f>IF(COUNT(AN34:AN35)=2,(AN34/AN35-1)*100,"")</f>
+        <f>IF(COUNT(AN34:AN35)=2,ROUND((AN34/AN35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA34" s="6">
-        <f>IF(COUNT(AS34:AS35)=2,(AS34/AS35-1)*100,"")</f>
+        <f>IF(COUNT(AS34:AS35)=2,ROUND((AS34/AS35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB34" s="5" t="n">
         <v>16.9</v>
       </c>
       <c r="BC34" s="6">
-        <f>IF(COUNT(BB34:BB35)=2,(BB34/BB35-1)*100,"")</f>
+        <f>IF(COUNT(BB34:BB35)=2,ROUND((BB34/BB35-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD34" s="6" t="n">
@@ -7709,11 +7709,11 @@
         <v>183.5</v>
       </c>
       <c r="D35" s="6">
-        <f>IF(COUNT(B35:B36)=2,(B35/B36-1)*100,"")</f>
+        <f>IF(COUNT(B35:B36)=2,ROUND((B35/B36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E35" s="6">
-        <f>IF(COUNT(C35:C36)=2,(C35/C36-1)*100,"")</f>
+        <f>IF(COUNT(C35:C36)=2,ROUND((C35/C36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F35" s="5" t="n">
@@ -7837,42 +7837,42 @@
         <v>111.02</v>
       </c>
       <c r="AT35" s="6">
-        <f>IF(COUNT(J35:J36)=2,(J35/J36-1)*100,"")</f>
+        <f>IF(COUNT(J35:J36)=2,ROUND((J35/J36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU35" s="6">
-        <f>IF(COUNT(O35:O36)=2,(O35/O36-1)*100,"")</f>
+        <f>IF(COUNT(O35:O36)=2,ROUND((O35/O36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV35" s="6">
-        <f>IF(COUNT(T35:T36)=2,(T35/T36-1)*100,"")</f>
+        <f>IF(COUNT(T35:T36)=2,ROUND((T35/T36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW35" s="6">
-        <f>IF(COUNT(Y35:Y36)=2,(Y35/Y36-1)*100,"")</f>
+        <f>IF(COUNT(Y35:Y36)=2,ROUND((Y35/Y36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX35" s="6">
-        <f>IF(COUNT(AD35:AD36)=2,(AD35/AD36-1)*100,"")</f>
+        <f>IF(COUNT(AD35:AD36)=2,ROUND((AD35/AD36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY35" s="6">
-        <f>IF(COUNT(AI35:AI36)=2,(AI35/AI36-1)*100,"")</f>
+        <f>IF(COUNT(AI35:AI36)=2,ROUND((AI35/AI36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ35" s="6">
-        <f>IF(COUNT(AN35:AN36)=2,(AN35/AN36-1)*100,"")</f>
+        <f>IF(COUNT(AN35:AN36)=2,ROUND((AN35/AN36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA35" s="6">
-        <f>IF(COUNT(AS35:AS36)=2,(AS35/AS36-1)*100,"")</f>
+        <f>IF(COUNT(AS35:AS36)=2,ROUND((AS35/AS36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB35" s="5" t="n">
         <v>16.13</v>
       </c>
       <c r="BC35" s="6">
-        <f>IF(COUNT(BB35:BB36)=2,(BB35/BB36-1)*100,"")</f>
+        <f>IF(COUNT(BB35:BB36)=2,ROUND((BB35/BB36-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD35" s="6" t="n">
@@ -7924,11 +7924,11 @@
         <v>185.21</v>
       </c>
       <c r="D36" s="6">
-        <f>IF(COUNT(B36:B37)=2,(B36/B37-1)*100,"")</f>
+        <f>IF(COUNT(B36:B37)=2,ROUND((B36/B37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E36" s="6">
-        <f>IF(COUNT(C36:C37)=2,(C36/C37-1)*100,"")</f>
+        <f>IF(COUNT(C36:C37)=2,ROUND((C36/C37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F36" s="5" t="n">
@@ -8052,42 +8052,42 @@
         <v>110.21</v>
       </c>
       <c r="AT36" s="6">
-        <f>IF(COUNT(J36:J37)=2,(J36/J37-1)*100,"")</f>
+        <f>IF(COUNT(J36:J37)=2,ROUND((J36/J37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU36" s="6">
-        <f>IF(COUNT(O36:O37)=2,(O36/O37-1)*100,"")</f>
+        <f>IF(COUNT(O36:O37)=2,ROUND((O36/O37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV36" s="6">
-        <f>IF(COUNT(T36:T37)=2,(T36/T37-1)*100,"")</f>
+        <f>IF(COUNT(T36:T37)=2,ROUND((T36/T37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW36" s="6">
-        <f>IF(COUNT(Y36:Y37)=2,(Y36/Y37-1)*100,"")</f>
+        <f>IF(COUNT(Y36:Y37)=2,ROUND((Y36/Y37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX36" s="6">
-        <f>IF(COUNT(AD36:AD37)=2,(AD36/AD37-1)*100,"")</f>
+        <f>IF(COUNT(AD36:AD37)=2,ROUND((AD36/AD37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY36" s="6">
-        <f>IF(COUNT(AI36:AI37)=2,(AI36/AI37-1)*100,"")</f>
+        <f>IF(COUNT(AI36:AI37)=2,ROUND((AI36/AI37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ36" s="6">
-        <f>IF(COUNT(AN36:AN37)=2,(AN36/AN37-1)*100,"")</f>
+        <f>IF(COUNT(AN36:AN37)=2,ROUND((AN36/AN37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA36" s="6">
-        <f>IF(COUNT(AS36:AS37)=2,(AS36/AS37-1)*100,"")</f>
+        <f>IF(COUNT(AS36:AS37)=2,ROUND((AS36/AS37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB36" s="5" t="n">
         <v>15.57</v>
       </c>
       <c r="BC36" s="6">
-        <f>IF(COUNT(BB36:BB37)=2,(BB36/BB37-1)*100,"")</f>
+        <f>IF(COUNT(BB36:BB37)=2,ROUND((BB36/BB37-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD36" s="6" t="n">
@@ -8139,11 +8139,11 @@
         <v>182.53</v>
       </c>
       <c r="D37" s="6">
-        <f>IF(COUNT(B37:B38)=2,(B37/B38-1)*100,"")</f>
+        <f>IF(COUNT(B37:B38)=2,ROUND((B37/B38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E37" s="6">
-        <f>IF(COUNT(C37:C38)=2,(C37/C38-1)*100,"")</f>
+        <f>IF(COUNT(C37:C38)=2,ROUND((C37/C38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F37" s="5" t="n">
@@ -8267,42 +8267,42 @@
         <v>109.6</v>
       </c>
       <c r="AT37" s="6">
-        <f>IF(COUNT(J37:J38)=2,(J37/J38-1)*100,"")</f>
+        <f>IF(COUNT(J37:J38)=2,ROUND((J37/J38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU37" s="6">
-        <f>IF(COUNT(O37:O38)=2,(O37/O38-1)*100,"")</f>
+        <f>IF(COUNT(O37:O38)=2,ROUND((O37/O38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV37" s="6">
-        <f>IF(COUNT(T37:T38)=2,(T37/T38-1)*100,"")</f>
+        <f>IF(COUNT(T37:T38)=2,ROUND((T37/T38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW37" s="6">
-        <f>IF(COUNT(Y37:Y38)=2,(Y37/Y38-1)*100,"")</f>
+        <f>IF(COUNT(Y37:Y38)=2,ROUND((Y37/Y38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX37" s="6">
-        <f>IF(COUNT(AD37:AD38)=2,(AD37/AD38-1)*100,"")</f>
+        <f>IF(COUNT(AD37:AD38)=2,ROUND((AD37/AD38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY37" s="6">
-        <f>IF(COUNT(AI37:AI38)=2,(AI37/AI38-1)*100,"")</f>
+        <f>IF(COUNT(AI37:AI38)=2,ROUND((AI37/AI38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ37" s="6">
-        <f>IF(COUNT(AN37:AN38)=2,(AN37/AN38-1)*100,"")</f>
+        <f>IF(COUNT(AN37:AN38)=2,ROUND((AN37/AN38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA37" s="6">
-        <f>IF(COUNT(AS37:AS38)=2,(AS37/AS38-1)*100,"")</f>
+        <f>IF(COUNT(AS37:AS38)=2,ROUND((AS37/AS38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB37" s="5" t="n">
         <v>16.15</v>
       </c>
       <c r="BC37" s="6">
-        <f>IF(COUNT(BB37:BB38)=2,(BB37/BB38-1)*100,"")</f>
+        <f>IF(COUNT(BB37:BB38)=2,ROUND((BB37/BB38-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD37" s="6" t="n">
@@ -8354,11 +8354,11 @@
         <v>182.68</v>
       </c>
       <c r="D38" s="6">
-        <f>IF(COUNT(B38:B39)=2,(B38/B39-1)*100,"")</f>
+        <f>IF(COUNT(B38:B39)=2,ROUND((B38/B39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E38" s="6">
-        <f>IF(COUNT(C38:C39)=2,(C38/C39-1)*100,"")</f>
+        <f>IF(COUNT(C38:C39)=2,ROUND((C38/C39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F38" s="5" t="n">
@@ -8482,42 +8482,42 @@
         <v>109.74</v>
       </c>
       <c r="AT38" s="6">
-        <f>IF(COUNT(J38:J39)=2,(J38/J39-1)*100,"")</f>
+        <f>IF(COUNT(J38:J39)=2,ROUND((J38/J39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU38" s="6">
-        <f>IF(COUNT(O38:O39)=2,(O38/O39-1)*100,"")</f>
+        <f>IF(COUNT(O38:O39)=2,ROUND((O38/O39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV38" s="6">
-        <f>IF(COUNT(T38:T39)=2,(T38/T39-1)*100,"")</f>
+        <f>IF(COUNT(T38:T39)=2,ROUND((T38/T39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW38" s="6">
-        <f>IF(COUNT(Y38:Y39)=2,(Y38/Y39-1)*100,"")</f>
+        <f>IF(COUNT(Y38:Y39)=2,ROUND((Y38/Y39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX38" s="6">
-        <f>IF(COUNT(AD38:AD39)=2,(AD38/AD39-1)*100,"")</f>
+        <f>IF(COUNT(AD38:AD39)=2,ROUND((AD38/AD39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY38" s="6">
-        <f>IF(COUNT(AI38:AI39)=2,(AI38/AI39-1)*100,"")</f>
+        <f>IF(COUNT(AI38:AI39)=2,ROUND((AI38/AI39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ38" s="6">
-        <f>IF(COUNT(AN38:AN39)=2,(AN38/AN39-1)*100,"")</f>
+        <f>IF(COUNT(AN38:AN39)=2,ROUND((AN38/AN39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA38" s="6">
-        <f>IF(COUNT(AS38:AS39)=2,(AS38/AS39-1)*100,"")</f>
+        <f>IF(COUNT(AS38:AS39)=2,ROUND((AS38/AS39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB38" s="5" t="n">
         <v>16.59</v>
       </c>
       <c r="BC38" s="6">
-        <f>IF(COUNT(BB38:BB39)=2,(BB38/BB39-1)*100,"")</f>
+        <f>IF(COUNT(BB38:BB39)=2,ROUND((BB38/BB39-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD38" s="6" t="n">
@@ -8569,11 +8569,11 @@
         <v>183.4</v>
       </c>
       <c r="D39" s="6">
-        <f>IF(COUNT(B39:B40)=2,(B39/B40-1)*100,"")</f>
+        <f>IF(COUNT(B39:B40)=2,ROUND((B39/B40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E39" s="6">
-        <f>IF(COUNT(C39:C40)=2,(C39/C40-1)*100,"")</f>
+        <f>IF(COUNT(C39:C40)=2,ROUND((C39/C40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F39" s="5" t="n">
@@ -8697,42 +8697,42 @@
         <v>107.13</v>
       </c>
       <c r="AT39" s="6">
-        <f>IF(COUNT(J39:J40)=2,(J39/J40-1)*100,"")</f>
+        <f>IF(COUNT(J39:J40)=2,ROUND((J39/J40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU39" s="6">
-        <f>IF(COUNT(O39:O40)=2,(O39/O40-1)*100,"")</f>
+        <f>IF(COUNT(O39:O40)=2,ROUND((O39/O40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV39" s="6">
-        <f>IF(COUNT(T39:T40)=2,(T39/T40-1)*100,"")</f>
+        <f>IF(COUNT(T39:T40)=2,ROUND((T39/T40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW39" s="6">
-        <f>IF(COUNT(Y39:Y40)=2,(Y39/Y40-1)*100,"")</f>
+        <f>IF(COUNT(Y39:Y40)=2,ROUND((Y39/Y40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX39" s="6">
-        <f>IF(COUNT(AD39:AD40)=2,(AD39/AD40-1)*100,"")</f>
+        <f>IF(COUNT(AD39:AD40)=2,ROUND((AD39/AD40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY39" s="6">
-        <f>IF(COUNT(AI39:AI40)=2,(AI39/AI40-1)*100,"")</f>
+        <f>IF(COUNT(AI39:AI40)=2,ROUND((AI39/AI40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ39" s="6">
-        <f>IF(COUNT(AN39:AN40)=2,(AN39/AN40-1)*100,"")</f>
+        <f>IF(COUNT(AN39:AN40)=2,ROUND((AN39/AN40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA39" s="6">
-        <f>IF(COUNT(AS39:AS40)=2,(AS39/AS40-1)*100,"")</f>
+        <f>IF(COUNT(AS39:AS40)=2,ROUND((AS39/AS40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB39" s="5" t="n">
         <v>16.45</v>
       </c>
       <c r="BC39" s="6">
-        <f>IF(COUNT(BB39:BB40)=2,(BB39/BB40-1)*100,"")</f>
+        <f>IF(COUNT(BB39:BB40)=2,ROUND((BB39/BB40-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD39" s="6" t="n">
@@ -8784,11 +8784,11 @@
         <v>180.59</v>
       </c>
       <c r="D40" s="6">
-        <f>IF(COUNT(B40:B41)=2,(B40/B41-1)*100,"")</f>
+        <f>IF(COUNT(B40:B41)=2,ROUND((B40/B41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E40" s="6">
-        <f>IF(COUNT(C40:C41)=2,(C40/C41-1)*100,"")</f>
+        <f>IF(COUNT(C40:C41)=2,ROUND((C40/C41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F40" s="5" t="n">
@@ -8912,42 +8912,42 @@
         <v>107.88</v>
       </c>
       <c r="AT40" s="6">
-        <f>IF(COUNT(J40:J41)=2,(J40/J41-1)*100,"")</f>
+        <f>IF(COUNT(J40:J41)=2,ROUND((J40/J41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU40" s="6">
-        <f>IF(COUNT(O40:O41)=2,(O40/O41-1)*100,"")</f>
+        <f>IF(COUNT(O40:O41)=2,ROUND((O40/O41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV40" s="6">
-        <f>IF(COUNT(T40:T41)=2,(T40/T41-1)*100,"")</f>
+        <f>IF(COUNT(T40:T41)=2,ROUND((T40/T41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW40" s="6">
-        <f>IF(COUNT(Y40:Y41)=2,(Y40/Y41-1)*100,"")</f>
+        <f>IF(COUNT(Y40:Y41)=2,ROUND((Y40/Y41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX40" s="6">
-        <f>IF(COUNT(AD40:AD41)=2,(AD40/AD41-1)*100,"")</f>
+        <f>IF(COUNT(AD40:AD41)=2,ROUND((AD40/AD41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY40" s="6">
-        <f>IF(COUNT(AI40:AI41)=2,(AI40/AI41-1)*100,"")</f>
+        <f>IF(COUNT(AI40:AI41)=2,ROUND((AI40/AI41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ40" s="6">
-        <f>IF(COUNT(AN40:AN41)=2,(AN40/AN41-1)*100,"")</f>
+        <f>IF(COUNT(AN40:AN41)=2,ROUND((AN40/AN41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA40" s="6">
-        <f>IF(COUNT(AS40:AS41)=2,(AS40/AS41-1)*100,"")</f>
+        <f>IF(COUNT(AS40:AS41)=2,ROUND((AS40/AS41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB40" s="5" t="n">
         <v>17.65</v>
       </c>
       <c r="BC40" s="6">
-        <f>IF(COUNT(BB40:BB41)=2,(BB40/BB41-1)*100,"")</f>
+        <f>IF(COUNT(BB40:BB41)=2,ROUND((BB40/BB41-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD40" s="6" t="n">
@@ -8999,11 +8999,11 @@
         <v>176.27</v>
       </c>
       <c r="D41" s="6">
-        <f>IF(COUNT(B41:B42)=2,(B41/B42-1)*100,"")</f>
+        <f>IF(COUNT(B41:B42)=2,ROUND((B41/B42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E41" s="6">
-        <f>IF(COUNT(C41:C42)=2,(C41/C42-1)*100,"")</f>
+        <f>IF(COUNT(C41:C42)=2,ROUND((C41/C42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F41" s="5" t="n">
@@ -9127,42 +9127,42 @@
         <v>106.18</v>
       </c>
       <c r="AT41" s="6">
-        <f>IF(COUNT(J41:J42)=2,(J41/J42-1)*100,"")</f>
+        <f>IF(COUNT(J41:J42)=2,ROUND((J41/J42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU41" s="6">
-        <f>IF(COUNT(O41:O42)=2,(O41/O42-1)*100,"")</f>
+        <f>IF(COUNT(O41:O42)=2,ROUND((O41/O42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV41" s="6">
-        <f>IF(COUNT(T41:T42)=2,(T41/T42-1)*100,"")</f>
+        <f>IF(COUNT(T41:T42)=2,ROUND((T41/T42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW41" s="6">
-        <f>IF(COUNT(Y41:Y42)=2,(Y41/Y42-1)*100,"")</f>
+        <f>IF(COUNT(Y41:Y42)=2,ROUND((Y41/Y42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX41" s="6">
-        <f>IF(COUNT(AD41:AD42)=2,(AD41/AD42-1)*100,"")</f>
+        <f>IF(COUNT(AD41:AD42)=2,ROUND((AD41/AD42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY41" s="6">
-        <f>IF(COUNT(AI41:AI42)=2,(AI41/AI42-1)*100,"")</f>
+        <f>IF(COUNT(AI41:AI42)=2,ROUND((AI41/AI42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ41" s="6">
-        <f>IF(COUNT(AN41:AN42)=2,(AN41/AN42-1)*100,"")</f>
+        <f>IF(COUNT(AN41:AN42)=2,ROUND((AN41/AN42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA41" s="6">
-        <f>IF(COUNT(AS41:AS42)=2,(AS41/AS42-1)*100,"")</f>
+        <f>IF(COUNT(AS41:AS42)=2,ROUND((AS41/AS42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB41" s="5" t="n">
         <v>18.41</v>
       </c>
       <c r="BC41" s="6">
-        <f>IF(COUNT(BB41:BB42)=2,(BB41/BB42-1)*100,"")</f>
+        <f>IF(COUNT(BB41:BB42)=2,ROUND((BB41/BB42-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD41" s="6" t="n">
@@ -9214,11 +9214,11 @@
         <v>176.82</v>
       </c>
       <c r="D42" s="6">
-        <f>IF(COUNT(B42:B43)=2,(B42/B43-1)*100,"")</f>
+        <f>IF(COUNT(B42:B43)=2,ROUND((B42/B43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E42" s="6">
-        <f>IF(COUNT(C42:C43)=2,(C42/C43-1)*100,"")</f>
+        <f>IF(COUNT(C42:C43)=2,ROUND((C42/C43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F42" s="5" t="n">
@@ -9342,42 +9342,42 @@
         <v>105.58</v>
       </c>
       <c r="AT42" s="6">
-        <f>IF(COUNT(J42:J43)=2,(J42/J43-1)*100,"")</f>
+        <f>IF(COUNT(J42:J43)=2,ROUND((J42/J43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU42" s="6">
-        <f>IF(COUNT(O42:O43)=2,(O42/O43-1)*100,"")</f>
+        <f>IF(COUNT(O42:O43)=2,ROUND((O42/O43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV42" s="6">
-        <f>IF(COUNT(T42:T43)=2,(T42/T43-1)*100,"")</f>
+        <f>IF(COUNT(T42:T43)=2,ROUND((T42/T43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW42" s="6">
-        <f>IF(COUNT(Y42:Y43)=2,(Y42/Y43-1)*100,"")</f>
+        <f>IF(COUNT(Y42:Y43)=2,ROUND((Y42/Y43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX42" s="6">
-        <f>IF(COUNT(AD42:AD43)=2,(AD42/AD43-1)*100,"")</f>
+        <f>IF(COUNT(AD42:AD43)=2,ROUND((AD42/AD43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY42" s="6">
-        <f>IF(COUNT(AI42:AI43)=2,(AI42/AI43-1)*100,"")</f>
+        <f>IF(COUNT(AI42:AI43)=2,ROUND((AI42/AI43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ42" s="6">
-        <f>IF(COUNT(AN42:AN43)=2,(AN42/AN43-1)*100,"")</f>
+        <f>IF(COUNT(AN42:AN43)=2,ROUND((AN42/AN43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA42" s="6">
-        <f>IF(COUNT(AS42:AS43)=2,(AS42/AS43-1)*100,"")</f>
+        <f>IF(COUNT(AS42:AS43)=2,ROUND((AS42/AS43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB42" s="5" t="n">
         <v>18.89</v>
       </c>
       <c r="BC42" s="6">
-        <f>IF(COUNT(BB42:BB43)=2,(BB42/BB43-1)*100,"")</f>
+        <f>IF(COUNT(BB42:BB43)=2,ROUND((BB42/BB43-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD42" s="6" t="n">
@@ -9429,11 +9429,11 @@
         <v>176.82</v>
       </c>
       <c r="D43" s="6">
-        <f>IF(COUNT(B43:B44)=2,(B43/B44-1)*100,"")</f>
+        <f>IF(COUNT(B43:B44)=2,ROUND((B43/B44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E43" s="6">
-        <f>IF(COUNT(C43:C44)=2,(C43/C44-1)*100,"")</f>
+        <f>IF(COUNT(C43:C44)=2,ROUND((C43/C44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F43" s="5" t="n">
@@ -9557,42 +9557,42 @@
         <v>106.54</v>
       </c>
       <c r="AT43" s="6">
-        <f>IF(COUNT(J43:J44)=2,(J43/J44-1)*100,"")</f>
+        <f>IF(COUNT(J43:J44)=2,ROUND((J43/J44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU43" s="6">
-        <f>IF(COUNT(O43:O44)=2,(O43/O44-1)*100,"")</f>
+        <f>IF(COUNT(O43:O44)=2,ROUND((O43/O44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV43" s="6">
-        <f>IF(COUNT(T43:T44)=2,(T43/T44-1)*100,"")</f>
+        <f>IF(COUNT(T43:T44)=2,ROUND((T43/T44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW43" s="6">
-        <f>IF(COUNT(Y43:Y44)=2,(Y43/Y44-1)*100,"")</f>
+        <f>IF(COUNT(Y43:Y44)=2,ROUND((Y43/Y44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX43" s="6">
-        <f>IF(COUNT(AD43:AD44)=2,(AD43/AD44-1)*100,"")</f>
+        <f>IF(COUNT(AD43:AD44)=2,ROUND((AD43/AD44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY43" s="6">
-        <f>IF(COUNT(AI43:AI44)=2,(AI43/AI44-1)*100,"")</f>
+        <f>IF(COUNT(AI43:AI44)=2,ROUND((AI43/AI44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ43" s="6">
-        <f>IF(COUNT(AN43:AN44)=2,(AN43/AN44-1)*100,"")</f>
+        <f>IF(COUNT(AN43:AN44)=2,ROUND((AN43/AN44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA43" s="6">
-        <f>IF(COUNT(AS43:AS44)=2,(AS43/AS44-1)*100,"")</f>
+        <f>IF(COUNT(AS43:AS44)=2,ROUND((AS43/AS44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB43" s="5" t="n">
         <v>18.63</v>
       </c>
       <c r="BC43" s="6">
-        <f>IF(COUNT(BB43:BB44)=2,(BB43/BB44-1)*100,"")</f>
+        <f>IF(COUNT(BB43:BB44)=2,ROUND((BB43/BB44-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD43" s="6" t="n">
@@ -9644,11 +9644,11 @@
         <v>177.18</v>
       </c>
       <c r="D44" s="6">
-        <f>IF(COUNT(B44:B45)=2,(B44/B45-1)*100,"")</f>
+        <f>IF(COUNT(B44:B45)=2,ROUND((B44/B45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E44" s="6">
-        <f>IF(COUNT(C44:C45)=2,(C44/C45-1)*100,"")</f>
+        <f>IF(COUNT(C44:C45)=2,ROUND((C44/C45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F44" s="5" t="n">
@@ -9772,42 +9772,42 @@
         <v>107.27</v>
       </c>
       <c r="AT44" s="6">
-        <f>IF(COUNT(J44:J45)=2,(J44/J45-1)*100,"")</f>
+        <f>IF(COUNT(J44:J45)=2,ROUND((J44/J45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU44" s="6">
-        <f>IF(COUNT(O44:O45)=2,(O44/O45-1)*100,"")</f>
+        <f>IF(COUNT(O44:O45)=2,ROUND((O44/O45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV44" s="6">
-        <f>IF(COUNT(T44:T45)=2,(T44/T45-1)*100,"")</f>
+        <f>IF(COUNT(T44:T45)=2,ROUND((T44/T45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW44" s="6">
-        <f>IF(COUNT(Y44:Y45)=2,(Y44/Y45-1)*100,"")</f>
+        <f>IF(COUNT(Y44:Y45)=2,ROUND((Y44/Y45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX44" s="6">
-        <f>IF(COUNT(AD44:AD45)=2,(AD44/AD45-1)*100,"")</f>
+        <f>IF(COUNT(AD44:AD45)=2,ROUND((AD44/AD45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY44" s="6">
-        <f>IF(COUNT(AI44:AI45)=2,(AI44/AI45-1)*100,"")</f>
+        <f>IF(COUNT(AI44:AI45)=2,ROUND((AI44/AI45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ44" s="6">
-        <f>IF(COUNT(AN44:AN45)=2,(AN44/AN45-1)*100,"")</f>
+        <f>IF(COUNT(AN44:AN45)=2,ROUND((AN44/AN45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA44" s="6">
-        <f>IF(COUNT(AS44:AS45)=2,(AS44/AS45-1)*100,"")</f>
+        <f>IF(COUNT(AS44:AS45)=2,ROUND((AS44/AS45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB44" s="5" t="n">
         <v>19.49</v>
       </c>
       <c r="BC44" s="6">
-        <f>IF(COUNT(BB44:BB45)=2,(BB44/BB45-1)*100,"")</f>
+        <f>IF(COUNT(BB44:BB45)=2,ROUND((BB44/BB45-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD44" s="6" t="n">
@@ -9859,11 +9859,11 @@
         <v>182.43</v>
       </c>
       <c r="D45" s="6">
-        <f>IF(COUNT(B45:B46)=2,(B45/B46-1)*100,"")</f>
+        <f>IF(COUNT(B45:B46)=2,ROUND((B45/B46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E45" s="6">
-        <f>IF(COUNT(C45:C46)=2,(C45/C46-1)*100,"")</f>
+        <f>IF(COUNT(C45:C46)=2,ROUND((C45/C46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F45" s="5" t="n">
@@ -9987,42 +9987,42 @@
         <v>106.86</v>
       </c>
       <c r="AT45" s="6">
-        <f>IF(COUNT(J45:J46)=2,(J45/J46-1)*100,"")</f>
+        <f>IF(COUNT(J45:J46)=2,ROUND((J45/J46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU45" s="6">
-        <f>IF(COUNT(O45:O46)=2,(O45/O46-1)*100,"")</f>
+        <f>IF(COUNT(O45:O46)=2,ROUND((O45/O46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV45" s="6">
-        <f>IF(COUNT(T45:T46)=2,(T45/T46-1)*100,"")</f>
+        <f>IF(COUNT(T45:T46)=2,ROUND((T45/T46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW45" s="6">
-        <f>IF(COUNT(Y45:Y46)=2,(Y45/Y46-1)*100,"")</f>
+        <f>IF(COUNT(Y45:Y46)=2,ROUND((Y45/Y46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX45" s="6">
-        <f>IF(COUNT(AD45:AD46)=2,(AD45/AD46-1)*100,"")</f>
+        <f>IF(COUNT(AD45:AD46)=2,ROUND((AD45/AD46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY45" s="6">
-        <f>IF(COUNT(AI45:AI46)=2,(AI45/AI46-1)*100,"")</f>
+        <f>IF(COUNT(AI45:AI46)=2,ROUND((AI45/AI46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ45" s="6">
-        <f>IF(COUNT(AN45:AN46)=2,(AN45/AN46-1)*100,"")</f>
+        <f>IF(COUNT(AN45:AN46)=2,ROUND((AN45/AN46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA45" s="6">
-        <f>IF(COUNT(AS45:AS46)=2,(AS45/AS46-1)*100,"")</f>
+        <f>IF(COUNT(AS45:AS46)=2,ROUND((AS45/AS46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB45" s="5" t="n">
         <v>17.28</v>
       </c>
       <c r="BC45" s="6">
-        <f>IF(COUNT(BB45:BB46)=2,(BB45/BB46-1)*100,"")</f>
+        <f>IF(COUNT(BB45:BB46)=2,ROUND((BB45/BB46-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD45" s="6" t="n">
@@ -10074,11 +10074,11 @@
         <v>183.86</v>
       </c>
       <c r="D46" s="6">
-        <f>IF(COUNT(B46:B47)=2,(B46/B47-1)*100,"")</f>
+        <f>IF(COUNT(B46:B47)=2,ROUND((B46/B47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E46" s="6">
-        <f>IF(COUNT(C46:C47)=2,(C46/C47-1)*100,"")</f>
+        <f>IF(COUNT(C46:C47)=2,ROUND((C46/C47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F46" s="5" t="n">
@@ -10202,42 +10202,42 @@
         <v>109.166</v>
       </c>
       <c r="AT46" s="6">
-        <f>IF(COUNT(J46:J47)=2,(J46/J47-1)*100,"")</f>
+        <f>IF(COUNT(J46:J47)=2,ROUND((J46/J47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU46" s="6">
-        <f>IF(COUNT(O46:O47)=2,(O46/O47-1)*100,"")</f>
+        <f>IF(COUNT(O46:O47)=2,ROUND((O46/O47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV46" s="6">
-        <f>IF(COUNT(T46:T47)=2,(T46/T47-1)*100,"")</f>
+        <f>IF(COUNT(T46:T47)=2,ROUND((T46/T47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW46" s="6">
-        <f>IF(COUNT(Y46:Y47)=2,(Y46/Y47-1)*100,"")</f>
+        <f>IF(COUNT(Y46:Y47)=2,ROUND((Y46/Y47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX46" s="6">
-        <f>IF(COUNT(AD46:AD47)=2,(AD46/AD47-1)*100,"")</f>
+        <f>IF(COUNT(AD46:AD47)=2,ROUND((AD46/AD47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY46" s="6">
-        <f>IF(COUNT(AI46:AI47)=2,(AI46/AI47-1)*100,"")</f>
+        <f>IF(COUNT(AI46:AI47)=2,ROUND((AI46/AI47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ46" s="6">
-        <f>IF(COUNT(AN46:AN47)=2,(AN46/AN47-1)*100,"")</f>
+        <f>IF(COUNT(AN46:AN47)=2,ROUND((AN46/AN47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA46" s="6">
-        <f>IF(COUNT(AS46:AS47)=2,(AS46/AS47-1)*100,"")</f>
+        <f>IF(COUNT(AS46:AS47)=2,ROUND((AS46/AS47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB46" s="5" t="n">
         <v>16.4</v>
       </c>
       <c r="BC46" s="6">
-        <f>IF(COUNT(BB46:BB47)=2,(BB46/BB47-1)*100,"")</f>
+        <f>IF(COUNT(BB46:BB47)=2,ROUND((BB46/BB47-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD46" s="6" t="n">
@@ -10289,11 +10289,11 @@
         <v>180</v>
       </c>
       <c r="D47" s="6">
-        <f>IF(COUNT(B47:B48)=2,(B47/B48-1)*100,"")</f>
+        <f>IF(COUNT(B47:B48)=2,ROUND((B47/B48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E47" s="6">
-        <f>IF(COUNT(C47:C48)=2,(C47/C48-1)*100,"")</f>
+        <f>IF(COUNT(C47:C48)=2,ROUND((C47/C48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F47" s="5" t="n">
@@ -10417,42 +10417,42 @@
         <v>108.9166</v>
       </c>
       <c r="AT47" s="6">
-        <f>IF(COUNT(J47:J48)=2,(J47/J48-1)*100,"")</f>
+        <f>IF(COUNT(J47:J48)=2,ROUND((J47/J48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU47" s="6">
-        <f>IF(COUNT(O47:O48)=2,(O47/O48-1)*100,"")</f>
+        <f>IF(COUNT(O47:O48)=2,ROUND((O47/O48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV47" s="6">
-        <f>IF(COUNT(T47:T48)=2,(T47/T48-1)*100,"")</f>
+        <f>IF(COUNT(T47:T48)=2,ROUND((T47/T48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW47" s="6">
-        <f>IF(COUNT(Y47:Y48)=2,(Y47/Y48-1)*100,"")</f>
+        <f>IF(COUNT(Y47:Y48)=2,ROUND((Y47/Y48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX47" s="6">
-        <f>IF(COUNT(AD47:AD48)=2,(AD47/AD48-1)*100,"")</f>
+        <f>IF(COUNT(AD47:AD48)=2,ROUND((AD47/AD48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY47" s="6">
-        <f>IF(COUNT(AI47:AI48)=2,(AI47/AI48-1)*100,"")</f>
+        <f>IF(COUNT(AI47:AI48)=2,ROUND((AI47/AI48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ47" s="6">
-        <f>IF(COUNT(AN47:AN48)=2,(AN47/AN48-1)*100,"")</f>
+        <f>IF(COUNT(AN47:AN48)=2,ROUND((AN47/AN48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA47" s="6">
-        <f>IF(COUNT(AS47:AS48)=2,(AS47/AS48-1)*100,"")</f>
+        <f>IF(COUNT(AS47:AS48)=2,ROUND((AS47/AS48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB47" s="5" t="n">
         <v>18.44</v>
       </c>
       <c r="BC47" s="6">
-        <f>IF(COUNT(BB47:BB48)=2,(BB47/BB48-1)*100,"")</f>
+        <f>IF(COUNT(BB47:BB48)=2,ROUND((BB47/BB48-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD47" s="6" t="n">
@@ -10504,11 +10504,11 @@
         <v>184.56</v>
       </c>
       <c r="D48" s="6">
-        <f>IF(COUNT(B48:B49)=2,(B48/B49-1)*100,"")</f>
+        <f>IF(COUNT(B48:B49)=2,ROUND((B48/B49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E48" s="6">
-        <f>IF(COUNT(C48:C49)=2,(C48/C49-1)*100,"")</f>
+        <f>IF(COUNT(C48:C49)=2,ROUND((C48/C49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F48" s="5" t="n">
@@ -10632,42 +10632,42 @@
         <v>112.0286</v>
       </c>
       <c r="AT48" s="6">
-        <f>IF(COUNT(J48:J49)=2,(J48/J49-1)*100,"")</f>
+        <f>IF(COUNT(J48:J49)=2,ROUND((J48/J49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU48" s="6">
-        <f>IF(COUNT(O48:O49)=2,(O48/O49-1)*100,"")</f>
+        <f>IF(COUNT(O48:O49)=2,ROUND((O48/O49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV48" s="6">
-        <f>IF(COUNT(T48:T49)=2,(T48/T49-1)*100,"")</f>
+        <f>IF(COUNT(T48:T49)=2,ROUND((T48/T49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW48" s="6">
-        <f>IF(COUNT(Y48:Y49)=2,(Y48/Y49-1)*100,"")</f>
+        <f>IF(COUNT(Y48:Y49)=2,ROUND((Y48/Y49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX48" s="6">
-        <f>IF(COUNT(AD48:AD49)=2,(AD48/AD49-1)*100,"")</f>
+        <f>IF(COUNT(AD48:AD49)=2,ROUND((AD48/AD49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY48" s="6">
-        <f>IF(COUNT(AI48:AI49)=2,(AI48/AI49-1)*100,"")</f>
+        <f>IF(COUNT(AI48:AI49)=2,ROUND((AI48/AI49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ48" s="6">
-        <f>IF(COUNT(AN48:AN49)=2,(AN48/AN49-1)*100,"")</f>
+        <f>IF(COUNT(AN48:AN49)=2,ROUND((AN48/AN49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA48" s="6">
-        <f>IF(COUNT(AS48:AS49)=2,(AS48/AS49-1)*100,"")</f>
+        <f>IF(COUNT(AS48:AS49)=2,ROUND((AS48/AS49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB48" s="5" t="n">
         <v>16.41</v>
       </c>
       <c r="BC48" s="6">
-        <f>IF(COUNT(BB48:BB49)=2,(BB48/BB49-1)*100,"")</f>
+        <f>IF(COUNT(BB48:BB49)=2,ROUND((BB48/BB49-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD48" s="6" t="n">
@@ -10719,11 +10719,11 @@
         <v>186.69</v>
       </c>
       <c r="D49" s="6">
-        <f>IF(COUNT(B49:B50)=2,(B49/B50-1)*100,"")</f>
+        <f>IF(COUNT(B49:B50)=2,ROUND((B49/B50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E49" s="6">
-        <f>IF(COUNT(C49:C50)=2,(C49/C50-1)*100,"")</f>
+        <f>IF(COUNT(C49:C50)=2,ROUND((C49/C50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F49" s="5" t="n">
@@ -10847,42 +10847,42 @@
         <v>111.8989</v>
       </c>
       <c r="AT49" s="6">
-        <f>IF(COUNT(J49:J50)=2,(J49/J50-1)*100,"")</f>
+        <f>IF(COUNT(J49:J50)=2,ROUND((J49/J50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU49" s="6">
-        <f>IF(COUNT(O49:O50)=2,(O49/O50-1)*100,"")</f>
+        <f>IF(COUNT(O49:O50)=2,ROUND((O49/O50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV49" s="6">
-        <f>IF(COUNT(T49:T50)=2,(T49/T50-1)*100,"")</f>
+        <f>IF(COUNT(T49:T50)=2,ROUND((T49/T50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW49" s="6">
-        <f>IF(COUNT(Y49:Y50)=2,(Y49/Y50-1)*100,"")</f>
+        <f>IF(COUNT(Y49:Y50)=2,ROUND((Y49/Y50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX49" s="6">
-        <f>IF(COUNT(AD49:AD50)=2,(AD49/AD50-1)*100,"")</f>
+        <f>IF(COUNT(AD49:AD50)=2,ROUND((AD49/AD50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY49" s="6">
-        <f>IF(COUNT(AI49:AI50)=2,(AI49/AI50-1)*100,"")</f>
+        <f>IF(COUNT(AI49:AI50)=2,ROUND((AI49/AI50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ49" s="6">
-        <f>IF(COUNT(AN49:AN50)=2,(AN49/AN50-1)*100,"")</f>
+        <f>IF(COUNT(AN49:AN50)=2,ROUND((AN49/AN50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA49" s="6">
-        <f>IF(COUNT(AS49:AS50)=2,(AS49/AS50-1)*100,"")</f>
+        <f>IF(COUNT(AS49:AS50)=2,ROUND((AS49/AS50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB49" s="5" t="n">
         <v>16.2</v>
       </c>
       <c r="BC49" s="6">
-        <f>IF(COUNT(BB49:BB50)=2,(BB49/BB50-1)*100,"")</f>
+        <f>IF(COUNT(BB49:BB50)=2,ROUND((BB49/BB50-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD49" s="6" t="n">
@@ -10934,11 +10934,11 @@
         <v>180.68</v>
       </c>
       <c r="D50" s="6">
-        <f>IF(COUNT(B50:B51)=2,(B50/B51-1)*100,"")</f>
+        <f>IF(COUNT(B50:B51)=2,ROUND((B50/B51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E50" s="6">
-        <f>IF(COUNT(C50:C51)=2,(C50/C51-1)*100,"")</f>
+        <f>IF(COUNT(C50:C51)=2,ROUND((C50/C51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F50" s="5" t="n">
@@ -11062,42 +11062,42 @@
         <v>111.3603</v>
       </c>
       <c r="AT50" s="6">
-        <f>IF(COUNT(J50:J51)=2,(J50/J51-1)*100,"")</f>
+        <f>IF(COUNT(J50:J51)=2,ROUND((J50/J51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU50" s="6">
-        <f>IF(COUNT(O50:O51)=2,(O50/O51-1)*100,"")</f>
+        <f>IF(COUNT(O50:O51)=2,ROUND((O50/O51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV50" s="6">
-        <f>IF(COUNT(T50:T51)=2,(T50/T51-1)*100,"")</f>
+        <f>IF(COUNT(T50:T51)=2,ROUND((T50/T51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW50" s="6">
-        <f>IF(COUNT(Y50:Y51)=2,(Y50/Y51-1)*100,"")</f>
+        <f>IF(COUNT(Y50:Y51)=2,ROUND((Y50/Y51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX50" s="6">
-        <f>IF(COUNT(AD50:AD51)=2,(AD50/AD51-1)*100,"")</f>
+        <f>IF(COUNT(AD50:AD51)=2,ROUND((AD50/AD51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY50" s="6">
-        <f>IF(COUNT(AI50:AI51)=2,(AI50/AI51-1)*100,"")</f>
+        <f>IF(COUNT(AI50:AI51)=2,ROUND((AI50/AI51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ50" s="6">
-        <f>IF(COUNT(AN50:AN51)=2,(AN50/AN51-1)*100,"")</f>
+        <f>IF(COUNT(AN50:AN51)=2,ROUND((AN50/AN51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA50" s="6">
-        <f>IF(COUNT(AS50:AS51)=2,(AS50/AS51-1)*100,"")</f>
+        <f>IF(COUNT(AS50:AS51)=2,ROUND((AS50/AS51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB50" s="5" t="n">
         <v>17.68</v>
       </c>
       <c r="BC50" s="6">
-        <f>IF(COUNT(BB50:BB51)=2,(BB50/BB51-1)*100,"")</f>
+        <f>IF(COUNT(BB50:BB51)=2,ROUND((BB50/BB51-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD50" s="6" t="n">
@@ -11149,11 +11149,11 @@
         <v>178.87</v>
       </c>
       <c r="D51" s="6">
-        <f>IF(COUNT(B51:B52)=2,(B51/B52-1)*100,"")</f>
+        <f>IF(COUNT(B51:B52)=2,ROUND((B51/B52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E51" s="6">
-        <f>IF(COUNT(C51:C52)=2,(C51/C52-1)*100,"")</f>
+        <f>IF(COUNT(C51:C52)=2,ROUND((C51/C52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F51" s="5" t="n">
@@ -11277,42 +11277,42 @@
         <v>111.8291</v>
       </c>
       <c r="AT51" s="6">
-        <f>IF(COUNT(J51:J52)=2,(J51/J52-1)*100,"")</f>
+        <f>IF(COUNT(J51:J52)=2,ROUND((J51/J52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU51" s="6">
-        <f>IF(COUNT(O51:O52)=2,(O51/O52-1)*100,"")</f>
+        <f>IF(COUNT(O51:O52)=2,ROUND((O51/O52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV51" s="6">
-        <f>IF(COUNT(T51:T52)=2,(T51/T52-1)*100,"")</f>
+        <f>IF(COUNT(T51:T52)=2,ROUND((T51/T52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW51" s="6">
-        <f>IF(COUNT(Y51:Y52)=2,(Y51/Y52-1)*100,"")</f>
+        <f>IF(COUNT(Y51:Y52)=2,ROUND((Y51/Y52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX51" s="6">
-        <f>IF(COUNT(AD51:AD52)=2,(AD51/AD52-1)*100,"")</f>
+        <f>IF(COUNT(AD51:AD52)=2,ROUND((AD51/AD52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY51" s="6">
-        <f>IF(COUNT(AI51:AI52)=2,(AI51/AI52-1)*100,"")</f>
+        <f>IF(COUNT(AI51:AI52)=2,ROUND((AI51/AI52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ51" s="6">
-        <f>IF(COUNT(AN51:AN52)=2,(AN51/AN52-1)*100,"")</f>
+        <f>IF(COUNT(AN51:AN52)=2,ROUND((AN51/AN52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA51" s="6">
-        <f>IF(COUNT(AS51:AS52)=2,(AS51/AS52-1)*100,"")</f>
+        <f>IF(COUNT(AS51:AS52)=2,ROUND((AS51/AS52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB51" s="5" t="n">
         <v>19.44</v>
       </c>
       <c r="BC51" s="6">
-        <f>IF(COUNT(BB51:BB52)=2,(BB51/BB52-1)*100,"")</f>
+        <f>IF(COUNT(BB51:BB52)=2,ROUND((BB51/BB52-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD51" s="6" t="n">
@@ -11364,11 +11364,11 @@
         <v>172.89</v>
       </c>
       <c r="D52" s="6">
-        <f>IF(COUNT(B52:B53)=2,(B52/B53-1)*100,"")</f>
+        <f>IF(COUNT(B52:B53)=2,ROUND((B52/B53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E52" s="6">
-        <f>IF(COUNT(C52:C53)=2,(C52/C53-1)*100,"")</f>
+        <f>IF(COUNT(C52:C53)=2,ROUND((C52/C53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F52" s="5" t="n">
@@ -11492,42 +11492,42 @@
         <v>110.722</v>
       </c>
       <c r="AT52" s="6">
-        <f>IF(COUNT(J52:J53)=2,(J52/J53-1)*100,"")</f>
+        <f>IF(COUNT(J52:J53)=2,ROUND((J52/J53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU52" s="6">
-        <f>IF(COUNT(O52:O53)=2,(O52/O53-1)*100,"")</f>
+        <f>IF(COUNT(O52:O53)=2,ROUND((O52/O53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV52" s="6">
-        <f>IF(COUNT(T52:T53)=2,(T52/T53-1)*100,"")</f>
+        <f>IF(COUNT(T52:T53)=2,ROUND((T52/T53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW52" s="6">
-        <f>IF(COUNT(Y52:Y53)=2,(Y52/Y53-1)*100,"")</f>
+        <f>IF(COUNT(Y52:Y53)=2,ROUND((Y52/Y53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX52" s="6">
-        <f>IF(COUNT(AD52:AD53)=2,(AD52/AD53-1)*100,"")</f>
+        <f>IF(COUNT(AD52:AD53)=2,ROUND((AD52/AD53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY52" s="6">
-        <f>IF(COUNT(AI52:AI53)=2,(AI52/AI53-1)*100,"")</f>
+        <f>IF(COUNT(AI52:AI53)=2,ROUND((AI52/AI53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ52" s="6">
-        <f>IF(COUNT(AN52:AN53)=2,(AN52/AN53-1)*100,"")</f>
+        <f>IF(COUNT(AN52:AN53)=2,ROUND((AN52/AN53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA52" s="6">
-        <f>IF(COUNT(AS52:AS53)=2,(AS52/AS53-1)*100,"")</f>
+        <f>IF(COUNT(AS52:AS53)=2,ROUND((AS52/AS53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB52" s="5" t="n">
         <v>22.22</v>
       </c>
       <c r="BC52" s="6">
-        <f>IF(COUNT(BB52:BB53)=2,(BB52/BB53-1)*100,"")</f>
+        <f>IF(COUNT(BB52:BB53)=2,ROUND((BB52/BB53-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD52" s="6" t="n">
@@ -11579,11 +11579,11 @@
         <v>178.67</v>
       </c>
       <c r="D53" s="6">
-        <f>IF(COUNT(B53:B54)=2,(B53/B54-1)*100,"")</f>
+        <f>IF(COUNT(B53:B54)=2,ROUND((B53/B54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E53" s="6">
-        <f>IF(COUNT(C53:C54)=2,(C53/C54-1)*100,"")</f>
+        <f>IF(COUNT(C53:C54)=2,ROUND((C53/C54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F53" s="5" t="n">
@@ -11707,42 +11707,42 @@
         <v>111.1907</v>
       </c>
       <c r="AT53" s="6">
-        <f>IF(COUNT(J53:J54)=2,(J53/J54-1)*100,"")</f>
+        <f>IF(COUNT(J53:J54)=2,ROUND((J53/J54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU53" s="6">
-        <f>IF(COUNT(O53:O54)=2,(O53/O54-1)*100,"")</f>
+        <f>IF(COUNT(O53:O54)=2,ROUND((O53/O54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV53" s="6">
-        <f>IF(COUNT(T53:T54)=2,(T53/T54-1)*100,"")</f>
+        <f>IF(COUNT(T53:T54)=2,ROUND((T53/T54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW53" s="6">
-        <f>IF(COUNT(Y53:Y54)=2,(Y53/Y54-1)*100,"")</f>
+        <f>IF(COUNT(Y53:Y54)=2,ROUND((Y53/Y54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX53" s="6">
-        <f>IF(COUNT(AD53:AD54)=2,(AD53/AD54-1)*100,"")</f>
+        <f>IF(COUNT(AD53:AD54)=2,ROUND((AD53/AD54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY53" s="6">
-        <f>IF(COUNT(AI53:AI54)=2,(AI53/AI54-1)*100,"")</f>
+        <f>IF(COUNT(AI53:AI54)=2,ROUND((AI53/AI54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ53" s="6">
-        <f>IF(COUNT(AN53:AN54)=2,(AN53/AN54-1)*100,"")</f>
+        <f>IF(COUNT(AN53:AN54)=2,ROUND((AN53/AN54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA53" s="6">
-        <f>IF(COUNT(AS53:AS54)=2,(AS53/AS54-1)*100,"")</f>
+        <f>IF(COUNT(AS53:AS54)=2,ROUND((AS53/AS54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB53" s="5" t="n">
         <v>19.87</v>
       </c>
       <c r="BC53" s="6">
-        <f>IF(COUNT(BB53:BB54)=2,(BB53/BB54-1)*100,"")</f>
+        <f>IF(COUNT(BB53:BB54)=2,ROUND((BB53/BB54-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD53" s="6" t="n">
@@ -11794,11 +11794,11 @@
         <v>179.65</v>
       </c>
       <c r="D54" s="6">
-        <f>IF(COUNT(B54:B55)=2,(B54/B55-1)*100,"")</f>
+        <f>IF(COUNT(B54:B55)=2,ROUND((B54/B55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E54" s="6">
-        <f>IF(COUNT(C54:C55)=2,(C54/C55-1)*100,"")</f>
+        <f>IF(COUNT(C54:C55)=2,ROUND((C54/C55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F54" s="5" t="n">
@@ -11922,42 +11922,42 @@
         <v>110.8017</v>
       </c>
       <c r="AT54" s="6">
-        <f>IF(COUNT(J54:J55)=2,(J54/J55-1)*100,"")</f>
+        <f>IF(COUNT(J54:J55)=2,ROUND((J54/J55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU54" s="6">
-        <f>IF(COUNT(O54:O55)=2,(O54/O55-1)*100,"")</f>
+        <f>IF(COUNT(O54:O55)=2,ROUND((O54/O55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV54" s="6">
-        <f>IF(COUNT(T54:T55)=2,(T54/T55-1)*100,"")</f>
+        <f>IF(COUNT(T54:T55)=2,ROUND((T54/T55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW54" s="6">
-        <f>IF(COUNT(Y54:Y55)=2,(Y54/Y55-1)*100,"")</f>
+        <f>IF(COUNT(Y54:Y55)=2,ROUND((Y54/Y55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX54" s="6">
-        <f>IF(COUNT(AD54:AD55)=2,(AD54/AD55-1)*100,"")</f>
+        <f>IF(COUNT(AD54:AD55)=2,ROUND((AD54/AD55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY54" s="6">
-        <f>IF(COUNT(AI54:AI55)=2,(AI54/AI55-1)*100,"")</f>
+        <f>IF(COUNT(AI54:AI55)=2,ROUND((AI54/AI55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ54" s="6">
-        <f>IF(COUNT(AN54:AN55)=2,(AN54/AN55-1)*100,"")</f>
+        <f>IF(COUNT(AN54:AN55)=2,ROUND((AN54/AN55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA54" s="6">
-        <f>IF(COUNT(AS54:AS55)=2,(AS54/AS55-1)*100,"")</f>
+        <f>IF(COUNT(AS54:AS55)=2,ROUND((AS54/AS55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB54" s="5" t="n">
         <v>18.92</v>
       </c>
       <c r="BC54" s="6">
-        <f>IF(COUNT(BB54:BB55)=2,(BB54/BB55-1)*100,"")</f>
+        <f>IF(COUNT(BB54:BB55)=2,ROUND((BB54/BB55-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD54" s="6" t="n">
@@ -12009,11 +12009,11 @@
         <v>178.71</v>
       </c>
       <c r="D55" s="6">
-        <f>IF(COUNT(B55:B56)=2,(B55/B56-1)*100,"")</f>
+        <f>IF(COUNT(B55:B56)=2,ROUND((B55/B56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E55" s="6">
-        <f>IF(COUNT(C55:C56)=2,(C55/C56-1)*100,"")</f>
+        <f>IF(COUNT(C55:C56)=2,ROUND((C55/C56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F55" s="5" t="n">
@@ -12137,42 +12137,42 @@
         <v>111.3802</v>
       </c>
       <c r="AT55" s="6">
-        <f>IF(COUNT(J55:J56)=2,(J55/J56-1)*100,"")</f>
+        <f>IF(COUNT(J55:J56)=2,ROUND((J55/J56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU55" s="6">
-        <f>IF(COUNT(O55:O56)=2,(O55/O56-1)*100,"")</f>
+        <f>IF(COUNT(O55:O56)=2,ROUND((O55/O56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV55" s="6">
-        <f>IF(COUNT(T55:T56)=2,(T55/T56-1)*100,"")</f>
+        <f>IF(COUNT(T55:T56)=2,ROUND((T55/T56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW55" s="6">
-        <f>IF(COUNT(Y55:Y56)=2,(Y55/Y56-1)*100,"")</f>
+        <f>IF(COUNT(Y55:Y56)=2,ROUND((Y55/Y56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX55" s="6">
-        <f>IF(COUNT(AD55:AD56)=2,(AD55/AD56-1)*100,"")</f>
+        <f>IF(COUNT(AD55:AD56)=2,ROUND((AD55/AD56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY55" s="6">
-        <f>IF(COUNT(AI55:AI56)=2,(AI55/AI56-1)*100,"")</f>
+        <f>IF(COUNT(AI55:AI56)=2,ROUND((AI55/AI56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ55" s="6">
-        <f>IF(COUNT(AN55:AN56)=2,(AN55/AN56-1)*100,"")</f>
+        <f>IF(COUNT(AN55:AN56)=2,ROUND((AN55/AN56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA55" s="6">
-        <f>IF(COUNT(AS55:AS56)=2,(AS55/AS56-1)*100,"")</f>
+        <f>IF(COUNT(AS55:AS56)=2,ROUND((AS55/AS56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB55" s="5" t="n">
         <v>21.51</v>
       </c>
       <c r="BC55" s="6">
-        <f>IF(COUNT(BB55:BB56)=2,(BB55/BB56-1)*100,"")</f>
+        <f>IF(COUNT(BB55:BB56)=2,ROUND((BB55/BB56-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD55" s="6" t="n">
@@ -12224,11 +12224,11 @@
         <v>188.65</v>
       </c>
       <c r="D56" s="6">
-        <f>IF(COUNT(B56:B57)=2,(B56/B57-1)*100,"")</f>
+        <f>IF(COUNT(B56:B57)=2,ROUND((B56/B57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E56" s="6">
-        <f>IF(COUNT(C56:C57)=2,(C56/C57-1)*100,"")</f>
+        <f>IF(COUNT(C56:C57)=2,ROUND((C56/C57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F56" s="5" t="n">
@@ -12352,42 +12352,42 @@
         <v>112.8165</v>
       </c>
       <c r="AT56" s="6">
-        <f>IF(COUNT(J56:J57)=2,(J56/J57-1)*100,"")</f>
+        <f>IF(COUNT(J56:J57)=2,ROUND((J56/J57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU56" s="6">
-        <f>IF(COUNT(O56:O57)=2,(O56/O57-1)*100,"")</f>
+        <f>IF(COUNT(O56:O57)=2,ROUND((O56/O57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV56" s="6">
-        <f>IF(COUNT(T56:T57)=2,(T56/T57-1)*100,"")</f>
+        <f>IF(COUNT(T56:T57)=2,ROUND((T56/T57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW56" s="6">
-        <f>IF(COUNT(Y56:Y57)=2,(Y56/Y57-1)*100,"")</f>
+        <f>IF(COUNT(Y56:Y57)=2,ROUND((Y56/Y57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX56" s="6">
-        <f>IF(COUNT(AD56:AD57)=2,(AD56/AD57-1)*100,"")</f>
+        <f>IF(COUNT(AD56:AD57)=2,ROUND((AD56/AD57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY56" s="6">
-        <f>IF(COUNT(AI56:AI57)=2,(AI56/AI57-1)*100,"")</f>
+        <f>IF(COUNT(AI56:AI57)=2,ROUND((AI56/AI57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ56" s="6">
-        <f>IF(COUNT(AN56:AN57)=2,(AN56/AN57-1)*100,"")</f>
+        <f>IF(COUNT(AN56:AN57)=2,ROUND((AN56/AN57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA56" s="6">
-        <f>IF(COUNT(AS56:AS57)=2,(AS56/AS57-1)*100,"")</f>
+        <f>IF(COUNT(AS56:AS57)=2,ROUND((AS56/AS57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB56" s="5" t="n">
         <v>15.4</v>
       </c>
       <c r="BC56" s="6">
-        <f>IF(COUNT(BB56:BB57)=2,(BB56/BB57-1)*100,"")</f>
+        <f>IF(COUNT(BB56:BB57)=2,ROUND((BB56/BB57-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD56" s="6" t="n">
@@ -12439,11 +12439,11 @@
         <v>187.13</v>
       </c>
       <c r="D57" s="6">
-        <f>IF(COUNT(B57:B58)=2,(B57/B58-1)*100,"")</f>
+        <f>IF(COUNT(B57:B58)=2,ROUND((B57/B58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E57" s="6">
-        <f>IF(COUNT(C57:C58)=2,(C57/C58-1)*100,"")</f>
+        <f>IF(COUNT(C57:C58)=2,ROUND((C57/C58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F57" s="5" t="n">
@@ -12567,42 +12567,42 @@
         <v>111.7892</v>
       </c>
       <c r="AT57" s="6">
-        <f>IF(COUNT(J57:J58)=2,(J57/J58-1)*100,"")</f>
+        <f>IF(COUNT(J57:J58)=2,ROUND((J57/J58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU57" s="6">
-        <f>IF(COUNT(O57:O58)=2,(O57/O58-1)*100,"")</f>
+        <f>IF(COUNT(O57:O58)=2,ROUND((O57/O58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV57" s="6">
-        <f>IF(COUNT(T57:T58)=2,(T57/T58-1)*100,"")</f>
+        <f>IF(COUNT(T57:T58)=2,ROUND((T57/T58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW57" s="6">
-        <f>IF(COUNT(Y57:Y58)=2,(Y57/Y58-1)*100,"")</f>
+        <f>IF(COUNT(Y57:Y58)=2,ROUND((Y57/Y58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX57" s="6">
-        <f>IF(COUNT(AD57:AD58)=2,(AD57/AD58-1)*100,"")</f>
+        <f>IF(COUNT(AD57:AD58)=2,ROUND((AD57/AD58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY57" s="6">
-        <f>IF(COUNT(AI57:AI58)=2,(AI57/AI58-1)*100,"")</f>
+        <f>IF(COUNT(AI57:AI58)=2,ROUND((AI57/AI58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ57" s="6">
-        <f>IF(COUNT(AN57:AN58)=2,(AN57/AN58-1)*100,"")</f>
+        <f>IF(COUNT(AN57:AN58)=2,ROUND((AN57/AN58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA57" s="6">
-        <f>IF(COUNT(AS57:AS58)=2,(AS57/AS58-1)*100,"")</f>
+        <f>IF(COUNT(AS57:AS58)=2,ROUND((AS57/AS58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB57" s="5" t="n">
         <v>16.06</v>
       </c>
       <c r="BC57" s="6">
-        <f>IF(COUNT(BB57:BB58)=2,(BB57/BB58-1)*100,"")</f>
+        <f>IF(COUNT(BB57:BB58)=2,ROUND((BB57/BB58-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD57" s="6" t="n">
@@ -12654,11 +12654,11 @@
         <v>189.9</v>
       </c>
       <c r="D58" s="6">
-        <f>IF(COUNT(B58:B59)=2,(B58/B59-1)*100,"")</f>
+        <f>IF(COUNT(B58:B59)=2,ROUND((B58/B59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E58" s="6">
-        <f>IF(COUNT(C58:C59)=2,(C58/C59-1)*100,"")</f>
+        <f>IF(COUNT(C58:C59)=2,ROUND((C58/C59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F58" s="5" t="n">
@@ -12782,42 +12782,42 @@
         <v>113.2753</v>
       </c>
       <c r="AT58" s="6">
-        <f>IF(COUNT(J58:J59)=2,(J58/J59-1)*100,"")</f>
+        <f>IF(COUNT(J58:J59)=2,ROUND((J58/J59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU58" s="6">
-        <f>IF(COUNT(O58:O59)=2,(O58/O59-1)*100,"")</f>
+        <f>IF(COUNT(O58:O59)=2,ROUND((O58/O59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV58" s="6">
-        <f>IF(COUNT(T58:T59)=2,(T58/T59-1)*100,"")</f>
+        <f>IF(COUNT(T58:T59)=2,ROUND((T58/T59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW58" s="6">
-        <f>IF(COUNT(Y58:Y59)=2,(Y58/Y59-1)*100,"")</f>
+        <f>IF(COUNT(Y58:Y59)=2,ROUND((Y58/Y59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX58" s="6">
-        <f>IF(COUNT(AD58:AD59)=2,(AD58/AD59-1)*100,"")</f>
+        <f>IF(COUNT(AD58:AD59)=2,ROUND((AD58/AD59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY58" s="6">
-        <f>IF(COUNT(AI58:AI59)=2,(AI58/AI59-1)*100,"")</f>
+        <f>IF(COUNT(AI58:AI59)=2,ROUND((AI58/AI59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ58" s="6">
-        <f>IF(COUNT(AN58:AN59)=2,(AN58/AN59-1)*100,"")</f>
+        <f>IF(COUNT(AN58:AN59)=2,ROUND((AN58/AN59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA58" s="6">
-        <f>IF(COUNT(AS58:AS59)=2,(AS58/AS59-1)*100,"")</f>
+        <f>IF(COUNT(AS58:AS59)=2,ROUND((AS58/AS59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB58" s="5" t="n">
         <v>15.77</v>
       </c>
       <c r="BC58" s="6">
-        <f>IF(COUNT(BB58:BB59)=2,(BB58/BB59-1)*100,"")</f>
+        <f>IF(COUNT(BB58:BB59)=2,ROUND((BB58/BB59-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD58" s="6" t="n">
@@ -12869,11 +12869,11 @@
         <v>189.42</v>
       </c>
       <c r="D59" s="6">
-        <f>IF(COUNT(B59:B60)=2,(B59/B60-1)*100,"")</f>
+        <f>IF(COUNT(B59:B60)=2,ROUND((B59/B60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E59" s="6">
-        <f>IF(COUNT(C59:C60)=2,(C59/C60-1)*100,"")</f>
+        <f>IF(COUNT(C59:C60)=2,ROUND((C59/C60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F59" s="5" t="n">
@@ -12997,42 +12997,42 @@
         <v>115.31</v>
       </c>
       <c r="AT59" s="6">
-        <f>IF(COUNT(J59:J60)=2,(J59/J60-1)*100,"")</f>
+        <f>IF(COUNT(J59:J60)=2,ROUND((J59/J60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU59" s="6">
-        <f>IF(COUNT(O59:O60)=2,(O59/O60-1)*100,"")</f>
+        <f>IF(COUNT(O59:O60)=2,ROUND((O59/O60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV59" s="6">
-        <f>IF(COUNT(T59:T60)=2,(T59/T60-1)*100,"")</f>
+        <f>IF(COUNT(T59:T60)=2,ROUND((T59/T60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW59" s="6">
-        <f>IF(COUNT(Y59:Y60)=2,(Y59/Y60-1)*100,"")</f>
+        <f>IF(COUNT(Y59:Y60)=2,ROUND((Y59/Y60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX59" s="6">
-        <f>IF(COUNT(AD59:AD60)=2,(AD59/AD60-1)*100,"")</f>
+        <f>IF(COUNT(AD59:AD60)=2,ROUND((AD59/AD60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY59" s="6">
-        <f>IF(COUNT(AI59:AI60)=2,(AI59/AI60-1)*100,"")</f>
+        <f>IF(COUNT(AI59:AI60)=2,ROUND((AI59/AI60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ59" s="6">
-        <f>IF(COUNT(AN59:AN60)=2,(AN59/AN60-1)*100,"")</f>
+        <f>IF(COUNT(AN59:AN60)=2,ROUND((AN59/AN60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA59" s="6">
-        <f>IF(COUNT(AS59:AS60)=2,(AS59/AS60-1)*100,"")</f>
+        <f>IF(COUNT(AS59:AS60)=2,ROUND((AS59/AS60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB59" s="5" t="n">
         <v>16.05</v>
       </c>
       <c r="BC59" s="6">
-        <f>IF(COUNT(BB59:BB60)=2,(BB59/BB60-1)*100,"")</f>
+        <f>IF(COUNT(BB59:BB60)=2,ROUND((BB59/BB60-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD59" s="6" t="n">
@@ -13084,11 +13084,11 @@
         <v>188.5</v>
       </c>
       <c r="D60" s="6">
-        <f>IF(COUNT(B60:B61)=2,(B60/B61-1)*100,"")</f>
+        <f>IF(COUNT(B60:B61)=2,ROUND((B60/B61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E60" s="6">
-        <f>IF(COUNT(C60:C61)=2,(C60/C61-1)*100,"")</f>
+        <f>IF(COUNT(C60:C61)=2,ROUND((C60/C61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F60" s="5" t="n">
@@ -13212,42 +13212,42 @@
         <v>115.3898</v>
       </c>
       <c r="AT60" s="6">
-        <f>IF(COUNT(J60:J61)=2,(J60/J61-1)*100,"")</f>
+        <f>IF(COUNT(J60:J61)=2,ROUND((J60/J61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU60" s="6">
-        <f>IF(COUNT(O60:O61)=2,(O60/O61-1)*100,"")</f>
+        <f>IF(COUNT(O60:O61)=2,ROUND((O60/O61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV60" s="6">
-        <f>IF(COUNT(T60:T61)=2,(T60/T61-1)*100,"")</f>
+        <f>IF(COUNT(T60:T61)=2,ROUND((T60/T61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW60" s="6">
-        <f>IF(COUNT(Y60:Y61)=2,(Y60/Y61-1)*100,"")</f>
+        <f>IF(COUNT(Y60:Y61)=2,ROUND((Y60/Y61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX60" s="6">
-        <f>IF(COUNT(AD60:AD61)=2,(AD60/AD61-1)*100,"")</f>
+        <f>IF(COUNT(AD60:AD61)=2,ROUND((AD60/AD61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY60" s="6">
-        <f>IF(COUNT(AI60:AI61)=2,(AI60/AI61-1)*100,"")</f>
+        <f>IF(COUNT(AI60:AI61)=2,ROUND((AI60/AI61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ60" s="6">
-        <f>IF(COUNT(AN60:AN61)=2,(AN60/AN61-1)*100,"")</f>
+        <f>IF(COUNT(AN60:AN61)=2,ROUND((AN60/AN61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA60" s="6">
-        <f>IF(COUNT(AS60:AS61)=2,(AS60/AS61-1)*100,"")</f>
+        <f>IF(COUNT(AS60:AS61)=2,ROUND((AS60/AS61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB60" s="5" t="n">
         <v>15.32</v>
       </c>
       <c r="BC60" s="6">
-        <f>IF(COUNT(BB60:BB61)=2,(BB60/BB61-1)*100,"")</f>
+        <f>IF(COUNT(BB60:BB61)=2,ROUND((BB60/BB61-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD60" s="6" t="n">
@@ -13299,11 +13299,11 @@
         <v>187.68</v>
       </c>
       <c r="D61" s="6">
-        <f>IF(COUNT(B61:B62)=2,(B61/B62-1)*100,"")</f>
+        <f>IF(COUNT(B61:B62)=2,ROUND((B61/B62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E61" s="6">
-        <f>IF(COUNT(C61:C62)=2,(C61/C62-1)*100,"")</f>
+        <f>IF(COUNT(C61:C62)=2,ROUND((C61/C62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F61" s="5" t="n">
@@ -13427,42 +13427,42 @@
         <v>116.3673</v>
       </c>
       <c r="AT61" s="6">
-        <f>IF(COUNT(J61:J62)=2,(J61/J62-1)*100,"")</f>
+        <f>IF(COUNT(J61:J62)=2,ROUND((J61/J62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU61" s="6">
-        <f>IF(COUNT(O61:O62)=2,(O61/O62-1)*100,"")</f>
+        <f>IF(COUNT(O61:O62)=2,ROUND((O61/O62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV61" s="6">
-        <f>IF(COUNT(T61:T62)=2,(T61/T62-1)*100,"")</f>
+        <f>IF(COUNT(T61:T62)=2,ROUND((T61/T62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW61" s="6">
-        <f>IF(COUNT(Y61:Y62)=2,(Y61/Y62-1)*100,"")</f>
+        <f>IF(COUNT(Y61:Y62)=2,ROUND((Y61/Y62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX61" s="6">
-        <f>IF(COUNT(AD61:AD62)=2,(AD61/AD62-1)*100,"")</f>
+        <f>IF(COUNT(AD61:AD62)=2,ROUND((AD61/AD62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY61" s="6">
-        <f>IF(COUNT(AI61:AI62)=2,(AI61/AI62-1)*100,"")</f>
+        <f>IF(COUNT(AI61:AI62)=2,ROUND((AI61/AI62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ61" s="6">
-        <f>IF(COUNT(AN61:AN62)=2,(AN61/AN62-1)*100,"")</f>
+        <f>IF(COUNT(AN61:AN62)=2,ROUND((AN61/AN62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA61" s="6">
-        <f>IF(COUNT(AS61:AS62)=2,(AS61/AS62-1)*100,"")</f>
+        <f>IF(COUNT(AS61:AS62)=2,ROUND((AS61/AS62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB61" s="5" t="n">
         <v>15.74</v>
       </c>
       <c r="BC61" s="6">
-        <f>IF(COUNT(BB61:BB62)=2,(BB61/BB62-1)*100,"")</f>
+        <f>IF(COUNT(BB61:BB62)=2,ROUND((BB61/BB62-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD61" s="6" t="n">
@@ -13514,11 +13514,11 @@
         <v>185.59</v>
       </c>
       <c r="D62" s="6">
-        <f>IF(COUNT(B62:B63)=2,(B62/B63-1)*100,"")</f>
+        <f>IF(COUNT(B62:B63)=2,ROUND((B62/B63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E62" s="6">
-        <f>IF(COUNT(C62:C63)=2,(C62/C63-1)*100,"")</f>
+        <f>IF(COUNT(C62:C63)=2,ROUND((C62/C63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F62" s="5" t="n">
@@ -13642,42 +13642,42 @@
         <v>115.9583</v>
       </c>
       <c r="AT62" s="6">
-        <f>IF(COUNT(J62:J63)=2,(J62/J63-1)*100,"")</f>
+        <f>IF(COUNT(J62:J63)=2,ROUND((J62/J63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU62" s="6">
-        <f>IF(COUNT(O62:O63)=2,(O62/O63-1)*100,"")</f>
+        <f>IF(COUNT(O62:O63)=2,ROUND((O62/O63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV62" s="6">
-        <f>IF(COUNT(T62:T63)=2,(T62/T63-1)*100,"")</f>
+        <f>IF(COUNT(T62:T63)=2,ROUND((T62/T63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW62" s="6">
-        <f>IF(COUNT(Y62:Y63)=2,(Y62/Y63-1)*100,"")</f>
+        <f>IF(COUNT(Y62:Y63)=2,ROUND((Y62/Y63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX62" s="6">
-        <f>IF(COUNT(AD62:AD63)=2,(AD62/AD63-1)*100,"")</f>
+        <f>IF(COUNT(AD62:AD63)=2,ROUND((AD62/AD63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY62" s="6">
-        <f>IF(COUNT(AI62:AI63)=2,(AI62/AI63-1)*100,"")</f>
+        <f>IF(COUNT(AI62:AI63)=2,ROUND((AI62/AI63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ62" s="6">
-        <f>IF(COUNT(AN62:AN63)=2,(AN62/AN63-1)*100,"")</f>
+        <f>IF(COUNT(AN62:AN63)=2,ROUND((AN62/AN63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA62" s="6">
-        <f>IF(COUNT(AS62:AS63)=2,(AS62/AS63-1)*100,"")</f>
+        <f>IF(COUNT(AS62:AS63)=2,ROUND((AS62/AS63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB62" s="5" t="n">
         <v>16.29</v>
       </c>
       <c r="BC62" s="6">
-        <f>IF(COUNT(BB62:BB63)=2,(BB62/BB63-1)*100,"")</f>
+        <f>IF(COUNT(BB62:BB63)=2,ROUND((BB62/BB63-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD62" s="6" t="n">
@@ -13729,11 +13729,11 @@
         <v>185.57</v>
       </c>
       <c r="D63" s="6">
-        <f>IF(COUNT(B63:B64)=2,(B63/B64-1)*100,"")</f>
+        <f>IF(COUNT(B63:B64)=2,ROUND((B63/B64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E63" s="6">
-        <f>IF(COUNT(C63:C64)=2,(C63/C64-1)*100,"")</f>
+        <f>IF(COUNT(C63:C64)=2,ROUND((C63/C64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F63" s="5" t="n">
@@ -13857,42 +13857,42 @@
         <v>115.2502</v>
       </c>
       <c r="AT63" s="6">
-        <f>IF(COUNT(J63:J64)=2,(J63/J64-1)*100,"")</f>
+        <f>IF(COUNT(J63:J64)=2,ROUND((J63/J64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU63" s="6">
-        <f>IF(COUNT(O63:O64)=2,(O63/O64-1)*100,"")</f>
+        <f>IF(COUNT(O63:O64)=2,ROUND((O63/O64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV63" s="6">
-        <f>IF(COUNT(T63:T64)=2,(T63/T64-1)*100,"")</f>
+        <f>IF(COUNT(T63:T64)=2,ROUND((T63/T64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW63" s="6">
-        <f>IF(COUNT(Y63:Y64)=2,(Y63/Y64-1)*100,"")</f>
+        <f>IF(COUNT(Y63:Y64)=2,ROUND((Y63/Y64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX63" s="6">
-        <f>IF(COUNT(AD63:AD64)=2,(AD63/AD64-1)*100,"")</f>
+        <f>IF(COUNT(AD63:AD64)=2,ROUND((AD63/AD64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY63" s="6">
-        <f>IF(COUNT(AI63:AI64)=2,(AI63/AI64-1)*100,"")</f>
+        <f>IF(COUNT(AI63:AI64)=2,ROUND((AI63/AI64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ63" s="6">
-        <f>IF(COUNT(AN63:AN64)=2,(AN63/AN64-1)*100,"")</f>
+        <f>IF(COUNT(AN63:AN64)=2,ROUND((AN63/AN64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA63" s="6">
-        <f>IF(COUNT(AS63:AS64)=2,(AS63/AS64-1)*100,"")</f>
+        <f>IF(COUNT(AS63:AS64)=2,ROUND((AS63/AS64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB63" s="5" t="n">
         <v>17.01</v>
       </c>
       <c r="BC63" s="6">
-        <f>IF(COUNT(BB63:BB64)=2,(BB63/BB64-1)*100,"")</f>
+        <f>IF(COUNT(BB63:BB64)=2,ROUND((BB63/BB64-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD63" s="6" t="n">
@@ -13944,11 +13944,11 @@
         <v>183.39</v>
       </c>
       <c r="D64" s="6">
-        <f>IF(COUNT(B64:B65)=2,(B64/B65-1)*100,"")</f>
+        <f>IF(COUNT(B64:B65)=2,ROUND((B64/B65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E64" s="6">
-        <f>IF(COUNT(C64:C65)=2,(C64/C65-1)*100,"")</f>
+        <f>IF(COUNT(C64:C65)=2,ROUND((C64/C65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F64" s="5" t="n">
@@ -14072,42 +14072,42 @@
         <v>115.1604</v>
       </c>
       <c r="AT64" s="6">
-        <f>IF(COUNT(J64:J65)=2,(J64/J65-1)*100,"")</f>
+        <f>IF(COUNT(J64:J65)=2,ROUND((J64/J65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU64" s="6">
-        <f>IF(COUNT(O64:O65)=2,(O64/O65-1)*100,"")</f>
+        <f>IF(COUNT(O64:O65)=2,ROUND((O64/O65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV64" s="6">
-        <f>IF(COUNT(T64:T65)=2,(T64/T65-1)*100,"")</f>
+        <f>IF(COUNT(T64:T65)=2,ROUND((T64/T65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW64" s="6">
-        <f>IF(COUNT(Y64:Y65)=2,(Y64/Y65-1)*100,"")</f>
+        <f>IF(COUNT(Y64:Y65)=2,ROUND((Y64/Y65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX64" s="6">
-        <f>IF(COUNT(AD64:AD65)=2,(AD64/AD65-1)*100,"")</f>
+        <f>IF(COUNT(AD64:AD65)=2,ROUND((AD64/AD65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY64" s="6">
-        <f>IF(COUNT(AI64:AI65)=2,(AI64/AI65-1)*100,"")</f>
+        <f>IF(COUNT(AI64:AI65)=2,ROUND((AI64/AI65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ64" s="6">
-        <f>IF(COUNT(AN64:AN65)=2,(AN64/AN65-1)*100,"")</f>
+        <f>IF(COUNT(AN64:AN65)=2,ROUND((AN64/AN65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA64" s="6">
-        <f>IF(COUNT(AS64:AS65)=2,(AS64/AS65-1)*100,"")</f>
+        <f>IF(COUNT(AS64:AS65)=2,ROUND((AS64/AS65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB64" s="5" t="n">
         <v>16.7</v>
       </c>
       <c r="BC64" s="6">
-        <f>IF(COUNT(BB64:BB65)=2,(BB64/BB65-1)*100,"")</f>
+        <f>IF(COUNT(BB64:BB65)=2,ROUND((BB64/BB65-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD64" s="6" t="n">
@@ -14159,11 +14159,11 @@
         <v>182.04</v>
       </c>
       <c r="D65" s="6">
-        <f>IF(COUNT(B65:B66)=2,(B65/B66-1)*100,"")</f>
+        <f>IF(COUNT(B65:B66)=2,ROUND((B65/B66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E65" s="6">
-        <f>IF(COUNT(C65:C66)=2,(C65/C66-1)*100,"")</f>
+        <f>IF(COUNT(C65:C66)=2,ROUND((C65/C66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F65" s="5" t="n">
@@ -14287,42 +14287,42 @@
         <v>115.7987</v>
       </c>
       <c r="AT65" s="6">
-        <f>IF(COUNT(J65:J66)=2,(J65/J66-1)*100,"")</f>
+        <f>IF(COUNT(J65:J66)=2,ROUND((J65/J66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU65" s="6">
-        <f>IF(COUNT(O65:O66)=2,(O65/O66-1)*100,"")</f>
+        <f>IF(COUNT(O65:O66)=2,ROUND((O65/O66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV65" s="6">
-        <f>IF(COUNT(T65:T66)=2,(T65/T66-1)*100,"")</f>
+        <f>IF(COUNT(T65:T66)=2,ROUND((T65/T66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW65" s="6">
-        <f>IF(COUNT(Y65:Y66)=2,(Y65/Y66-1)*100,"")</f>
+        <f>IF(COUNT(Y65:Y66)=2,ROUND((Y65/Y66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX65" s="6">
-        <f>IF(COUNT(AD65:AD66)=2,(AD65/AD66-1)*100,"")</f>
+        <f>IF(COUNT(AD65:AD66)=2,ROUND((AD65/AD66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY65" s="6">
-        <f>IF(COUNT(AI65:AI66)=2,(AI65/AI66-1)*100,"")</f>
+        <f>IF(COUNT(AI65:AI66)=2,ROUND((AI65/AI66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ65" s="6">
-        <f>IF(COUNT(AN65:AN66)=2,(AN65/AN66-1)*100,"")</f>
+        <f>IF(COUNT(AN65:AN66)=2,ROUND((AN65/AN66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA65" s="6">
-        <f>IF(COUNT(AS65:AS66)=2,(AS65/AS66-1)*100,"")</f>
+        <f>IF(COUNT(AS65:AS66)=2,ROUND((AS65/AS66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB65" s="5" t="n">
         <v>16.76</v>
       </c>
       <c r="BC65" s="6">
-        <f>IF(COUNT(BB65:BB66)=2,(BB65/BB66-1)*100,"")</f>
+        <f>IF(COUNT(BB65:BB66)=2,ROUND((BB65/BB66-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD65" s="6" t="n">
@@ -14374,11 +14374,11 @@
         <v>181.4</v>
       </c>
       <c r="D66" s="6">
-        <f>IF(COUNT(B66:B67)=2,(B66/B67-1)*100,"")</f>
+        <f>IF(COUNT(B66:B67)=2,ROUND((B66/B67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E66" s="6">
-        <f>IF(COUNT(C66:C67)=2,(C66/C67-1)*100,"")</f>
+        <f>IF(COUNT(C66:C67)=2,ROUND((C66/C67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F66" s="5" t="n">
@@ -14502,42 +14502,42 @@
         <v>115.7987</v>
       </c>
       <c r="AT66" s="6">
-        <f>IF(COUNT(J66:J67)=2,(J66/J67-1)*100,"")</f>
+        <f>IF(COUNT(J66:J67)=2,ROUND((J66/J67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU66" s="6">
-        <f>IF(COUNT(O66:O67)=2,(O66/O67-1)*100,"")</f>
+        <f>IF(COUNT(O66:O67)=2,ROUND((O66/O67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV66" s="6">
-        <f>IF(COUNT(T66:T67)=2,(T66/T67-1)*100,"")</f>
+        <f>IF(COUNT(T66:T67)=2,ROUND((T66/T67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW66" s="6">
-        <f>IF(COUNT(Y66:Y67)=2,(Y66/Y67-1)*100,"")</f>
+        <f>IF(COUNT(Y66:Y67)=2,ROUND((Y66/Y67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX66" s="6">
-        <f>IF(COUNT(AD66:AD67)=2,(AD66/AD67-1)*100,"")</f>
+        <f>IF(COUNT(AD66:AD67)=2,ROUND((AD66/AD67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY66" s="6">
-        <f>IF(COUNT(AI66:AI67)=2,(AI66/AI67-1)*100,"")</f>
+        <f>IF(COUNT(AI66:AI67)=2,ROUND((AI66/AI67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ66" s="6">
-        <f>IF(COUNT(AN66:AN67)=2,(AN66/AN67-1)*100,"")</f>
+        <f>IF(COUNT(AN66:AN67)=2,ROUND((AN66/AN67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA66" s="6">
-        <f>IF(COUNT(AS66:AS67)=2,(AS66/AS67-1)*100,"")</f>
+        <f>IF(COUNT(AS66:AS67)=2,ROUND((AS66/AS67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB66" s="5" t="n">
         <v>17.44</v>
       </c>
       <c r="BC66" s="6">
-        <f>IF(COUNT(BB66:BB67)=2,(BB66/BB67-1)*100,"")</f>
+        <f>IF(COUNT(BB66:BB67)=2,ROUND((BB66/BB67-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD66" s="6" t="n">
@@ -14589,11 +14589,11 @@
         <v>177.64</v>
       </c>
       <c r="D67" s="6">
-        <f>IF(COUNT(B67:B68)=2,(B67/B68-1)*100,"")</f>
+        <f>IF(COUNT(B67:B68)=2,ROUND((B67/B68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E67" s="6">
-        <f>IF(COUNT(C67:C68)=2,(C67/C68-1)*100,"")</f>
+        <f>IF(COUNT(C67:C68)=2,ROUND((C67/C68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F67" s="5" t="n">
@@ -14717,42 +14717,42 @@
         <v>115.5494</v>
       </c>
       <c r="AT67" s="6">
-        <f>IF(COUNT(J67:J68)=2,(J67/J68-1)*100,"")</f>
+        <f>IF(COUNT(J67:J68)=2,ROUND((J67/J68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU67" s="6">
-        <f>IF(COUNT(O67:O68)=2,(O67/O68-1)*100,"")</f>
+        <f>IF(COUNT(O67:O68)=2,ROUND((O67/O68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV67" s="6">
-        <f>IF(COUNT(T67:T68)=2,(T67/T68-1)*100,"")</f>
+        <f>IF(COUNT(T67:T68)=2,ROUND((T67/T68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW67" s="6">
-        <f>IF(COUNT(Y67:Y68)=2,(Y67/Y68-1)*100,"")</f>
+        <f>IF(COUNT(Y67:Y68)=2,ROUND((Y67/Y68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX67" s="6">
-        <f>IF(COUNT(AD67:AD68)=2,(AD67/AD68-1)*100,"")</f>
+        <f>IF(COUNT(AD67:AD68)=2,ROUND((AD67/AD68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY67" s="6">
-        <f>IF(COUNT(AI67:AI68)=2,(AI67/AI68-1)*100,"")</f>
+        <f>IF(COUNT(AI67:AI68)=2,ROUND((AI67/AI68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ67" s="6">
-        <f>IF(COUNT(AN67:AN68)=2,(AN67/AN68-1)*100,"")</f>
+        <f>IF(COUNT(AN67:AN68)=2,ROUND((AN67/AN68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA67" s="6">
-        <f>IF(COUNT(AS67:AS68)=2,(AS67/AS68-1)*100,"")</f>
+        <f>IF(COUNT(AS67:AS68)=2,ROUND((AS67/AS68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB67" s="5" t="n">
         <v>18.06</v>
       </c>
       <c r="BC67" s="6">
-        <f>IF(COUNT(BB67:BB68)=2,(BB67/BB68-1)*100,"")</f>
+        <f>IF(COUNT(BB67:BB68)=2,ROUND((BB67/BB68-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD67" s="6" t="n">
@@ -14804,11 +14804,11 @@
         <v>180.04</v>
       </c>
       <c r="D68" s="6">
-        <f>IF(COUNT(B68:B69)=2,(B68/B69-1)*100,"")</f>
+        <f>IF(COUNT(B68:B69)=2,ROUND((B68/B69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E68" s="6">
-        <f>IF(COUNT(C68:C69)=2,(C68/C69-1)*100,"")</f>
+        <f>IF(COUNT(C68:C69)=2,ROUND((C68/C69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F68" s="5" t="n">
@@ -14932,42 +14932,42 @@
         <v>116.6765</v>
       </c>
       <c r="AT68" s="6">
-        <f>IF(COUNT(J68:J69)=2,(J68/J69-1)*100,"")</f>
+        <f>IF(COUNT(J68:J69)=2,ROUND((J68/J69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU68" s="6">
-        <f>IF(COUNT(O68:O69)=2,(O68/O69-1)*100,"")</f>
+        <f>IF(COUNT(O68:O69)=2,ROUND((O68/O69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV68" s="6">
-        <f>IF(COUNT(T68:T69)=2,(T68/T69-1)*100,"")</f>
+        <f>IF(COUNT(T68:T69)=2,ROUND((T68/T69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW68" s="6">
-        <f>IF(COUNT(Y68:Y69)=2,(Y68/Y69-1)*100,"")</f>
+        <f>IF(COUNT(Y68:Y69)=2,ROUND((Y68/Y69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX68" s="6">
-        <f>IF(COUNT(AD68:AD69)=2,(AD68/AD69-1)*100,"")</f>
+        <f>IF(COUNT(AD68:AD69)=2,ROUND((AD68/AD69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY68" s="6">
-        <f>IF(COUNT(AI68:AI69)=2,(AI68/AI69-1)*100,"")</f>
+        <f>IF(COUNT(AI68:AI69)=2,ROUND((AI68/AI69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ68" s="6">
-        <f>IF(COUNT(AN68:AN69)=2,(AN68/AN69-1)*100,"")</f>
+        <f>IF(COUNT(AN68:AN69)=2,ROUND((AN68/AN69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA68" s="6">
-        <f>IF(COUNT(AS68:AS69)=2,(AS68/AS69-1)*100,"")</f>
+        <f>IF(COUNT(AS68:AS69)=2,ROUND((AS68/AS69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB68" s="5" t="n">
         <v>17.82</v>
       </c>
       <c r="BC68" s="6">
-        <f>IF(COUNT(BB68:BB69)=2,(BB68/BB69-1)*100,"")</f>
+        <f>IF(COUNT(BB68:BB69)=2,ROUND((BB68/BB69-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD68" s="6" t="n">
@@ -15019,11 +15019,11 @@
         <v>180.37</v>
       </c>
       <c r="D69" s="6">
-        <f>IF(COUNT(B69:B70)=2,(B69/B70-1)*100,"")</f>
+        <f>IF(COUNT(B69:B70)=2,ROUND((B69/B70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E69" s="6">
-        <f>IF(COUNT(C69:C70)=2,(C69/C70-1)*100,"")</f>
+        <f>IF(COUNT(C69:C70)=2,ROUND((C69/C70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F69" s="5" t="n">
@@ -15147,42 +15147,42 @@
         <v>115.7788</v>
       </c>
       <c r="AT69" s="6">
-        <f>IF(COUNT(J69:J70)=2,(J69/J70-1)*100,"")</f>
+        <f>IF(COUNT(J69:J70)=2,ROUND((J69/J70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU69" s="6">
-        <f>IF(COUNT(O69:O70)=2,(O69/O70-1)*100,"")</f>
+        <f>IF(COUNT(O69:O70)=2,ROUND((O69/O70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV69" s="6">
-        <f>IF(COUNT(T69:T70)=2,(T69/T70-1)*100,"")</f>
+        <f>IF(COUNT(T69:T70)=2,ROUND((T69/T70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW69" s="6">
-        <f>IF(COUNT(Y69:Y70)=2,(Y69/Y70-1)*100,"")</f>
+        <f>IF(COUNT(Y69:Y70)=2,ROUND((Y69/Y70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX69" s="6">
-        <f>IF(COUNT(AD69:AD70)=2,(AD69/AD70-1)*100,"")</f>
+        <f>IF(COUNT(AD69:AD70)=2,ROUND((AD69/AD70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY69" s="6">
-        <f>IF(COUNT(AI69:AI70)=2,(AI69/AI70-1)*100,"")</f>
+        <f>IF(COUNT(AI69:AI70)=2,ROUND((AI69/AI70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ69" s="6">
-        <f>IF(COUNT(AN69:AN70)=2,(AN69/AN70-1)*100,"")</f>
+        <f>IF(COUNT(AN69:AN70)=2,ROUND((AN69/AN70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA69" s="6">
-        <f>IF(COUNT(AS69:AS70)=2,(AS69/AS70-1)*100,"")</f>
+        <f>IF(COUNT(AS69:AS70)=2,ROUND((AS69/AS70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB69" s="5" t="n">
         <v>18.43</v>
       </c>
       <c r="BC69" s="6">
-        <f>IF(COUNT(BB69:BB70)=2,(BB69/BB70-1)*100,"")</f>
+        <f>IF(COUNT(BB69:BB70)=2,ROUND((BB69/BB70-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD69" s="6" t="n">
@@ -15234,11 +15234,11 @@
         <v>184.9</v>
       </c>
       <c r="D70" s="6">
-        <f>IF(COUNT(B70:B71)=2,(B70/B71-1)*100,"")</f>
+        <f>IF(COUNT(B70:B71)=2,ROUND((B70/B71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E70" s="6">
-        <f>IF(COUNT(C70:C71)=2,(C70/C71-1)*100,"")</f>
+        <f>IF(COUNT(C70:C71)=2,ROUND((C70/C71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F70" s="5" t="n">
@@ -15362,42 +15362,42 @@
         <v>116.8061</v>
       </c>
       <c r="AT70" s="6">
-        <f>IF(COUNT(J70:J71)=2,(J70/J71-1)*100,"")</f>
+        <f>IF(COUNT(J70:J71)=2,ROUND((J70/J71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU70" s="6">
-        <f>IF(COUNT(O70:O71)=2,(O70/O71-1)*100,"")</f>
+        <f>IF(COUNT(O70:O71)=2,ROUND((O70/O71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV70" s="6">
-        <f>IF(COUNT(T70:T71)=2,(T70/T71-1)*100,"")</f>
+        <f>IF(COUNT(T70:T71)=2,ROUND((T70/T71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW70" s="6">
-        <f>IF(COUNT(Y70:Y71)=2,(Y70/Y71-1)*100,"")</f>
+        <f>IF(COUNT(Y70:Y71)=2,ROUND((Y70/Y71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX70" s="6">
-        <f>IF(COUNT(AD70:AD71)=2,(AD70/AD71-1)*100,"")</f>
+        <f>IF(COUNT(AD70:AD71)=2,ROUND((AD70/AD71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY70" s="6">
-        <f>IF(COUNT(AI70:AI71)=2,(AI70/AI71-1)*100,"")</f>
+        <f>IF(COUNT(AI70:AI71)=2,ROUND((AI70/AI71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ70" s="6">
-        <f>IF(COUNT(AN70:AN71)=2,(AN70/AN71-1)*100,"")</f>
+        <f>IF(COUNT(AN70:AN71)=2,ROUND((AN70/AN71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA70" s="6">
-        <f>IF(COUNT(AS70:AS71)=2,(AS70/AS71-1)*100,"")</f>
+        <f>IF(COUNT(AS70:AS71)=2,ROUND((AS70/AS71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB70" s="5" t="n">
         <v>17.26</v>
       </c>
       <c r="BC70" s="6">
-        <f>IF(COUNT(BB70:BB71)=2,(BB70/BB71-1)*100,"")</f>
+        <f>IF(COUNT(BB70:BB71)=2,ROUND((BB70/BB71-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD70" s="6" t="n">
@@ -15449,11 +15449,11 @@
         <v>182.13</v>
       </c>
       <c r="D71" s="6">
-        <f>IF(COUNT(B71:B72)=2,(B71/B72-1)*100,"")</f>
+        <f>IF(COUNT(B71:B72)=2,ROUND((B71/B72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E71" s="6">
-        <f>IF(COUNT(C71:C72)=2,(C71/C72-1)*100,"")</f>
+        <f>IF(COUNT(C71:C72)=2,ROUND((C71/C72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F71" s="5" t="n">
@@ -15577,42 +15577,42 @@
         <v>116.457</v>
       </c>
       <c r="AT71" s="6">
-        <f>IF(COUNT(J71:J72)=2,(J71/J72-1)*100,"")</f>
+        <f>IF(COUNT(J71:J72)=2,ROUND((J71/J72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU71" s="6">
-        <f>IF(COUNT(O71:O72)=2,(O71/O72-1)*100,"")</f>
+        <f>IF(COUNT(O71:O72)=2,ROUND((O71/O72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV71" s="6">
-        <f>IF(COUNT(T71:T72)=2,(T71/T72-1)*100,"")</f>
+        <f>IF(COUNT(T71:T72)=2,ROUND((T71/T72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW71" s="6">
-        <f>IF(COUNT(Y71:Y72)=2,(Y71/Y72-1)*100,"")</f>
+        <f>IF(COUNT(Y71:Y72)=2,ROUND((Y71/Y72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX71" s="6">
-        <f>IF(COUNT(AD71:AD72)=2,(AD71/AD72-1)*100,"")</f>
+        <f>IF(COUNT(AD71:AD72)=2,ROUND((AD71/AD72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY71" s="6">
-        <f>IF(COUNT(AI71:AI72)=2,(AI71/AI72-1)*100,"")</f>
+        <f>IF(COUNT(AI71:AI72)=2,ROUND((AI71/AI72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ71" s="6">
-        <f>IF(COUNT(AN71:AN72)=2,(AN71/AN72-1)*100,"")</f>
+        <f>IF(COUNT(AN71:AN72)=2,ROUND((AN71/AN72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA71" s="6">
-        <f>IF(COUNT(AS71:AS72)=2,(AS71/AS72-1)*100,"")</f>
+        <f>IF(COUNT(AS71:AS72)=2,ROUND((AS71/AS72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB71" s="5" t="n">
         <v>17.87</v>
       </c>
       <c r="BC71" s="6">
-        <f>IF(COUNT(BB71:BB72)=2,(BB71/BB72-1)*100,"")</f>
+        <f>IF(COUNT(BB71:BB72)=2,ROUND((BB71/BB72-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD71" s="6" t="n">
@@ -15664,11 +15664,11 @@
         <v>180.05</v>
       </c>
       <c r="D72" s="6">
-        <f>IF(COUNT(B72:B73)=2,(B72/B73-1)*100,"")</f>
+        <f>IF(COUNT(B72:B73)=2,ROUND((B72/B73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E72" s="6">
-        <f>IF(COUNT(C72:C73)=2,(C72/C73-1)*100,"")</f>
+        <f>IF(COUNT(C72:C73)=2,ROUND((C72/C73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F72" s="5" t="n">
@@ -15792,42 +15792,42 @@
         <v>115.5594</v>
       </c>
       <c r="AT72" s="6">
-        <f>IF(COUNT(J72:J73)=2,(J72/J73-1)*100,"")</f>
+        <f>IF(COUNT(J72:J73)=2,ROUND((J72/J73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU72" s="6">
-        <f>IF(COUNT(O72:O73)=2,(O72/O73-1)*100,"")</f>
+        <f>IF(COUNT(O72:O73)=2,ROUND((O72/O73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV72" s="6">
-        <f>IF(COUNT(T72:T73)=2,(T72/T73-1)*100,"")</f>
+        <f>IF(COUNT(T72:T73)=2,ROUND((T72/T73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW72" s="6">
-        <f>IF(COUNT(Y72:Y73)=2,(Y72/Y73-1)*100,"")</f>
+        <f>IF(COUNT(Y72:Y73)=2,ROUND((Y72/Y73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX72" s="6">
-        <f>IF(COUNT(AD72:AD73)=2,(AD72/AD73-1)*100,"")</f>
+        <f>IF(COUNT(AD72:AD73)=2,ROUND((AD72/AD73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY72" s="6">
-        <f>IF(COUNT(AI72:AI73)=2,(AI72/AI73-1)*100,"")</f>
+        <f>IF(COUNT(AI72:AI73)=2,ROUND((AI72/AI73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ72" s="6">
-        <f>IF(COUNT(AN72:AN73)=2,(AN72/AN73-1)*100,"")</f>
+        <f>IF(COUNT(AN72:AN73)=2,ROUND((AN72/AN73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA72" s="6">
-        <f>IF(COUNT(AS72:AS73)=2,(AS72/AS73-1)*100,"")</f>
+        <f>IF(COUNT(AS72:AS73)=2,ROUND((AS72/AS73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB72" s="5" t="n">
         <v>17.99</v>
       </c>
       <c r="BC72" s="6">
-        <f>IF(COUNT(BB72:BB73)=2,(BB72/BB73-1)*100,"")</f>
+        <f>IF(COUNT(BB72:BB73)=2,ROUND((BB72/BB73-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD72" s="6" t="n">
@@ -15879,11 +15879,11 @@
         <v>180.64</v>
       </c>
       <c r="D73" s="6">
-        <f>IF(COUNT(B73:B74)=2,(B73/B74-1)*100,"")</f>
+        <f>IF(COUNT(B73:B74)=2,ROUND((B73/B74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="E73" s="6">
-        <f>IF(COUNT(C73:C74)=2,(C73/C74-1)*100,"")</f>
+        <f>IF(COUNT(C73:C74)=2,ROUND((C73/C74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="F73" s="5" t="n">
@@ -16007,42 +16007,42 @@
         <v>115.2801</v>
       </c>
       <c r="AT73" s="6">
-        <f>IF(COUNT(J73:J74)=2,(J73/J74-1)*100,"")</f>
+        <f>IF(COUNT(J73:J74)=2,ROUND((J73/J74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AU73" s="6">
-        <f>IF(COUNT(O73:O74)=2,(O73/O74-1)*100,"")</f>
+        <f>IF(COUNT(O73:O74)=2,ROUND((O73/O74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AV73" s="6">
-        <f>IF(COUNT(T73:T74)=2,(T73/T74-1)*100,"")</f>
+        <f>IF(COUNT(T73:T74)=2,ROUND((T73/T74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AW73" s="6">
-        <f>IF(COUNT(Y73:Y74)=2,(Y73/Y74-1)*100,"")</f>
+        <f>IF(COUNT(Y73:Y74)=2,ROUND((Y73/Y74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AX73" s="6">
-        <f>IF(COUNT(AD73:AD74)=2,(AD73/AD74-1)*100,"")</f>
+        <f>IF(COUNT(AD73:AD74)=2,ROUND((AD73/AD74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AY73" s="6">
-        <f>IF(COUNT(AI73:AI74)=2,(AI73/AI74-1)*100,"")</f>
+        <f>IF(COUNT(AI73:AI74)=2,ROUND((AI73/AI74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="AZ73" s="6">
-        <f>IF(COUNT(AN73:AN74)=2,(AN73/AN74-1)*100,"")</f>
+        <f>IF(COUNT(AN73:AN74)=2,ROUND((AN73/AN74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BA73" s="6">
-        <f>IF(COUNT(AS73:AS74)=2,(AS73/AS74-1)*100,"")</f>
+        <f>IF(COUNT(AS73:AS74)=2,ROUND((AS73/AS74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BB73" s="5" t="n">
         <v>18.38</v>
       </c>
       <c r="BC73" s="6">
-        <f>IF(COUNT(BB73:BB74)=2,(BB73/BB74-1)*100,"")</f>
+        <f>IF(COUNT(BB73:BB74)=2,ROUND((BB73/BB74-1)*100,4),"")</f>
         <v/>
       </c>
       <c r="BD73" s="6" t="n">

</xml_diff>

<commit_message>
fix: align blank column layout with manual EEM format
</commit_message>
<xml_diff>
--- a/04_结果/示例审批/两基金_m30新版式示例_公式说明版.xlsx
+++ b/04_结果/示例审批/两基金_m30新版式示例_公式说明版.xlsx
@@ -557,7 +557,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   表内按区块排列：基金区、每支ETF、ETF区结束后均用空白列分隔；外部 VIX→回报。</t>
+          <t xml:space="preserve">   表内按区块排列：基金区、每支ETF、ETF区、VIX区结束后均用空白列分隔。</t>
         </is>
       </c>
     </row>
@@ -988,12 +988,15 @@
         <f>BQ3/(BQ3+BQ4)</f>
         <v/>
       </c>
-      <c r="BR2" s="3" t="n"/>
-      <c r="BS2" s="3">
-        <f>BS3/(BS3+BS4)</f>
-        <v/>
-      </c>
-      <c r="BT2" s="3" t="n"/>
+      <c r="BR2" s="3">
+        <f>BR3/(BR3+BR4)</f>
+        <v/>
+      </c>
+      <c r="BS2" s="3" t="n"/>
+      <c r="BT2" s="3">
+        <f>BT3/(BT3+BT4)</f>
+        <v/>
+      </c>
       <c r="BU2" s="3">
         <f>BU3/(BU3+BU4)</f>
         <v/>
@@ -1002,10 +1005,7 @@
         <f>BV3/(BV3+BV4)</f>
         <v/>
       </c>
-      <c r="BW2" s="3">
-        <f>BW3/(BW3+BW4)</f>
-        <v/>
-      </c>
+      <c r="BW2" s="3" t="n"/>
       <c r="BX2" s="3">
         <f>BX3/(BX3+BX4)</f>
         <v/>
@@ -1290,12 +1290,15 @@
         <f>COUNTIF(BQ16:BQ75,"&gt;0")</f>
         <v/>
       </c>
-      <c r="BR3" s="3" t="n"/>
-      <c r="BS3" s="3">
-        <f>COUNTIF(BS16:BS75,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="BT3" s="3" t="n"/>
+      <c r="BR3" s="3">
+        <f>COUNTIF(BR16:BR75,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="BS3" s="3" t="n"/>
+      <c r="BT3" s="3">
+        <f>COUNTIF(BT16:BT75,"&gt;0")</f>
+        <v/>
+      </c>
       <c r="BU3" s="3">
         <f>COUNTIF(BU16:BU75,"&gt;0")</f>
         <v/>
@@ -1304,10 +1307,7 @@
         <f>COUNTIF(BV16:BV75,"&gt;0")</f>
         <v/>
       </c>
-      <c r="BW3" s="3">
-        <f>COUNTIF(BW16:BW75,"&gt;0")</f>
-        <v/>
-      </c>
+      <c r="BW3" s="3" t="n"/>
       <c r="BX3" s="3">
         <f>COUNTIF(BX16:BX75,"&gt;0")</f>
         <v/>
@@ -1592,12 +1592,15 @@
         <f>COUNTIF(BQ16:BQ75,"&lt;0")</f>
         <v/>
       </c>
-      <c r="BR4" s="3" t="n"/>
-      <c r="BS4" s="3">
-        <f>COUNTIF(BS16:BS75,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="BT4" s="3" t="n"/>
+      <c r="BR4" s="3">
+        <f>COUNTIF(BR16:BR75,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="BS4" s="3" t="n"/>
+      <c r="BT4" s="3">
+        <f>COUNTIF(BT16:BT75,"&lt;0")</f>
+        <v/>
+      </c>
       <c r="BU4" s="3">
         <f>COUNTIF(BU16:BU75,"&lt;0")</f>
         <v/>
@@ -1606,10 +1609,7 @@
         <f>COUNTIF(BV16:BV75,"&lt;0")</f>
         <v/>
       </c>
-      <c r="BW4" s="3">
-        <f>COUNTIF(BW16:BW75,"&lt;0")</f>
-        <v/>
-      </c>
+      <c r="BW4" s="3" t="n"/>
       <c r="BX4" s="3">
         <f>COUNTIF(BX16:BX75,"&lt;0")</f>
         <v/>
@@ -1894,12 +1894,15 @@
         <f>AVERAGE(BQ16:BQ75)</f>
         <v/>
       </c>
-      <c r="BR5" s="3" t="n"/>
-      <c r="BS5" s="3">
-        <f>AVERAGE(BS16:BS75)</f>
-        <v/>
-      </c>
-      <c r="BT5" s="3" t="n"/>
+      <c r="BR5" s="3">
+        <f>AVERAGE(BR16:BR75)</f>
+        <v/>
+      </c>
+      <c r="BS5" s="3" t="n"/>
+      <c r="BT5" s="3">
+        <f>AVERAGE(BT16:BT75)</f>
+        <v/>
+      </c>
       <c r="BU5" s="3">
         <f>AVERAGE(BU16:BU75)</f>
         <v/>
@@ -1908,10 +1911,7 @@
         <f>AVERAGE(BV16:BV75)</f>
         <v/>
       </c>
-      <c r="BW5" s="3">
-        <f>AVERAGE(BW16:BW75)</f>
-        <v/>
-      </c>
+      <c r="BW5" s="3" t="n"/>
       <c r="BX5" s="3">
         <f>AVERAGE(BX16:BX75)</f>
         <v/>
@@ -2196,12 +2196,15 @@
         <f>MAX(BQ16:BQ75)</f>
         <v/>
       </c>
-      <c r="BR6" s="3" t="n"/>
-      <c r="BS6" s="3">
-        <f>MAX(BS16:BS75)</f>
-        <v/>
-      </c>
-      <c r="BT6" s="3" t="n"/>
+      <c r="BR6" s="3">
+        <f>MAX(BR16:BR75)</f>
+        <v/>
+      </c>
+      <c r="BS6" s="3" t="n"/>
+      <c r="BT6" s="3">
+        <f>MAX(BT16:BT75)</f>
+        <v/>
+      </c>
       <c r="BU6" s="3">
         <f>MAX(BU16:BU75)</f>
         <v/>
@@ -2210,10 +2213,7 @@
         <f>MAX(BV16:BV75)</f>
         <v/>
       </c>
-      <c r="BW6" s="3">
-        <f>MAX(BW16:BW75)</f>
-        <v/>
-      </c>
+      <c r="BW6" s="3" t="n"/>
       <c r="BX6" s="3">
         <f>MAX(BX16:BX75)</f>
         <v/>
@@ -2498,12 +2498,15 @@
         <f>MIN(BQ16:BQ75)</f>
         <v/>
       </c>
-      <c r="BR7" s="3" t="n"/>
-      <c r="BS7" s="3">
-        <f>MIN(BS16:BS75)</f>
-        <v/>
-      </c>
-      <c r="BT7" s="3" t="n"/>
+      <c r="BR7" s="3">
+        <f>MIN(BR16:BR75)</f>
+        <v/>
+      </c>
+      <c r="BS7" s="3" t="n"/>
+      <c r="BT7" s="3">
+        <f>MIN(BT16:BT75)</f>
+        <v/>
+      </c>
       <c r="BU7" s="3">
         <f>MIN(BU16:BU75)</f>
         <v/>
@@ -2512,10 +2515,7 @@
         <f>MIN(BV16:BV75)</f>
         <v/>
       </c>
-      <c r="BW7" s="3">
-        <f>MIN(BW16:BW75)</f>
-        <v/>
-      </c>
+      <c r="BW7" s="3" t="n"/>
       <c r="BX7" s="3">
         <f>MIN(BX16:BX75)</f>
         <v/>
@@ -2800,12 +2800,15 @@
         <f>COUNT(BQ16:BQ75)</f>
         <v/>
       </c>
-      <c r="BR8" s="3" t="n"/>
-      <c r="BS8" s="3">
-        <f>COUNT(BS16:BS75)</f>
-        <v/>
-      </c>
-      <c r="BT8" s="3" t="n"/>
+      <c r="BR8" s="3">
+        <f>COUNT(BR16:BR75)</f>
+        <v/>
+      </c>
+      <c r="BS8" s="3" t="n"/>
+      <c r="BT8" s="3">
+        <f>COUNT(BT16:BT75)</f>
+        <v/>
+      </c>
       <c r="BU8" s="3">
         <f>COUNT(BU16:BU75)</f>
         <v/>
@@ -2814,10 +2817,7 @@
         <f>COUNT(BV16:BV75)</f>
         <v/>
       </c>
-      <c r="BW8" s="3">
-        <f>COUNT(BW16:BW75)</f>
-        <v/>
-      </c>
+      <c r="BW8" s="3" t="n"/>
       <c r="BX8" s="3">
         <f>COUNT(BX16:BX75)</f>
         <v/>
@@ -3102,12 +3102,15 @@
         <f>STDEV(BQ16:BQ75)</f>
         <v/>
       </c>
-      <c r="BR9" s="3" t="n"/>
-      <c r="BS9" s="3">
-        <f>STDEV(BS16:BS75)</f>
-        <v/>
-      </c>
-      <c r="BT9" s="3" t="n"/>
+      <c r="BR9" s="3">
+        <f>STDEV(BR16:BR75)</f>
+        <v/>
+      </c>
+      <c r="BS9" s="3" t="n"/>
+      <c r="BT9" s="3">
+        <f>STDEV(BT16:BT75)</f>
+        <v/>
+      </c>
       <c r="BU9" s="3">
         <f>STDEV(BU16:BU75)</f>
         <v/>
@@ -3116,10 +3119,7 @@
         <f>STDEV(BV16:BV75)</f>
         <v/>
       </c>
-      <c r="BW9" s="3">
-        <f>STDEV(BW16:BW75)</f>
-        <v/>
-      </c>
+      <c r="BW9" s="3" t="n"/>
       <c r="BX9" s="3">
         <f>STDEV(BX16:BX75)</f>
         <v/>
@@ -3404,12 +3404,15 @@
         <f>SUM(BQ16:BQ75)</f>
         <v/>
       </c>
-      <c r="BR10" s="3" t="n"/>
-      <c r="BS10" s="3">
-        <f>SUM(BS16:BS75)</f>
-        <v/>
-      </c>
-      <c r="BT10" s="3" t="n"/>
+      <c r="BR10" s="3">
+        <f>SUM(BR16:BR75)</f>
+        <v/>
+      </c>
+      <c r="BS10" s="3" t="n"/>
+      <c r="BT10" s="3">
+        <f>SUM(BT16:BT75)</f>
+        <v/>
+      </c>
       <c r="BU10" s="3">
         <f>SUM(BU16:BU75)</f>
         <v/>
@@ -3418,10 +3421,7 @@
         <f>SUM(BV16:BV75)</f>
         <v/>
       </c>
-      <c r="BW10" s="3">
-        <f>SUM(BW16:BW75)</f>
-        <v/>
-      </c>
+      <c r="BW10" s="3" t="n"/>
       <c r="BX10" s="3">
         <f>SUM(BX16:BX75)</f>
         <v/>
@@ -3932,28 +3932,28 @@
           <t>GDX回报</t>
         </is>
       </c>
-      <c r="BR15" s="4" t="inlineStr"/>
-      <c r="BS15" s="4" t="inlineStr">
+      <c r="BR15" s="4" t="inlineStr">
         <is>
           <t>XLC回报</t>
         </is>
       </c>
-      <c r="BT15" s="4" t="inlineStr"/>
-      <c r="BU15" s="4" t="inlineStr">
+      <c r="BS15" s="4" t="inlineStr"/>
+      <c r="BT15" s="4" t="inlineStr">
         <is>
           <t>VIX_Close</t>
         </is>
       </c>
-      <c r="BV15" s="4" t="inlineStr">
+      <c r="BU15" s="4" t="inlineStr">
         <is>
           <t>VIX回报</t>
         </is>
       </c>
-      <c r="BW15" s="4" t="inlineStr">
+      <c r="BV15" s="4" t="inlineStr">
         <is>
           <t>VIX_Chg%</t>
         </is>
       </c>
+      <c r="BW15" s="4" t="inlineStr"/>
       <c r="BX15" s="4" t="inlineStr">
         <is>
           <t>VIX&gt;0 且 该基金当日回报&lt;=-2%，买基金第二天</t>
@@ -4196,22 +4196,22 @@
         <f>IF(COUNT(BA16:BA17)=2,ROUND((BA16/BA17-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR16" s="5" t="inlineStr"/>
-      <c r="BS16" s="6">
+      <c r="BR16" s="6">
         <f>IF(COUNT(BH16:BH17)=2,ROUND((BH16/BH17-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT16" s="5" t="inlineStr"/>
-      <c r="BU16" s="5" t="n">
+      <c r="BS16" s="5" t="inlineStr"/>
+      <c r="BT16" s="5" t="n">
         <v>16.5</v>
       </c>
-      <c r="BV16" s="6">
-        <f>IF(COUNT(BU16:BU17)=2,ROUND((BU16/BU17-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW16" s="6" t="n">
+      <c r="BU16" s="6">
+        <f>IF(COUNT(BT16:BT17)=2,ROUND((BT16/BT17-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV16" s="6" t="n">
         <v>4.0353</v>
       </c>
+      <c r="BW16" s="5" t="inlineStr"/>
       <c r="BX16" s="6" t="inlineStr"/>
       <c r="BY16" s="6" t="inlineStr"/>
       <c r="BZ16" s="6" t="inlineStr"/>
@@ -4428,24 +4428,24 @@
         <f>IF(COUNT(BA17:BA18)=2,ROUND((BA17/BA18-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR17" s="5" t="inlineStr"/>
-      <c r="BS17" s="6">
+      <c r="BR17" s="6">
         <f>IF(COUNT(BH17:BH18)=2,ROUND((BH17/BH18-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT17" s="5" t="inlineStr"/>
-      <c r="BU17" s="5" t="n">
+      <c r="BS17" s="5" t="inlineStr"/>
+      <c r="BT17" s="5" t="n">
         <v>15.86</v>
       </c>
-      <c r="BV17" s="6">
-        <f>IF(COUNT(BU17:BU18)=2,ROUND((BU17/BU18-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW17" s="6" t="n">
+      <c r="BU17" s="6">
+        <f>IF(COUNT(BT17:BT18)=2,ROUND((BT17/BT18-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV17" s="6" t="n">
         <v>-0.8129999999999999</v>
       </c>
+      <c r="BW17" s="5" t="inlineStr"/>
       <c r="BX17" s="6">
-        <f>IF(AND(BW17&gt;$BX$12,D17&lt;=$BX$13),D16,"")</f>
+        <f>IF(AND(BV17&gt;$BX$12,D17&lt;=$BX$13),D16,"")</f>
         <v/>
       </c>
       <c r="BY17" s="6">
@@ -4461,7 +4461,7 @@
         <v/>
       </c>
       <c r="CB17" s="6">
-        <f>IF(AND(BQ17&gt;$CB$12,BS17&lt;$CB$13),E16,"")</f>
+        <f>IF(AND(BQ17&gt;$CB$12,BR17&lt;$CB$13),E16,"")</f>
         <v/>
       </c>
       <c r="CC17" s="6">
@@ -4678,24 +4678,24 @@
         <f>IF(COUNT(BA18:BA19)=2,ROUND((BA18/BA19-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR18" s="5" t="inlineStr"/>
-      <c r="BS18" s="6">
+      <c r="BR18" s="6">
         <f>IF(COUNT(BH18:BH19)=2,ROUND((BH18/BH19-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT18" s="5" t="inlineStr"/>
-      <c r="BU18" s="5" t="n">
+      <c r="BS18" s="5" t="inlineStr"/>
+      <c r="BT18" s="5" t="n">
         <v>15.99</v>
       </c>
-      <c r="BV18" s="6">
-        <f>IF(COUNT(BU18:BU19)=2,ROUND((BU18/BU19-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW18" s="6" t="n">
+      <c r="BU18" s="6">
+        <f>IF(COUNT(BT18:BT19)=2,ROUND((BT18/BT19-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV18" s="6" t="n">
         <v>-6.4365</v>
       </c>
+      <c r="BW18" s="5" t="inlineStr"/>
       <c r="BX18" s="6">
-        <f>IF(AND(BW18&gt;$BX$12,D18&lt;=$BX$13),D17,"")</f>
+        <f>IF(AND(BV18&gt;$BX$12,D18&lt;=$BX$13),D17,"")</f>
         <v/>
       </c>
       <c r="BY18" s="6">
@@ -4711,7 +4711,7 @@
         <v/>
       </c>
       <c r="CB18" s="6">
-        <f>IF(AND(BQ18&gt;$CB$12,BS18&lt;$CB$13),E17,"")</f>
+        <f>IF(AND(BQ18&gt;$CB$12,BR18&lt;$CB$13),E17,"")</f>
         <v/>
       </c>
       <c r="CC18" s="6">
@@ -4928,24 +4928,24 @@
         <f>IF(COUNT(BA19:BA20)=2,ROUND((BA19/BA20-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR19" s="5" t="inlineStr"/>
-      <c r="BS19" s="6">
+      <c r="BR19" s="6">
         <f>IF(COUNT(BH19:BH20)=2,ROUND((BH19/BH20-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT19" s="5" t="inlineStr"/>
-      <c r="BU19" s="5" t="n">
+      <c r="BS19" s="5" t="inlineStr"/>
+      <c r="BT19" s="5" t="n">
         <v>17.09</v>
       </c>
-      <c r="BV19" s="6">
-        <f>IF(COUNT(BU19:BU20)=2,ROUND((BU19/BU20-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW19" s="6" t="n">
+      <c r="BU19" s="6">
+        <f>IF(COUNT(BT19:BT20)=2,ROUND((BT19/BT20-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV19" s="6" t="n">
         <v>-17.2798</v>
       </c>
+      <c r="BW19" s="5" t="inlineStr"/>
       <c r="BX19" s="6">
-        <f>IF(AND(BW19&gt;$BX$12,D19&lt;=$BX$13),D18,"")</f>
+        <f>IF(AND(BV19&gt;$BX$12,D19&lt;=$BX$13),D18,"")</f>
         <v/>
       </c>
       <c r="BY19" s="6">
@@ -4961,7 +4961,7 @@
         <v/>
       </c>
       <c r="CB19" s="6">
-        <f>IF(AND(BQ19&gt;$CB$12,BS19&lt;$CB$13),E18,"")</f>
+        <f>IF(AND(BQ19&gt;$CB$12,BR19&lt;$CB$13),E18,"")</f>
         <v/>
       </c>
       <c r="CC19" s="6">
@@ -5178,24 +5178,24 @@
         <f>IF(COUNT(BA20:BA21)=2,ROUND((BA20/BA21-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR20" s="5" t="inlineStr"/>
-      <c r="BS20" s="6">
+      <c r="BR20" s="6">
         <f>IF(COUNT(BH20:BH21)=2,ROUND((BH20/BH21-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT20" s="5" t="inlineStr"/>
-      <c r="BU20" s="5" t="n">
+      <c r="BS20" s="5" t="inlineStr"/>
+      <c r="BT20" s="5" t="n">
         <v>20.66</v>
       </c>
-      <c r="BV20" s="6">
-        <f>IF(COUNT(BU20:BU21)=2,ROUND((BU20/BU21-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW20" s="6" t="n">
+      <c r="BU20" s="6">
+        <f>IF(COUNT(BT20:BT21)=2,ROUND((BT20/BT21-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV20" s="6" t="n">
         <v>13.4541</v>
       </c>
+      <c r="BW20" s="5" t="inlineStr"/>
       <c r="BX20" s="6">
-        <f>IF(AND(BW20&gt;$BX$12,D20&lt;=$BX$13),D19,"")</f>
+        <f>IF(AND(BV20&gt;$BX$12,D20&lt;=$BX$13),D19,"")</f>
         <v/>
       </c>
       <c r="BY20" s="6">
@@ -5211,7 +5211,7 @@
         <v/>
       </c>
       <c r="CB20" s="6">
-        <f>IF(AND(BQ20&gt;$CB$12,BS20&lt;$CB$13),E19,"")</f>
+        <f>IF(AND(BQ20&gt;$CB$12,BR20&lt;$CB$13),E19,"")</f>
         <v/>
       </c>
       <c r="CC20" s="6">
@@ -5428,24 +5428,24 @@
         <f>IF(COUNT(BA21:BA22)=2,ROUND((BA21/BA22-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR21" s="5" t="inlineStr"/>
-      <c r="BS21" s="6">
+      <c r="BR21" s="6">
         <f>IF(COUNT(BH21:BH22)=2,ROUND((BH21/BH22-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT21" s="5" t="inlineStr"/>
-      <c r="BU21" s="5" t="n">
+      <c r="BS21" s="5" t="inlineStr"/>
+      <c r="BT21" s="5" t="n">
         <v>18.21</v>
       </c>
-      <c r="BV21" s="6">
-        <f>IF(COUNT(BU21:BU22)=2,ROUND((BU21/BU22-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW21" s="6" t="n">
+      <c r="BU21" s="6">
+        <f>IF(COUNT(BT21:BT22)=2,ROUND((BT21/BT22-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV21" s="6" t="n">
         <v>-2.4638</v>
       </c>
+      <c r="BW21" s="5" t="inlineStr"/>
       <c r="BX21" s="6">
-        <f>IF(AND(BW21&gt;$BX$12,D21&lt;=$BX$13),D20,"")</f>
+        <f>IF(AND(BV21&gt;$BX$12,D21&lt;=$BX$13),D20,"")</f>
         <v/>
       </c>
       <c r="BY21" s="6">
@@ -5461,7 +5461,7 @@
         <v/>
       </c>
       <c r="CB21" s="6">
-        <f>IF(AND(BQ21&gt;$CB$12,BS21&lt;$CB$13),E20,"")</f>
+        <f>IF(AND(BQ21&gt;$CB$12,BR21&lt;$CB$13),E20,"")</f>
         <v/>
       </c>
       <c r="CC21" s="6">
@@ -5678,24 +5678,24 @@
         <f>IF(COUNT(BA22:BA23)=2,ROUND((BA22/BA23-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR22" s="5" t="inlineStr"/>
-      <c r="BS22" s="6">
+      <c r="BR22" s="6">
         <f>IF(COUNT(BH22:BH23)=2,ROUND((BH22/BH23-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT22" s="5" t="inlineStr"/>
-      <c r="BU22" s="5" t="n">
+      <c r="BS22" s="5" t="inlineStr"/>
+      <c r="BT22" s="5" t="n">
         <v>18.67</v>
       </c>
-      <c r="BV22" s="6">
-        <f>IF(COUNT(BU22:BU23)=2,ROUND((BU22/BU23-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW22" s="6" t="n">
+      <c r="BU22" s="6">
+        <f>IF(COUNT(BT22:BT23)=2,ROUND((BT22/BT23-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV22" s="6" t="n">
         <v>0.4844</v>
       </c>
+      <c r="BW22" s="5" t="inlineStr"/>
       <c r="BX22" s="6">
-        <f>IF(AND(BW22&gt;$BX$12,D22&lt;=$BX$13),D21,"")</f>
+        <f>IF(AND(BV22&gt;$BX$12,D22&lt;=$BX$13),D21,"")</f>
         <v/>
       </c>
       <c r="BY22" s="6">
@@ -5711,7 +5711,7 @@
         <v/>
       </c>
       <c r="CB22" s="6">
-        <f>IF(AND(BQ22&gt;$CB$12,BS22&lt;$CB$13),E21,"")</f>
+        <f>IF(AND(BQ22&gt;$CB$12,BR22&lt;$CB$13),E21,"")</f>
         <v/>
       </c>
       <c r="CC22" s="6">
@@ -5928,24 +5928,24 @@
         <f>IF(COUNT(BA23:BA24)=2,ROUND((BA23/BA24-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR23" s="5" t="inlineStr"/>
-      <c r="BS23" s="6">
+      <c r="BR23" s="6">
         <f>IF(COUNT(BH23:BH24)=2,ROUND((BH23/BH24-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT23" s="5" t="inlineStr"/>
-      <c r="BU23" s="5" t="n">
+      <c r="BS23" s="5" t="inlineStr"/>
+      <c r="BT23" s="5" t="n">
         <v>18.58</v>
       </c>
-      <c r="BV23" s="6">
-        <f>IF(COUNT(BU23:BU24)=2,ROUND((BU23/BU24-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW23" s="6" t="n">
+      <c r="BU23" s="6">
+        <f>IF(COUNT(BT23:BT24)=2,ROUND((BT23/BT24-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV23" s="6" t="n">
         <v>-0.6417</v>
       </c>
+      <c r="BW23" s="5" t="inlineStr"/>
       <c r="BX23" s="6">
-        <f>IF(AND(BW23&gt;$BX$12,D23&lt;=$BX$13),D22,"")</f>
+        <f>IF(AND(BV23&gt;$BX$12,D23&lt;=$BX$13),D22,"")</f>
         <v/>
       </c>
       <c r="BY23" s="6">
@@ -5961,7 +5961,7 @@
         <v/>
       </c>
       <c r="CB23" s="6">
-        <f>IF(AND(BQ23&gt;$CB$12,BS23&lt;$CB$13),E22,"")</f>
+        <f>IF(AND(BQ23&gt;$CB$12,BR23&lt;$CB$13),E22,"")</f>
         <v/>
       </c>
       <c r="CC23" s="6">
@@ -6178,24 +6178,24 @@
         <f>IF(COUNT(BA24:BA25)=2,ROUND((BA24/BA25-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR24" s="5" t="inlineStr"/>
-      <c r="BS24" s="6">
+      <c r="BR24" s="6">
         <f>IF(COUNT(BH24:BH25)=2,ROUND((BH24/BH25-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT24" s="5" t="inlineStr"/>
-      <c r="BU24" s="5" t="n">
+      <c r="BS24" s="5" t="inlineStr"/>
+      <c r="BT24" s="5" t="n">
         <v>18.7</v>
       </c>
-      <c r="BV24" s="6">
-        <f>IF(COUNT(BU24:BU25)=2,ROUND((BU24/BU25-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW24" s="6" t="n">
+      <c r="BU24" s="6">
+        <f>IF(COUNT(BT24:BT25)=2,ROUND((BT24/BT25-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV24" s="6" t="n">
         <v>12.3798</v>
       </c>
+      <c r="BW24" s="5" t="inlineStr"/>
       <c r="BX24" s="6">
-        <f>IF(AND(BW24&gt;$BX$12,D24&lt;=$BX$13),D23,"")</f>
+        <f>IF(AND(BV24&gt;$BX$12,D24&lt;=$BX$13),D23,"")</f>
         <v/>
       </c>
       <c r="BY24" s="6">
@@ -6211,7 +6211,7 @@
         <v/>
       </c>
       <c r="CB24" s="6">
-        <f>IF(AND(BQ24&gt;$CB$12,BS24&lt;$CB$13),E23,"")</f>
+        <f>IF(AND(BQ24&gt;$CB$12,BR24&lt;$CB$13),E23,"")</f>
         <v/>
       </c>
       <c r="CC24" s="6">
@@ -6428,24 +6428,24 @@
         <f>IF(COUNT(BA25:BA26)=2,ROUND((BA25/BA26-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR25" s="5" t="inlineStr"/>
-      <c r="BS25" s="6">
+      <c r="BR25" s="6">
         <f>IF(COUNT(BH25:BH26)=2,ROUND((BH25/BH26-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT25" s="5" t="inlineStr"/>
-      <c r="BU25" s="5" t="n">
+      <c r="BS25" s="5" t="inlineStr"/>
+      <c r="BT25" s="5" t="n">
         <v>16.64</v>
       </c>
-      <c r="BV25" s="6">
-        <f>IF(COUNT(BU25:BU26)=2,ROUND((BU25/BU26-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW25" s="6" t="n">
+      <c r="BU25" s="6">
+        <f>IF(COUNT(BT25:BT26)=2,ROUND((BT25/BT26-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV25" s="6" t="n">
         <v>-2.4047</v>
       </c>
+      <c r="BW25" s="5" t="inlineStr"/>
       <c r="BX25" s="6">
-        <f>IF(AND(BW25&gt;$BX$12,D25&lt;=$BX$13),D24,"")</f>
+        <f>IF(AND(BV25&gt;$BX$12,D25&lt;=$BX$13),D24,"")</f>
         <v/>
       </c>
       <c r="BY25" s="6">
@@ -6461,7 +6461,7 @@
         <v/>
       </c>
       <c r="CB25" s="6">
-        <f>IF(AND(BQ25&gt;$CB$12,BS25&lt;$CB$13),E24,"")</f>
+        <f>IF(AND(BQ25&gt;$CB$12,BR25&lt;$CB$13),E24,"")</f>
         <v/>
       </c>
       <c r="CC25" s="6">
@@ -6678,24 +6678,24 @@
         <f>IF(COUNT(BA26:BA27)=2,ROUND((BA26/BA27-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR26" s="5" t="inlineStr"/>
-      <c r="BS26" s="6">
+      <c r="BR26" s="6">
         <f>IF(COUNT(BH26:BH27)=2,ROUND((BH26/BH27-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT26" s="5" t="inlineStr"/>
-      <c r="BU26" s="5" t="n">
+      <c r="BS26" s="5" t="inlineStr"/>
+      <c r="BT26" s="5" t="n">
         <v>17.05</v>
       </c>
-      <c r="BV26" s="6">
-        <f>IF(COUNT(BU26:BU27)=2,ROUND((BU26/BU27-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW26" s="6" t="n">
+      <c r="BU26" s="6">
+        <f>IF(COUNT(BT26:BT27)=2,ROUND((BT26/BT27-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV26" s="6" t="n">
         <v>-8.5791</v>
       </c>
+      <c r="BW26" s="5" t="inlineStr"/>
       <c r="BX26" s="6">
-        <f>IF(AND(BW26&gt;$BX$12,D26&lt;=$BX$13),D25,"")</f>
+        <f>IF(AND(BV26&gt;$BX$12,D26&lt;=$BX$13),D25,"")</f>
         <v/>
       </c>
       <c r="BY26" s="6">
@@ -6711,7 +6711,7 @@
         <v/>
       </c>
       <c r="CB26" s="6">
-        <f>IF(AND(BQ26&gt;$CB$12,BS26&lt;$CB$13),E25,"")</f>
+        <f>IF(AND(BQ26&gt;$CB$12,BR26&lt;$CB$13),E25,"")</f>
         <v/>
       </c>
       <c r="CC26" s="6">
@@ -6928,24 +6928,24 @@
         <f>IF(COUNT(BA27:BA28)=2,ROUND((BA27/BA28-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR27" s="5" t="inlineStr"/>
-      <c r="BS27" s="6">
+      <c r="BR27" s="6">
         <f>IF(COUNT(BH27:BH28)=2,ROUND((BH27/BH28-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT27" s="5" t="inlineStr"/>
-      <c r="BU27" s="5" t="n">
+      <c r="BS27" s="5" t="inlineStr"/>
+      <c r="BT27" s="5" t="n">
         <v>18.65</v>
       </c>
-      <c r="BV27" s="6">
-        <f>IF(COUNT(BU27:BU28)=2,ROUND((BU27/BU28-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW27" s="6" t="n">
+      <c r="BU27" s="6">
+        <f>IF(COUNT(BT27:BT28)=2,ROUND((BT27/BT28-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV27" s="6" t="n">
         <v>-0.6393</v>
       </c>
+      <c r="BW27" s="5" t="inlineStr"/>
       <c r="BX27" s="6">
-        <f>IF(AND(BW27&gt;$BX$12,D27&lt;=$BX$13),D26,"")</f>
+        <f>IF(AND(BV27&gt;$BX$12,D27&lt;=$BX$13),D26,"")</f>
         <v/>
       </c>
       <c r="BY27" s="6">
@@ -6961,7 +6961,7 @@
         <v/>
       </c>
       <c r="CB27" s="6">
-        <f>IF(AND(BQ27&gt;$CB$12,BS27&lt;$CB$13),E26,"")</f>
+        <f>IF(AND(BQ27&gt;$CB$12,BR27&lt;$CB$13),E26,"")</f>
         <v/>
       </c>
       <c r="CC27" s="6">
@@ -7178,24 +7178,24 @@
         <f>IF(COUNT(BA28:BA29)=2,ROUND((BA28/BA29-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR28" s="5" t="inlineStr"/>
-      <c r="BS28" s="6">
+      <c r="BR28" s="6">
         <f>IF(COUNT(BH28:BH29)=2,ROUND((BH28/BH29-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT28" s="5" t="inlineStr"/>
-      <c r="BU28" s="5" t="n">
+      <c r="BS28" s="5" t="inlineStr"/>
+      <c r="BT28" s="5" t="n">
         <v>18.77</v>
       </c>
-      <c r="BV28" s="6">
-        <f>IF(COUNT(BU28:BU29)=2,ROUND((BU28/BU29-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW28" s="6" t="n">
+      <c r="BU28" s="6">
+        <f>IF(COUNT(BT28:BT29)=2,ROUND((BT28/BT29-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV28" s="6" t="n">
         <v>12.1937</v>
       </c>
+      <c r="BW28" s="5" t="inlineStr"/>
       <c r="BX28" s="6">
-        <f>IF(AND(BW28&gt;$BX$12,D28&lt;=$BX$13),D27,"")</f>
+        <f>IF(AND(BV28&gt;$BX$12,D28&lt;=$BX$13),D27,"")</f>
         <v/>
       </c>
       <c r="BY28" s="6">
@@ -7211,7 +7211,7 @@
         <v/>
       </c>
       <c r="CB28" s="6">
-        <f>IF(AND(BQ28&gt;$CB$12,BS28&lt;$CB$13),E27,"")</f>
+        <f>IF(AND(BQ28&gt;$CB$12,BR28&lt;$CB$13),E27,"")</f>
         <v/>
       </c>
       <c r="CC28" s="6">
@@ -7428,24 +7428,24 @@
         <f>IF(COUNT(BA29:BA30)=2,ROUND((BA29/BA30-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR29" s="5" t="inlineStr"/>
-      <c r="BS29" s="6">
+      <c r="BR29" s="6">
         <f>IF(COUNT(BH29:BH30)=2,ROUND((BH29/BH30-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT29" s="5" t="inlineStr"/>
-      <c r="BU29" s="5" t="n">
+      <c r="BS29" s="5" t="inlineStr"/>
+      <c r="BT29" s="5" t="n">
         <v>16.73</v>
       </c>
-      <c r="BV29" s="6">
-        <f>IF(COUNT(BU29:BU30)=2,ROUND((BU29/BU30-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW29" s="6" t="n">
+      <c r="BU29" s="6">
+        <f>IF(COUNT(BT29:BT30)=2,ROUND((BT29/BT30-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV29" s="6" t="n">
         <v>6.7645</v>
       </c>
+      <c r="BW29" s="5" t="inlineStr"/>
       <c r="BX29" s="6">
-        <f>IF(AND(BW29&gt;$BX$12,D29&lt;=$BX$13),D28,"")</f>
+        <f>IF(AND(BV29&gt;$BX$12,D29&lt;=$BX$13),D28,"")</f>
         <v/>
       </c>
       <c r="BY29" s="6">
@@ -7461,7 +7461,7 @@
         <v/>
       </c>
       <c r="CB29" s="6">
-        <f>IF(AND(BQ29&gt;$CB$12,BS29&lt;$CB$13),E28,"")</f>
+        <f>IF(AND(BQ29&gt;$CB$12,BR29&lt;$CB$13),E28,"")</f>
         <v/>
       </c>
       <c r="CC29" s="6">
@@ -7678,24 +7678,24 @@
         <f>IF(COUNT(BA30:BA31)=2,ROUND((BA30/BA31-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR30" s="5" t="inlineStr"/>
-      <c r="BS30" s="6">
+      <c r="BR30" s="6">
         <f>IF(COUNT(BH30:BH31)=2,ROUND((BH30/BH31-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT30" s="5" t="inlineStr"/>
-      <c r="BU30" s="5" t="n">
+      <c r="BS30" s="5" t="inlineStr"/>
+      <c r="BT30" s="5" t="n">
         <v>15.67</v>
       </c>
-      <c r="BV30" s="6">
-        <f>IF(COUNT(BU30:BU31)=2,ROUND((BU30/BU31-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW30" s="6" t="n">
+      <c r="BU30" s="6">
+        <f>IF(COUNT(BT30:BT31)=2,ROUND((BT30/BT31-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV30" s="6" t="n">
         <v>-5.0303</v>
       </c>
+      <c r="BW30" s="5" t="inlineStr"/>
       <c r="BX30" s="6">
-        <f>IF(AND(BW30&gt;$BX$12,D30&lt;=$BX$13),D29,"")</f>
+        <f>IF(AND(BV30&gt;$BX$12,D30&lt;=$BX$13),D29,"")</f>
         <v/>
       </c>
       <c r="BY30" s="6">
@@ -7711,7 +7711,7 @@
         <v/>
       </c>
       <c r="CB30" s="6">
-        <f>IF(AND(BQ30&gt;$CB$12,BS30&lt;$CB$13),E29,"")</f>
+        <f>IF(AND(BQ30&gt;$CB$12,BR30&lt;$CB$13),E29,"")</f>
         <v/>
       </c>
       <c r="CC30" s="6">
@@ -7928,24 +7928,24 @@
         <f>IF(COUNT(BA31:BA32)=2,ROUND((BA31/BA32-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR31" s="5" t="inlineStr"/>
-      <c r="BS31" s="6">
+      <c r="BR31" s="6">
         <f>IF(COUNT(BH31:BH32)=2,ROUND((BH31/BH32-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT31" s="5" t="inlineStr"/>
-      <c r="BU31" s="5" t="n">
+      <c r="BS31" s="5" t="inlineStr"/>
+      <c r="BT31" s="5" t="n">
         <v>16.5</v>
       </c>
-      <c r="BV31" s="6">
-        <f>IF(COUNT(BU31:BU32)=2,ROUND((BU31/BU32-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW31" s="6" t="n">
+      <c r="BU31" s="6">
+        <f>IF(COUNT(BT31:BT32)=2,ROUND((BT31/BT32-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV31" s="6" t="n">
         <v>-3.8462</v>
       </c>
+      <c r="BW31" s="5" t="inlineStr"/>
       <c r="BX31" s="6">
-        <f>IF(AND(BW31&gt;$BX$12,D31&lt;=$BX$13),D30,"")</f>
+        <f>IF(AND(BV31&gt;$BX$12,D31&lt;=$BX$13),D30,"")</f>
         <v/>
       </c>
       <c r="BY31" s="6">
@@ -7961,7 +7961,7 @@
         <v/>
       </c>
       <c r="CB31" s="6">
-        <f>IF(AND(BQ31&gt;$CB$12,BS31&lt;$CB$13),E30,"")</f>
+        <f>IF(AND(BQ31&gt;$CB$12,BR31&lt;$CB$13),E30,"")</f>
         <v/>
       </c>
       <c r="CC31" s="6">
@@ -8178,24 +8178,24 @@
         <f>IF(COUNT(BA32:BA33)=2,ROUND((BA32/BA33-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR32" s="5" t="inlineStr"/>
-      <c r="BS32" s="6">
+      <c r="BR32" s="6">
         <f>IF(COUNT(BH32:BH33)=2,ROUND((BH32/BH33-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT32" s="5" t="inlineStr"/>
-      <c r="BU32" s="5" t="n">
+      <c r="BS32" s="5" t="inlineStr"/>
+      <c r="BT32" s="5" t="n">
         <v>17.16</v>
       </c>
-      <c r="BV32" s="6">
-        <f>IF(COUNT(BU32:BU33)=2,ROUND((BU32/BU33-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW32" s="6" t="n">
+      <c r="BU32" s="6">
+        <f>IF(COUNT(BT32:BT33)=2,ROUND((BT32/BT33-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV32" s="6" t="n">
         <v>14.1717</v>
       </c>
+      <c r="BW32" s="5" t="inlineStr"/>
       <c r="BX32" s="6">
-        <f>IF(AND(BW32&gt;$BX$12,D32&lt;=$BX$13),D31,"")</f>
+        <f>IF(AND(BV32&gt;$BX$12,D32&lt;=$BX$13),D31,"")</f>
         <v/>
       </c>
       <c r="BY32" s="6">
@@ -8211,7 +8211,7 @@
         <v/>
       </c>
       <c r="CB32" s="6">
-        <f>IF(AND(BQ32&gt;$CB$12,BS32&lt;$CB$13),E31,"")</f>
+        <f>IF(AND(BQ32&gt;$CB$12,BR32&lt;$CB$13),E31,"")</f>
         <v/>
       </c>
       <c r="CC32" s="6">
@@ -8428,24 +8428,24 @@
         <f>IF(COUNT(BA33:BA34)=2,ROUND((BA33/BA34-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR33" s="5" t="inlineStr"/>
-      <c r="BS33" s="6">
+      <c r="BR33" s="6">
         <f>IF(COUNT(BH33:BH34)=2,ROUND((BH33/BH34-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT33" s="5" t="inlineStr"/>
-      <c r="BU33" s="5" t="n">
+      <c r="BS33" s="5" t="inlineStr"/>
+      <c r="BT33" s="5" t="n">
         <v>15.03</v>
       </c>
-      <c r="BV33" s="6">
-        <f>IF(COUNT(BU33:BU34)=2,ROUND((BU33/BU34-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW33" s="6" t="n">
+      <c r="BU33" s="6">
+        <f>IF(COUNT(BT33:BT34)=2,ROUND((BT33/BT34-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV33" s="6" t="n">
         <v>-5.1136</v>
       </c>
+      <c r="BW33" s="5" t="inlineStr"/>
       <c r="BX33" s="6">
-        <f>IF(AND(BW33&gt;$BX$12,D33&lt;=$BX$13),D32,"")</f>
+        <f>IF(AND(BV33&gt;$BX$12,D33&lt;=$BX$13),D32,"")</f>
         <v/>
       </c>
       <c r="BY33" s="6">
@@ -8461,7 +8461,7 @@
         <v/>
       </c>
       <c r="CB33" s="6">
-        <f>IF(AND(BQ33&gt;$CB$12,BS33&lt;$CB$13),E32,"")</f>
+        <f>IF(AND(BQ33&gt;$CB$12,BR33&lt;$CB$13),E32,"")</f>
         <v/>
       </c>
       <c r="CC33" s="6">
@@ -8678,24 +8678,24 @@
         <f>IF(COUNT(BA34:BA35)=2,ROUND((BA34/BA35-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR34" s="5" t="inlineStr"/>
-      <c r="BS34" s="6">
+      <c r="BR34" s="6">
         <f>IF(COUNT(BH34:BH35)=2,ROUND((BH34/BH35-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT34" s="5" t="inlineStr"/>
-      <c r="BU34" s="5" t="n">
+      <c r="BS34" s="5" t="inlineStr"/>
+      <c r="BT34" s="5" t="n">
         <v>15.84</v>
       </c>
-      <c r="BV34" s="6">
-        <f>IF(COUNT(BU34:BU35)=2,ROUND((BU34/BU35-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW34" s="6" t="n">
+      <c r="BU34" s="6">
+        <f>IF(COUNT(BT34:BT35)=2,ROUND((BT34/BT35-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV34" s="6" t="n">
         <v>-6.2722</v>
       </c>
+      <c r="BW34" s="5" t="inlineStr"/>
       <c r="BX34" s="6">
-        <f>IF(AND(BW34&gt;$BX$12,D34&lt;=$BX$13),D33,"")</f>
+        <f>IF(AND(BV34&gt;$BX$12,D34&lt;=$BX$13),D33,"")</f>
         <v/>
       </c>
       <c r="BY34" s="6">
@@ -8711,7 +8711,7 @@
         <v/>
       </c>
       <c r="CB34" s="6">
-        <f>IF(AND(BQ34&gt;$CB$12,BS34&lt;$CB$13),E33,"")</f>
+        <f>IF(AND(BQ34&gt;$CB$12,BR34&lt;$CB$13),E33,"")</f>
         <v/>
       </c>
       <c r="CC34" s="6">
@@ -8928,24 +8928,24 @@
         <f>IF(COUNT(BA35:BA36)=2,ROUND((BA35/BA36-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR35" s="5" t="inlineStr"/>
-      <c r="BS35" s="6">
+      <c r="BR35" s="6">
         <f>IF(COUNT(BH35:BH36)=2,ROUND((BH35/BH36-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT35" s="5" t="inlineStr"/>
-      <c r="BU35" s="5" t="n">
+      <c r="BS35" s="5" t="inlineStr"/>
+      <c r="BT35" s="5" t="n">
         <v>16.9</v>
       </c>
-      <c r="BV35" s="6">
-        <f>IF(COUNT(BU35:BU36)=2,ROUND((BU35/BU36-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW35" s="6" t="n">
+      <c r="BU35" s="6">
+        <f>IF(COUNT(BT35:BT36)=2,ROUND((BT35/BT36-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV35" s="6" t="n">
         <v>4.7737</v>
       </c>
+      <c r="BW35" s="5" t="inlineStr"/>
       <c r="BX35" s="6">
-        <f>IF(AND(BW35&gt;$BX$12,D35&lt;=$BX$13),D34,"")</f>
+        <f>IF(AND(BV35&gt;$BX$12,D35&lt;=$BX$13),D34,"")</f>
         <v/>
       </c>
       <c r="BY35" s="6">
@@ -8961,7 +8961,7 @@
         <v/>
       </c>
       <c r="CB35" s="6">
-        <f>IF(AND(BQ35&gt;$CB$12,BS35&lt;$CB$13),E34,"")</f>
+        <f>IF(AND(BQ35&gt;$CB$12,BR35&lt;$CB$13),E34,"")</f>
         <v/>
       </c>
       <c r="CC35" s="6">
@@ -9178,24 +9178,24 @@
         <f>IF(COUNT(BA36:BA37)=2,ROUND((BA36/BA37-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR36" s="5" t="inlineStr"/>
-      <c r="BS36" s="6">
+      <c r="BR36" s="6">
         <f>IF(COUNT(BH36:BH37)=2,ROUND((BH36/BH37-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT36" s="5" t="inlineStr"/>
-      <c r="BU36" s="5" t="n">
+      <c r="BS36" s="5" t="inlineStr"/>
+      <c r="BT36" s="5" t="n">
         <v>16.13</v>
       </c>
-      <c r="BV36" s="6">
-        <f>IF(COUNT(BU36:BU37)=2,ROUND((BU36/BU37-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW36" s="6" t="n">
+      <c r="BU36" s="6">
+        <f>IF(COUNT(BT36:BT37)=2,ROUND((BT36/BT37-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV36" s="6" t="n">
         <v>3.5967</v>
       </c>
+      <c r="BW36" s="5" t="inlineStr"/>
       <c r="BX36" s="6">
-        <f>IF(AND(BW36&gt;$BX$12,D36&lt;=$BX$13),D35,"")</f>
+        <f>IF(AND(BV36&gt;$BX$12,D36&lt;=$BX$13),D35,"")</f>
         <v/>
       </c>
       <c r="BY36" s="6">
@@ -9211,7 +9211,7 @@
         <v/>
       </c>
       <c r="CB36" s="6">
-        <f>IF(AND(BQ36&gt;$CB$12,BS36&lt;$CB$13),E35,"")</f>
+        <f>IF(AND(BQ36&gt;$CB$12,BR36&lt;$CB$13),E35,"")</f>
         <v/>
       </c>
       <c r="CC36" s="6">
@@ -9428,24 +9428,24 @@
         <f>IF(COUNT(BA37:BA38)=2,ROUND((BA37/BA38-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR37" s="5" t="inlineStr"/>
-      <c r="BS37" s="6">
+      <c r="BR37" s="6">
         <f>IF(COUNT(BH37:BH38)=2,ROUND((BH37/BH38-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT37" s="5" t="inlineStr"/>
-      <c r="BU37" s="5" t="n">
+      <c r="BS37" s="5" t="inlineStr"/>
+      <c r="BT37" s="5" t="n">
         <v>15.57</v>
       </c>
-      <c r="BV37" s="6">
-        <f>IF(COUNT(BU37:BU38)=2,ROUND((BU37/BU38-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW37" s="6" t="n">
+      <c r="BU37" s="6">
+        <f>IF(COUNT(BT37:BT38)=2,ROUND((BT37/BT38-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV37" s="6" t="n">
         <v>-3.5913</v>
       </c>
+      <c r="BW37" s="5" t="inlineStr"/>
       <c r="BX37" s="6">
-        <f>IF(AND(BW37&gt;$BX$12,D37&lt;=$BX$13),D36,"")</f>
+        <f>IF(AND(BV37&gt;$BX$12,D37&lt;=$BX$13),D36,"")</f>
         <v/>
       </c>
       <c r="BY37" s="6">
@@ -9461,7 +9461,7 @@
         <v/>
       </c>
       <c r="CB37" s="6">
-        <f>IF(AND(BQ37&gt;$CB$12,BS37&lt;$CB$13),E36,"")</f>
+        <f>IF(AND(BQ37&gt;$CB$12,BR37&lt;$CB$13),E36,"")</f>
         <v/>
       </c>
       <c r="CC37" s="6">
@@ -9678,24 +9678,24 @@
         <f>IF(COUNT(BA38:BA39)=2,ROUND((BA38/BA39-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR38" s="5" t="inlineStr"/>
-      <c r="BS38" s="6">
+      <c r="BR38" s="6">
         <f>IF(COUNT(BH38:BH39)=2,ROUND((BH38/BH39-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT38" s="5" t="inlineStr"/>
-      <c r="BU38" s="5" t="n">
+      <c r="BS38" s="5" t="inlineStr"/>
+      <c r="BT38" s="5" t="n">
         <v>16.15</v>
       </c>
-      <c r="BV38" s="6">
-        <f>IF(COUNT(BU38:BU39)=2,ROUND((BU38/BU39-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW38" s="6" t="n">
+      <c r="BU38" s="6">
+        <f>IF(COUNT(BT38:BT39)=2,ROUND((BT38/BT39-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV38" s="6" t="n">
         <v>-2.6522</v>
       </c>
+      <c r="BW38" s="5" t="inlineStr"/>
       <c r="BX38" s="6">
-        <f>IF(AND(BW38&gt;$BX$12,D38&lt;=$BX$13),D37,"")</f>
+        <f>IF(AND(BV38&gt;$BX$12,D38&lt;=$BX$13),D37,"")</f>
         <v/>
       </c>
       <c r="BY38" s="6">
@@ -9711,7 +9711,7 @@
         <v/>
       </c>
       <c r="CB38" s="6">
-        <f>IF(AND(BQ38&gt;$CB$12,BS38&lt;$CB$13),E37,"")</f>
+        <f>IF(AND(BQ38&gt;$CB$12,BR38&lt;$CB$13),E37,"")</f>
         <v/>
       </c>
       <c r="CC38" s="6">
@@ -9928,24 +9928,24 @@
         <f>IF(COUNT(BA39:BA40)=2,ROUND((BA39/BA40-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR39" s="5" t="inlineStr"/>
-      <c r="BS39" s="6">
+      <c r="BR39" s="6">
         <f>IF(COUNT(BH39:BH40)=2,ROUND((BH39/BH40-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT39" s="5" t="inlineStr"/>
-      <c r="BU39" s="5" t="n">
+      <c r="BS39" s="5" t="inlineStr"/>
+      <c r="BT39" s="5" t="n">
         <v>16.59</v>
       </c>
-      <c r="BV39" s="6">
-        <f>IF(COUNT(BU39:BU40)=2,ROUND((BU39/BU40-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW39" s="6" t="n">
+      <c r="BU39" s="6">
+        <f>IF(COUNT(BT39:BT40)=2,ROUND((BT39/BT40-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV39" s="6" t="n">
         <v>0.8511</v>
       </c>
+      <c r="BW39" s="5" t="inlineStr"/>
       <c r="BX39" s="6">
-        <f>IF(AND(BW39&gt;$BX$12,D39&lt;=$BX$13),D38,"")</f>
+        <f>IF(AND(BV39&gt;$BX$12,D39&lt;=$BX$13),D38,"")</f>
         <v/>
       </c>
       <c r="BY39" s="6">
@@ -9961,7 +9961,7 @@
         <v/>
       </c>
       <c r="CB39" s="6">
-        <f>IF(AND(BQ39&gt;$CB$12,BS39&lt;$CB$13),E38,"")</f>
+        <f>IF(AND(BQ39&gt;$CB$12,BR39&lt;$CB$13),E38,"")</f>
         <v/>
       </c>
       <c r="CC39" s="6">
@@ -10178,24 +10178,24 @@
         <f>IF(COUNT(BA40:BA41)=2,ROUND((BA40/BA41-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR40" s="5" t="inlineStr"/>
-      <c r="BS40" s="6">
+      <c r="BR40" s="6">
         <f>IF(COUNT(BH40:BH41)=2,ROUND((BH40/BH41-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT40" s="5" t="inlineStr"/>
-      <c r="BU40" s="5" t="n">
+      <c r="BS40" s="5" t="inlineStr"/>
+      <c r="BT40" s="5" t="n">
         <v>16.45</v>
       </c>
-      <c r="BV40" s="6">
-        <f>IF(COUNT(BU40:BU41)=2,ROUND((BU40/BU41-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW40" s="6" t="n">
+      <c r="BU40" s="6">
+        <f>IF(COUNT(BT40:BT41)=2,ROUND((BT40/BT41-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV40" s="6" t="n">
         <v>-6.7989</v>
       </c>
+      <c r="BW40" s="5" t="inlineStr"/>
       <c r="BX40" s="6">
-        <f>IF(AND(BW40&gt;$BX$12,D40&lt;=$BX$13),D39,"")</f>
+        <f>IF(AND(BV40&gt;$BX$12,D40&lt;=$BX$13),D39,"")</f>
         <v/>
       </c>
       <c r="BY40" s="6">
@@ -10211,7 +10211,7 @@
         <v/>
       </c>
       <c r="CB40" s="6">
-        <f>IF(AND(BQ40&gt;$CB$12,BS40&lt;$CB$13),E39,"")</f>
+        <f>IF(AND(BQ40&gt;$CB$12,BR40&lt;$CB$13),E39,"")</f>
         <v/>
       </c>
       <c r="CC40" s="6">
@@ -10428,24 +10428,24 @@
         <f>IF(COUNT(BA41:BA42)=2,ROUND((BA41/BA42-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR41" s="5" t="inlineStr"/>
-      <c r="BS41" s="6">
+      <c r="BR41" s="6">
         <f>IF(COUNT(BH41:BH42)=2,ROUND((BH41/BH42-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT41" s="5" t="inlineStr"/>
-      <c r="BU41" s="5" t="n">
+      <c r="BS41" s="5" t="inlineStr"/>
+      <c r="BT41" s="5" t="n">
         <v>17.65</v>
       </c>
-      <c r="BV41" s="6">
-        <f>IF(COUNT(BU41:BU42)=2,ROUND((BU41/BU42-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW41" s="6" t="n">
+      <c r="BU41" s="6">
+        <f>IF(COUNT(BT41:BT42)=2,ROUND((BT41/BT42-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV41" s="6" t="n">
         <v>-4.1282</v>
       </c>
+      <c r="BW41" s="5" t="inlineStr"/>
       <c r="BX41" s="6">
-        <f>IF(AND(BW41&gt;$BX$12,D41&lt;=$BX$13),D40,"")</f>
+        <f>IF(AND(BV41&gt;$BX$12,D41&lt;=$BX$13),D40,"")</f>
         <v/>
       </c>
       <c r="BY41" s="6">
@@ -10461,7 +10461,7 @@
         <v/>
       </c>
       <c r="CB41" s="6">
-        <f>IF(AND(BQ41&gt;$CB$12,BS41&lt;$CB$13),E40,"")</f>
+        <f>IF(AND(BQ41&gt;$CB$12,BR41&lt;$CB$13),E40,"")</f>
         <v/>
       </c>
       <c r="CC41" s="6">
@@ -10678,24 +10678,24 @@
         <f>IF(COUNT(BA42:BA43)=2,ROUND((BA42/BA43-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR42" s="5" t="inlineStr"/>
-      <c r="BS42" s="6">
+      <c r="BR42" s="6">
         <f>IF(COUNT(BH42:BH43)=2,ROUND((BH42/BH43-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT42" s="5" t="inlineStr"/>
-      <c r="BU42" s="5" t="n">
+      <c r="BS42" s="5" t="inlineStr"/>
+      <c r="BT42" s="5" t="n">
         <v>18.41</v>
       </c>
-      <c r="BV42" s="6">
-        <f>IF(COUNT(BU42:BU43)=2,ROUND((BU42/BU43-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW42" s="6" t="n">
+      <c r="BU42" s="6">
+        <f>IF(COUNT(BT42:BT43)=2,ROUND((BT42/BT43-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV42" s="6" t="n">
         <v>-2.541</v>
       </c>
+      <c r="BW42" s="5" t="inlineStr"/>
       <c r="BX42" s="6">
-        <f>IF(AND(BW42&gt;$BX$12,D42&lt;=$BX$13),D41,"")</f>
+        <f>IF(AND(BV42&gt;$BX$12,D42&lt;=$BX$13),D41,"")</f>
         <v/>
       </c>
       <c r="BY42" s="6">
@@ -10711,7 +10711,7 @@
         <v/>
       </c>
       <c r="CB42" s="6">
-        <f>IF(AND(BQ42&gt;$CB$12,BS42&lt;$CB$13),E41,"")</f>
+        <f>IF(AND(BQ42&gt;$CB$12,BR42&lt;$CB$13),E41,"")</f>
         <v/>
       </c>
       <c r="CC42" s="6">
@@ -10928,24 +10928,24 @@
         <f>IF(COUNT(BA43:BA44)=2,ROUND((BA43/BA44-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR43" s="5" t="inlineStr"/>
-      <c r="BS43" s="6">
+      <c r="BR43" s="6">
         <f>IF(COUNT(BH43:BH44)=2,ROUND((BH43/BH44-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT43" s="5" t="inlineStr"/>
-      <c r="BU43" s="5" t="n">
+      <c r="BS43" s="5" t="inlineStr"/>
+      <c r="BT43" s="5" t="n">
         <v>18.89</v>
       </c>
-      <c r="BV43" s="6">
-        <f>IF(COUNT(BU43:BU44)=2,ROUND((BU43/BU44-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW43" s="6" t="n">
+      <c r="BU43" s="6">
+        <f>IF(COUNT(BT43:BT44)=2,ROUND((BT43/BT44-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV43" s="6" t="n">
         <v>1.3956</v>
       </c>
+      <c r="BW43" s="5" t="inlineStr"/>
       <c r="BX43" s="6">
-        <f>IF(AND(BW43&gt;$BX$12,D43&lt;=$BX$13),D42,"")</f>
+        <f>IF(AND(BV43&gt;$BX$12,D43&lt;=$BX$13),D42,"")</f>
         <v/>
       </c>
       <c r="BY43" s="6">
@@ -10961,7 +10961,7 @@
         <v/>
       </c>
       <c r="CB43" s="6">
-        <f>IF(AND(BQ43&gt;$CB$12,BS43&lt;$CB$13),E42,"")</f>
+        <f>IF(AND(BQ43&gt;$CB$12,BR43&lt;$CB$13),E42,"")</f>
         <v/>
       </c>
       <c r="CC43" s="6">
@@ -11178,24 +11178,24 @@
         <f>IF(COUNT(BA44:BA45)=2,ROUND((BA44/BA45-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR44" s="5" t="inlineStr"/>
-      <c r="BS44" s="6">
+      <c r="BR44" s="6">
         <f>IF(COUNT(BH44:BH45)=2,ROUND((BH44/BH45-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT44" s="5" t="inlineStr"/>
-      <c r="BU44" s="5" t="n">
+      <c r="BS44" s="5" t="inlineStr"/>
+      <c r="BT44" s="5" t="n">
         <v>18.63</v>
       </c>
-      <c r="BV44" s="6">
-        <f>IF(COUNT(BU44:BU45)=2,ROUND((BU44/BU45-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW44" s="6" t="n">
+      <c r="BU44" s="6">
+        <f>IF(COUNT(BT44:BT45)=2,ROUND((BT44/BT45-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV44" s="6" t="n">
         <v>-4.4125</v>
       </c>
+      <c r="BW44" s="5" t="inlineStr"/>
       <c r="BX44" s="6">
-        <f>IF(AND(BW44&gt;$BX$12,D44&lt;=$BX$13),D43,"")</f>
+        <f>IF(AND(BV44&gt;$BX$12,D44&lt;=$BX$13),D43,"")</f>
         <v/>
       </c>
       <c r="BY44" s="6">
@@ -11211,7 +11211,7 @@
         <v/>
       </c>
       <c r="CB44" s="6">
-        <f>IF(AND(BQ44&gt;$CB$12,BS44&lt;$CB$13),E43,"")</f>
+        <f>IF(AND(BQ44&gt;$CB$12,BR44&lt;$CB$13),E43,"")</f>
         <v/>
       </c>
       <c r="CC44" s="6">
@@ -11428,24 +11428,24 @@
         <f>IF(COUNT(BA45:BA46)=2,ROUND((BA45/BA46-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR45" s="5" t="inlineStr"/>
-      <c r="BS45" s="6">
+      <c r="BR45" s="6">
         <f>IF(COUNT(BH45:BH46)=2,ROUND((BH45/BH46-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT45" s="5" t="inlineStr"/>
-      <c r="BU45" s="5" t="n">
+      <c r="BS45" s="5" t="inlineStr"/>
+      <c r="BT45" s="5" t="n">
         <v>19.49</v>
       </c>
-      <c r="BV45" s="6">
-        <f>IF(COUNT(BU45:BU46)=2,ROUND((BU45/BU46-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW45" s="6" t="n">
+      <c r="BU45" s="6">
+        <f>IF(COUNT(BT45:BT46)=2,ROUND((BT45/BT46-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV45" s="6" t="n">
         <v>12.7894</v>
       </c>
+      <c r="BW45" s="5" t="inlineStr"/>
       <c r="BX45" s="6">
-        <f>IF(AND(BW45&gt;$BX$12,D45&lt;=$BX$13),D44,"")</f>
+        <f>IF(AND(BV45&gt;$BX$12,D45&lt;=$BX$13),D44,"")</f>
         <v/>
       </c>
       <c r="BY45" s="6">
@@ -11461,7 +11461,7 @@
         <v/>
       </c>
       <c r="CB45" s="6">
-        <f>IF(AND(BQ45&gt;$CB$12,BS45&lt;$CB$13),E44,"")</f>
+        <f>IF(AND(BQ45&gt;$CB$12,BR45&lt;$CB$13),E44,"")</f>
         <v/>
       </c>
       <c r="CC45" s="6">
@@ -11678,24 +11678,24 @@
         <f>IF(COUNT(BA46:BA47)=2,ROUND((BA46/BA47-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR46" s="5" t="inlineStr"/>
-      <c r="BS46" s="6">
+      <c r="BR46" s="6">
         <f>IF(COUNT(BH46:BH47)=2,ROUND((BH46/BH47-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT46" s="5" t="inlineStr"/>
-      <c r="BU46" s="5" t="n">
+      <c r="BS46" s="5" t="inlineStr"/>
+      <c r="BT46" s="5" t="n">
         <v>17.28</v>
       </c>
-      <c r="BV46" s="6">
-        <f>IF(COUNT(BU46:BU47)=2,ROUND((BU46/BU47-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW46" s="6" t="n">
+      <c r="BU46" s="6">
+        <f>IF(COUNT(BT46:BT47)=2,ROUND((BT46/BT47-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV46" s="6" t="n">
         <v>5.3659</v>
       </c>
+      <c r="BW46" s="5" t="inlineStr"/>
       <c r="BX46" s="6">
-        <f>IF(AND(BW46&gt;$BX$12,D46&lt;=$BX$13),D45,"")</f>
+        <f>IF(AND(BV46&gt;$BX$12,D46&lt;=$BX$13),D45,"")</f>
         <v/>
       </c>
       <c r="BY46" s="6">
@@ -11711,7 +11711,7 @@
         <v/>
       </c>
       <c r="CB46" s="6">
-        <f>IF(AND(BQ46&gt;$CB$12,BS46&lt;$CB$13),E45,"")</f>
+        <f>IF(AND(BQ46&gt;$CB$12,BR46&lt;$CB$13),E45,"")</f>
         <v/>
       </c>
       <c r="CC46" s="6">
@@ -11928,24 +11928,24 @@
         <f>IF(COUNT(BA47:BA48)=2,ROUND((BA47/BA48-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR47" s="5" t="inlineStr"/>
-      <c r="BS47" s="6">
+      <c r="BR47" s="6">
         <f>IF(COUNT(BH47:BH48)=2,ROUND((BH47/BH48-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT47" s="5" t="inlineStr"/>
-      <c r="BU47" s="5" t="n">
+      <c r="BS47" s="5" t="inlineStr"/>
+      <c r="BT47" s="5" t="n">
         <v>16.4</v>
       </c>
-      <c r="BV47" s="6">
-        <f>IF(COUNT(BU47:BU48)=2,ROUND((BU47/BU48-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW47" s="6" t="n">
+      <c r="BU47" s="6">
+        <f>IF(COUNT(BT47:BT48)=2,ROUND((BT47/BT48-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV47" s="6" t="n">
         <v>-11.0629</v>
       </c>
+      <c r="BW47" s="5" t="inlineStr"/>
       <c r="BX47" s="6">
-        <f>IF(AND(BW47&gt;$BX$12,D47&lt;=$BX$13),D46,"")</f>
+        <f>IF(AND(BV47&gt;$BX$12,D47&lt;=$BX$13),D46,"")</f>
         <v/>
       </c>
       <c r="BY47" s="6">
@@ -11961,7 +11961,7 @@
         <v/>
       </c>
       <c r="CB47" s="6">
-        <f>IF(AND(BQ47&gt;$CB$12,BS47&lt;$CB$13),E46,"")</f>
+        <f>IF(AND(BQ47&gt;$CB$12,BR47&lt;$CB$13),E46,"")</f>
         <v/>
       </c>
       <c r="CC47" s="6">
@@ -12178,24 +12178,24 @@
         <f>IF(COUNT(BA48:BA49)=2,ROUND((BA48/BA49-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR48" s="5" t="inlineStr"/>
-      <c r="BS48" s="6">
+      <c r="BR48" s="6">
         <f>IF(COUNT(BH48:BH49)=2,ROUND((BH48/BH49-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT48" s="5" t="inlineStr"/>
-      <c r="BU48" s="5" t="n">
+      <c r="BS48" s="5" t="inlineStr"/>
+      <c r="BT48" s="5" t="n">
         <v>18.44</v>
       </c>
-      <c r="BV48" s="6">
-        <f>IF(COUNT(BU48:BU49)=2,ROUND((BU48/BU49-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW48" s="6" t="n">
+      <c r="BU48" s="6">
+        <f>IF(COUNT(BT48:BT49)=2,ROUND((BT48/BT49-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV48" s="6" t="n">
         <v>12.3705</v>
       </c>
+      <c r="BW48" s="5" t="inlineStr"/>
       <c r="BX48" s="6">
-        <f>IF(AND(BW48&gt;$BX$12,D48&lt;=$BX$13),D47,"")</f>
+        <f>IF(AND(BV48&gt;$BX$12,D48&lt;=$BX$13),D47,"")</f>
         <v/>
       </c>
       <c r="BY48" s="6">
@@ -12211,7 +12211,7 @@
         <v/>
       </c>
       <c r="CB48" s="6">
-        <f>IF(AND(BQ48&gt;$CB$12,BS48&lt;$CB$13),E47,"")</f>
+        <f>IF(AND(BQ48&gt;$CB$12,BR48&lt;$CB$13),E47,"")</f>
         <v/>
       </c>
       <c r="CC48" s="6">
@@ -12428,24 +12428,24 @@
         <f>IF(COUNT(BA49:BA50)=2,ROUND((BA49/BA50-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR49" s="5" t="inlineStr"/>
-      <c r="BS49" s="6">
+      <c r="BR49" s="6">
         <f>IF(COUNT(BH49:BH50)=2,ROUND((BH49/BH50-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT49" s="5" t="inlineStr"/>
-      <c r="BU49" s="5" t="n">
+      <c r="BS49" s="5" t="inlineStr"/>
+      <c r="BT49" s="5" t="n">
         <v>16.41</v>
       </c>
-      <c r="BV49" s="6">
-        <f>IF(COUNT(BU49:BU50)=2,ROUND((BU49/BU50-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW49" s="6" t="n">
+      <c r="BU49" s="6">
+        <f>IF(COUNT(BT49:BT50)=2,ROUND((BT49/BT50-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV49" s="6" t="n">
         <v>1.2963</v>
       </c>
+      <c r="BW49" s="5" t="inlineStr"/>
       <c r="BX49" s="6">
-        <f>IF(AND(BW49&gt;$BX$12,D49&lt;=$BX$13),D48,"")</f>
+        <f>IF(AND(BV49&gt;$BX$12,D49&lt;=$BX$13),D48,"")</f>
         <v/>
       </c>
       <c r="BY49" s="6">
@@ -12461,7 +12461,7 @@
         <v/>
       </c>
       <c r="CB49" s="6">
-        <f>IF(AND(BQ49&gt;$CB$12,BS49&lt;$CB$13),E48,"")</f>
+        <f>IF(AND(BQ49&gt;$CB$12,BR49&lt;$CB$13),E48,"")</f>
         <v/>
       </c>
       <c r="CC49" s="6">
@@ -12678,24 +12678,24 @@
         <f>IF(COUNT(BA50:BA51)=2,ROUND((BA50/BA51-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR50" s="5" t="inlineStr"/>
-      <c r="BS50" s="6">
+      <c r="BR50" s="6">
         <f>IF(COUNT(BH50:BH51)=2,ROUND((BH50/BH51-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT50" s="5" t="inlineStr"/>
-      <c r="BU50" s="5" t="n">
+      <c r="BS50" s="5" t="inlineStr"/>
+      <c r="BT50" s="5" t="n">
         <v>16.2</v>
       </c>
-      <c r="BV50" s="6">
-        <f>IF(COUNT(BU50:BU51)=2,ROUND((BU50/BU51-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW50" s="6" t="n">
+      <c r="BU50" s="6">
+        <f>IF(COUNT(BT50:BT51)=2,ROUND((BT50/BT51-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV50" s="6" t="n">
         <v>-8.371</v>
       </c>
+      <c r="BW50" s="5" t="inlineStr"/>
       <c r="BX50" s="6">
-        <f>IF(AND(BW50&gt;$BX$12,D50&lt;=$BX$13),D49,"")</f>
+        <f>IF(AND(BV50&gt;$BX$12,D50&lt;=$BX$13),D49,"")</f>
         <v/>
       </c>
       <c r="BY50" s="6">
@@ -12711,7 +12711,7 @@
         <v/>
       </c>
       <c r="CB50" s="6">
-        <f>IF(AND(BQ50&gt;$CB$12,BS50&lt;$CB$13),E49,"")</f>
+        <f>IF(AND(BQ50&gt;$CB$12,BR50&lt;$CB$13),E49,"")</f>
         <v/>
       </c>
       <c r="CC50" s="6">
@@ -12928,24 +12928,24 @@
         <f>IF(COUNT(BA51:BA52)=2,ROUND((BA51/BA52-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR51" s="5" t="inlineStr"/>
-      <c r="BS51" s="6">
+      <c r="BR51" s="6">
         <f>IF(COUNT(BH51:BH52)=2,ROUND((BH51/BH52-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT51" s="5" t="inlineStr"/>
-      <c r="BU51" s="5" t="n">
+      <c r="BS51" s="5" t="inlineStr"/>
+      <c r="BT51" s="5" t="n">
         <v>17.68</v>
       </c>
-      <c r="BV51" s="6">
-        <f>IF(COUNT(BU51:BU52)=2,ROUND((BU51/BU52-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW51" s="6" t="n">
+      <c r="BU51" s="6">
+        <f>IF(COUNT(BT51:BT52)=2,ROUND((BT51/BT52-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV51" s="6" t="n">
         <v>-9.0535</v>
       </c>
+      <c r="BW51" s="5" t="inlineStr"/>
       <c r="BX51" s="6">
-        <f>IF(AND(BW51&gt;$BX$12,D51&lt;=$BX$13),D50,"")</f>
+        <f>IF(AND(BV51&gt;$BX$12,D51&lt;=$BX$13),D50,"")</f>
         <v/>
       </c>
       <c r="BY51" s="6">
@@ -12961,7 +12961,7 @@
         <v/>
       </c>
       <c r="CB51" s="6">
-        <f>IF(AND(BQ51&gt;$CB$12,BS51&lt;$CB$13),E50,"")</f>
+        <f>IF(AND(BQ51&gt;$CB$12,BR51&lt;$CB$13),E50,"")</f>
         <v/>
       </c>
       <c r="CC51" s="6">
@@ -13178,24 +13178,24 @@
         <f>IF(COUNT(BA52:BA53)=2,ROUND((BA52/BA53-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR52" s="5" t="inlineStr"/>
-      <c r="BS52" s="6">
+      <c r="BR52" s="6">
         <f>IF(COUNT(BH52:BH53)=2,ROUND((BH52/BH53-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT52" s="5" t="inlineStr"/>
-      <c r="BU52" s="5" t="n">
+      <c r="BS52" s="5" t="inlineStr"/>
+      <c r="BT52" s="5" t="n">
         <v>19.44</v>
       </c>
-      <c r="BV52" s="6">
-        <f>IF(COUNT(BU52:BU53)=2,ROUND((BU52/BU53-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW52" s="6" t="n">
+      <c r="BU52" s="6">
+        <f>IF(COUNT(BT52:BT53)=2,ROUND((BT52/BT53-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV52" s="6" t="n">
         <v>-12.5113</v>
       </c>
+      <c r="BW52" s="5" t="inlineStr"/>
       <c r="BX52" s="6">
-        <f>IF(AND(BW52&gt;$BX$12,D52&lt;=$BX$13),D51,"")</f>
+        <f>IF(AND(BV52&gt;$BX$12,D52&lt;=$BX$13),D51,"")</f>
         <v/>
       </c>
       <c r="BY52" s="6">
@@ -13211,7 +13211,7 @@
         <v/>
       </c>
       <c r="CB52" s="6">
-        <f>IF(AND(BQ52&gt;$CB$12,BS52&lt;$CB$13),E51,"")</f>
+        <f>IF(AND(BQ52&gt;$CB$12,BR52&lt;$CB$13),E51,"")</f>
         <v/>
       </c>
       <c r="CC52" s="6">
@@ -13428,24 +13428,24 @@
         <f>IF(COUNT(BA53:BA54)=2,ROUND((BA53/BA54-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR53" s="5" t="inlineStr"/>
-      <c r="BS53" s="6">
+      <c r="BR53" s="6">
         <f>IF(COUNT(BH53:BH54)=2,ROUND((BH53/BH54-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT53" s="5" t="inlineStr"/>
-      <c r="BU53" s="5" t="n">
+      <c r="BS53" s="5" t="inlineStr"/>
+      <c r="BT53" s="5" t="n">
         <v>22.22</v>
       </c>
-      <c r="BV53" s="6">
-        <f>IF(COUNT(BU53:BU54)=2,ROUND((BU53/BU54-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW53" s="6" t="n">
+      <c r="BU53" s="6">
+        <f>IF(COUNT(BT53:BT54)=2,ROUND((BT53/BT54-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV53" s="6" t="n">
         <v>11.8269</v>
       </c>
+      <c r="BW53" s="5" t="inlineStr"/>
       <c r="BX53" s="6">
-        <f>IF(AND(BW53&gt;$BX$12,D53&lt;=$BX$13),D52,"")</f>
+        <f>IF(AND(BV53&gt;$BX$12,D53&lt;=$BX$13),D52,"")</f>
         <v/>
       </c>
       <c r="BY53" s="6">
@@ -13461,7 +13461,7 @@
         <v/>
       </c>
       <c r="CB53" s="6">
-        <f>IF(AND(BQ53&gt;$CB$12,BS53&lt;$CB$13),E52,"")</f>
+        <f>IF(AND(BQ53&gt;$CB$12,BR53&lt;$CB$13),E52,"")</f>
         <v/>
       </c>
       <c r="CC53" s="6">
@@ -13678,24 +13678,24 @@
         <f>IF(COUNT(BA54:BA55)=2,ROUND((BA54/BA55-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR54" s="5" t="inlineStr"/>
-      <c r="BS54" s="6">
+      <c r="BR54" s="6">
         <f>IF(COUNT(BH54:BH55)=2,ROUND((BH54/BH55-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT54" s="5" t="inlineStr"/>
-      <c r="BU54" s="5" t="n">
+      <c r="BS54" s="5" t="inlineStr"/>
+      <c r="BT54" s="5" t="n">
         <v>19.87</v>
       </c>
-      <c r="BV54" s="6">
-        <f>IF(COUNT(BU54:BU55)=2,ROUND((BU54/BU55-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW54" s="6" t="n">
+      <c r="BU54" s="6">
+        <f>IF(COUNT(BT54:BT55)=2,ROUND((BT54/BT55-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV54" s="6" t="n">
         <v>5.0211</v>
       </c>
+      <c r="BW54" s="5" t="inlineStr"/>
       <c r="BX54" s="6">
-        <f>IF(AND(BW54&gt;$BX$12,D54&lt;=$BX$13),D53,"")</f>
+        <f>IF(AND(BV54&gt;$BX$12,D54&lt;=$BX$13),D53,"")</f>
         <v/>
       </c>
       <c r="BY54" s="6">
@@ -13711,7 +13711,7 @@
         <v/>
       </c>
       <c r="CB54" s="6">
-        <f>IF(AND(BQ54&gt;$CB$12,BS54&lt;$CB$13),E53,"")</f>
+        <f>IF(AND(BQ54&gt;$CB$12,BR54&lt;$CB$13),E53,"")</f>
         <v/>
       </c>
       <c r="CC54" s="6">
@@ -13928,24 +13928,24 @@
         <f>IF(COUNT(BA55:BA56)=2,ROUND((BA55/BA56-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR55" s="5" t="inlineStr"/>
-      <c r="BS55" s="6">
+      <c r="BR55" s="6">
         <f>IF(COUNT(BH55:BH56)=2,ROUND((BH55/BH56-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT55" s="5" t="inlineStr"/>
-      <c r="BU55" s="5" t="n">
+      <c r="BS55" s="5" t="inlineStr"/>
+      <c r="BT55" s="5" t="n">
         <v>18.92</v>
       </c>
-      <c r="BV55" s="6">
-        <f>IF(COUNT(BU55:BU56)=2,ROUND((BU55/BU56-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW55" s="6" t="n">
+      <c r="BU55" s="6">
+        <f>IF(COUNT(BT55:BT56)=2,ROUND((BT55/BT56-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV55" s="6" t="n">
         <v>-12.0409</v>
       </c>
+      <c r="BW55" s="5" t="inlineStr"/>
       <c r="BX55" s="6">
-        <f>IF(AND(BW55&gt;$BX$12,D55&lt;=$BX$13),D54,"")</f>
+        <f>IF(AND(BV55&gt;$BX$12,D55&lt;=$BX$13),D54,"")</f>
         <v/>
       </c>
       <c r="BY55" s="6">
@@ -13961,7 +13961,7 @@
         <v/>
       </c>
       <c r="CB55" s="6">
-        <f>IF(AND(BQ55&gt;$CB$12,BS55&lt;$CB$13),E54,"")</f>
+        <f>IF(AND(BQ55&gt;$CB$12,BR55&lt;$CB$13),E54,"")</f>
         <v/>
       </c>
       <c r="CC55" s="6">
@@ -14178,24 +14178,24 @@
         <f>IF(COUNT(BA56:BA57)=2,ROUND((BA56/BA57-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR56" s="5" t="inlineStr"/>
-      <c r="BS56" s="6">
+      <c r="BR56" s="6">
         <f>IF(COUNT(BH56:BH57)=2,ROUND((BH56/BH57-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT56" s="5" t="inlineStr"/>
-      <c r="BU56" s="5" t="n">
+      <c r="BS56" s="5" t="inlineStr"/>
+      <c r="BT56" s="5" t="n">
         <v>21.51</v>
       </c>
-      <c r="BV56" s="6">
-        <f>IF(COUNT(BU56:BU57)=2,ROUND((BU56/BU57-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW56" s="6" t="n">
+      <c r="BU56" s="6">
+        <f>IF(COUNT(BT56:BT57)=2,ROUND((BT56/BT57-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV56" s="6" t="n">
         <v>39.6753</v>
       </c>
+      <c r="BW56" s="5" t="inlineStr"/>
       <c r="BX56" s="6">
-        <f>IF(AND(BW56&gt;$BX$12,D56&lt;=$BX$13),D55,"")</f>
+        <f>IF(AND(BV56&gt;$BX$12,D56&lt;=$BX$13),D55,"")</f>
         <v/>
       </c>
       <c r="BY56" s="6">
@@ -14211,7 +14211,7 @@
         <v/>
       </c>
       <c r="CB56" s="6">
-        <f>IF(AND(BQ56&gt;$CB$12,BS56&lt;$CB$13),E55,"")</f>
+        <f>IF(AND(BQ56&gt;$CB$12,BR56&lt;$CB$13),E55,"")</f>
         <v/>
       </c>
       <c r="CC56" s="6">
@@ -14428,24 +14428,24 @@
         <f>IF(COUNT(BA57:BA58)=2,ROUND((BA57/BA58-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR57" s="5" t="inlineStr"/>
-      <c r="BS57" s="6">
+      <c r="BR57" s="6">
         <f>IF(COUNT(BH57:BH58)=2,ROUND((BH57/BH58-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT57" s="5" t="inlineStr"/>
-      <c r="BU57" s="5" t="n">
+      <c r="BS57" s="5" t="inlineStr"/>
+      <c r="BT57" s="5" t="n">
         <v>15.4</v>
       </c>
-      <c r="BV57" s="6">
-        <f>IF(COUNT(BU57:BU58)=2,ROUND((BU57/BU58-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW57" s="6" t="n">
+      <c r="BU57" s="6">
+        <f>IF(COUNT(BT57:BT58)=2,ROUND((BT57/BT58-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV57" s="6" t="n">
         <v>-4.1096</v>
       </c>
+      <c r="BW57" s="5" t="inlineStr"/>
       <c r="BX57" s="6">
-        <f>IF(AND(BW57&gt;$BX$12,D57&lt;=$BX$13),D56,"")</f>
+        <f>IF(AND(BV57&gt;$BX$12,D57&lt;=$BX$13),D56,"")</f>
         <v/>
       </c>
       <c r="BY57" s="6">
@@ -14461,7 +14461,7 @@
         <v/>
       </c>
       <c r="CB57" s="6">
-        <f>IF(AND(BQ57&gt;$CB$12,BS57&lt;$CB$13),E56,"")</f>
+        <f>IF(AND(BQ57&gt;$CB$12,BR57&lt;$CB$13),E56,"")</f>
         <v/>
       </c>
       <c r="CC57" s="6">
@@ -14678,24 +14678,24 @@
         <f>IF(COUNT(BA58:BA59)=2,ROUND((BA58/BA59-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR58" s="5" t="inlineStr"/>
-      <c r="BS58" s="6">
+      <c r="BR58" s="6">
         <f>IF(COUNT(BH58:BH59)=2,ROUND((BH58/BH59-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT58" s="5" t="inlineStr"/>
-      <c r="BU58" s="5" t="n">
+      <c r="BS58" s="5" t="inlineStr"/>
+      <c r="BT58" s="5" t="n">
         <v>16.06</v>
       </c>
-      <c r="BV58" s="6">
-        <f>IF(COUNT(BU58:BU59)=2,ROUND((BU58/BU59-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW58" s="6" t="n">
+      <c r="BU58" s="6">
+        <f>IF(COUNT(BT58:BT59)=2,ROUND((BT58/BT59-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV58" s="6" t="n">
         <v>1.8389</v>
       </c>
+      <c r="BW58" s="5" t="inlineStr"/>
       <c r="BX58" s="6">
-        <f>IF(AND(BW58&gt;$BX$12,D58&lt;=$BX$13),D57,"")</f>
+        <f>IF(AND(BV58&gt;$BX$12,D58&lt;=$BX$13),D57,"")</f>
         <v/>
       </c>
       <c r="BY58" s="6">
@@ -14711,7 +14711,7 @@
         <v/>
       </c>
       <c r="CB58" s="6">
-        <f>IF(AND(BQ58&gt;$CB$12,BS58&lt;$CB$13),E57,"")</f>
+        <f>IF(AND(BQ58&gt;$CB$12,BR58&lt;$CB$13),E57,"")</f>
         <v/>
       </c>
       <c r="CC58" s="6">
@@ -14928,24 +14928,24 @@
         <f>IF(COUNT(BA59:BA60)=2,ROUND((BA59/BA60-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR59" s="5" t="inlineStr"/>
-      <c r="BS59" s="6">
+      <c r="BR59" s="6">
         <f>IF(COUNT(BH59:BH60)=2,ROUND((BH59/BH60-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT59" s="5" t="inlineStr"/>
-      <c r="BU59" s="5" t="n">
+      <c r="BS59" s="5" t="inlineStr"/>
+      <c r="BT59" s="5" t="n">
         <v>15.77</v>
       </c>
-      <c r="BV59" s="6">
-        <f>IF(COUNT(BU59:BU60)=2,ROUND((BU59/BU60-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW59" s="6" t="n">
+      <c r="BU59" s="6">
+        <f>IF(COUNT(BT59:BT60)=2,ROUND((BT59/BT60-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV59" s="6" t="n">
         <v>-1.7445</v>
       </c>
+      <c r="BW59" s="5" t="inlineStr"/>
       <c r="BX59" s="6">
-        <f>IF(AND(BW59&gt;$BX$12,D59&lt;=$BX$13),D58,"")</f>
+        <f>IF(AND(BV59&gt;$BX$12,D59&lt;=$BX$13),D58,"")</f>
         <v/>
       </c>
       <c r="BY59" s="6">
@@ -14961,7 +14961,7 @@
         <v/>
       </c>
       <c r="CB59" s="6">
-        <f>IF(AND(BQ59&gt;$CB$12,BS59&lt;$CB$13),E58,"")</f>
+        <f>IF(AND(BQ59&gt;$CB$12,BR59&lt;$CB$13),E58,"")</f>
         <v/>
       </c>
       <c r="CC59" s="6">
@@ -15178,24 +15178,24 @@
         <f>IF(COUNT(BA60:BA61)=2,ROUND((BA60/BA61-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR60" s="5" t="inlineStr"/>
-      <c r="BS60" s="6">
+      <c r="BR60" s="6">
         <f>IF(COUNT(BH60:BH61)=2,ROUND((BH60/BH61-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT60" s="5" t="inlineStr"/>
-      <c r="BU60" s="5" t="n">
+      <c r="BS60" s="5" t="inlineStr"/>
+      <c r="BT60" s="5" t="n">
         <v>16.05</v>
       </c>
-      <c r="BV60" s="6">
-        <f>IF(COUNT(BU60:BU61)=2,ROUND((BU60/BU61-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW60" s="6" t="n">
+      <c r="BU60" s="6">
+        <f>IF(COUNT(BT60:BT61)=2,ROUND((BT60/BT61-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV60" s="6" t="n">
         <v>4.765</v>
       </c>
+      <c r="BW60" s="5" t="inlineStr"/>
       <c r="BX60" s="6">
-        <f>IF(AND(BW60&gt;$BX$12,D60&lt;=$BX$13),D59,"")</f>
+        <f>IF(AND(BV60&gt;$BX$12,D60&lt;=$BX$13),D59,"")</f>
         <v/>
       </c>
       <c r="BY60" s="6">
@@ -15211,7 +15211,7 @@
         <v/>
       </c>
       <c r="CB60" s="6">
-        <f>IF(AND(BQ60&gt;$CB$12,BS60&lt;$CB$13),E59,"")</f>
+        <f>IF(AND(BQ60&gt;$CB$12,BR60&lt;$CB$13),E59,"")</f>
         <v/>
       </c>
       <c r="CC60" s="6">
@@ -15428,24 +15428,24 @@
         <f>IF(COUNT(BA61:BA62)=2,ROUND((BA61/BA62-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR61" s="5" t="inlineStr"/>
-      <c r="BS61" s="6">
+      <c r="BR61" s="6">
         <f>IF(COUNT(BH61:BH62)=2,ROUND((BH61/BH62-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT61" s="5" t="inlineStr"/>
-      <c r="BU61" s="5" t="n">
+      <c r="BS61" s="5" t="inlineStr"/>
+      <c r="BT61" s="5" t="n">
         <v>15.32</v>
       </c>
-      <c r="BV61" s="6">
-        <f>IF(COUNT(BU61:BU62)=2,ROUND((BU61/BU62-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW61" s="6" t="n">
+      <c r="BU61" s="6">
+        <f>IF(COUNT(BT61:BT62)=2,ROUND((BT61/BT62-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV61" s="6" t="n">
         <v>-2.6684</v>
       </c>
+      <c r="BW61" s="5" t="inlineStr"/>
       <c r="BX61" s="6">
-        <f>IF(AND(BW61&gt;$BX$12,D61&lt;=$BX$13),D60,"")</f>
+        <f>IF(AND(BV61&gt;$BX$12,D61&lt;=$BX$13),D60,"")</f>
         <v/>
       </c>
       <c r="BY61" s="6">
@@ -15461,7 +15461,7 @@
         <v/>
       </c>
       <c r="CB61" s="6">
-        <f>IF(AND(BQ61&gt;$CB$12,BS61&lt;$CB$13),E60,"")</f>
+        <f>IF(AND(BQ61&gt;$CB$12,BR61&lt;$CB$13),E60,"")</f>
         <v/>
       </c>
       <c r="CC61" s="6">
@@ -15678,24 +15678,24 @@
         <f>IF(COUNT(BA62:BA63)=2,ROUND((BA62/BA63-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR62" s="5" t="inlineStr"/>
-      <c r="BS62" s="6">
+      <c r="BR62" s="6">
         <f>IF(COUNT(BH62:BH63)=2,ROUND((BH62/BH63-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT62" s="5" t="inlineStr"/>
-      <c r="BU62" s="5" t="n">
+      <c r="BS62" s="5" t="inlineStr"/>
+      <c r="BT62" s="5" t="n">
         <v>15.74</v>
       </c>
-      <c r="BV62" s="6">
-        <f>IF(COUNT(BU62:BU63)=2,ROUND((BU62/BU63-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW62" s="6" t="n">
+      <c r="BU62" s="6">
+        <f>IF(COUNT(BT62:BT63)=2,ROUND((BT62/BT63-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV62" s="6" t="n">
         <v>-3.3763</v>
       </c>
+      <c r="BW62" s="5" t="inlineStr"/>
       <c r="BX62" s="6">
-        <f>IF(AND(BW62&gt;$BX$12,D62&lt;=$BX$13),D61,"")</f>
+        <f>IF(AND(BV62&gt;$BX$12,D62&lt;=$BX$13),D61,"")</f>
         <v/>
       </c>
       <c r="BY62" s="6">
@@ -15711,7 +15711,7 @@
         <v/>
       </c>
       <c r="CB62" s="6">
-        <f>IF(AND(BQ62&gt;$CB$12,BS62&lt;$CB$13),E61,"")</f>
+        <f>IF(AND(BQ62&gt;$CB$12,BR62&lt;$CB$13),E61,"")</f>
         <v/>
       </c>
       <c r="CC62" s="6">
@@ -15928,24 +15928,24 @@
         <f>IF(COUNT(BA63:BA64)=2,ROUND((BA63/BA64-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR63" s="5" t="inlineStr"/>
-      <c r="BS63" s="6">
+      <c r="BR63" s="6">
         <f>IF(COUNT(BH63:BH64)=2,ROUND((BH63/BH64-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT63" s="5" t="inlineStr"/>
-      <c r="BU63" s="5" t="n">
+      <c r="BS63" s="5" t="inlineStr"/>
+      <c r="BT63" s="5" t="n">
         <v>16.29</v>
       </c>
-      <c r="BV63" s="6">
-        <f>IF(COUNT(BU63:BU64)=2,ROUND((BU63/BU64-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW63" s="6" t="n">
+      <c r="BU63" s="6">
+        <f>IF(COUNT(BT63:BT64)=2,ROUND((BT63/BT64-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV63" s="6" t="n">
         <v>-4.2328</v>
       </c>
+      <c r="BW63" s="5" t="inlineStr"/>
       <c r="BX63" s="6">
-        <f>IF(AND(BW63&gt;$BX$12,D63&lt;=$BX$13),D62,"")</f>
+        <f>IF(AND(BV63&gt;$BX$12,D63&lt;=$BX$13),D62,"")</f>
         <v/>
       </c>
       <c r="BY63" s="6">
@@ -15961,7 +15961,7 @@
         <v/>
       </c>
       <c r="CB63" s="6">
-        <f>IF(AND(BQ63&gt;$CB$12,BS63&lt;$CB$13),E62,"")</f>
+        <f>IF(AND(BQ63&gt;$CB$12,BR63&lt;$CB$13),E62,"")</f>
         <v/>
       </c>
       <c r="CC63" s="6">
@@ -16178,24 +16178,24 @@
         <f>IF(COUNT(BA64:BA65)=2,ROUND((BA64/BA65-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR64" s="5" t="inlineStr"/>
-      <c r="BS64" s="6">
+      <c r="BR64" s="6">
         <f>IF(COUNT(BH64:BH65)=2,ROUND((BH64/BH65-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT64" s="5" t="inlineStr"/>
-      <c r="BU64" s="5" t="n">
+      <c r="BS64" s="5" t="inlineStr"/>
+      <c r="BT64" s="5" t="n">
         <v>17.01</v>
       </c>
-      <c r="BV64" s="6">
-        <f>IF(COUNT(BU64:BU65)=2,ROUND((BU64/BU65-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW64" s="6" t="n">
+      <c r="BU64" s="6">
+        <f>IF(COUNT(BT64:BT65)=2,ROUND((BT64/BT65-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV64" s="6" t="n">
         <v>1.8563</v>
       </c>
+      <c r="BW64" s="5" t="inlineStr"/>
       <c r="BX64" s="6">
-        <f>IF(AND(BW64&gt;$BX$12,D64&lt;=$BX$13),D63,"")</f>
+        <f>IF(AND(BV64&gt;$BX$12,D64&lt;=$BX$13),D63,"")</f>
         <v/>
       </c>
       <c r="BY64" s="6">
@@ -16211,7 +16211,7 @@
         <v/>
       </c>
       <c r="CB64" s="6">
-        <f>IF(AND(BQ64&gt;$CB$12,BS64&lt;$CB$13),E63,"")</f>
+        <f>IF(AND(BQ64&gt;$CB$12,BR64&lt;$CB$13),E63,"")</f>
         <v/>
       </c>
       <c r="CC64" s="6">
@@ -16428,24 +16428,24 @@
         <f>IF(COUNT(BA65:BA66)=2,ROUND((BA65/BA66-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR65" s="5" t="inlineStr"/>
-      <c r="BS65" s="6">
+      <c r="BR65" s="6">
         <f>IF(COUNT(BH65:BH66)=2,ROUND((BH65/BH66-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT65" s="5" t="inlineStr"/>
-      <c r="BU65" s="5" t="n">
+      <c r="BS65" s="5" t="inlineStr"/>
+      <c r="BT65" s="5" t="n">
         <v>16.7</v>
       </c>
-      <c r="BV65" s="6">
-        <f>IF(COUNT(BU65:BU66)=2,ROUND((BU65/BU66-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW65" s="6" t="n">
+      <c r="BU65" s="6">
+        <f>IF(COUNT(BT65:BT66)=2,ROUND((BT65/BT66-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV65" s="6" t="n">
         <v>-0.358</v>
       </c>
+      <c r="BW65" s="5" t="inlineStr"/>
       <c r="BX65" s="6">
-        <f>IF(AND(BW65&gt;$BX$12,D65&lt;=$BX$13),D64,"")</f>
+        <f>IF(AND(BV65&gt;$BX$12,D65&lt;=$BX$13),D64,"")</f>
         <v/>
       </c>
       <c r="BY65" s="6">
@@ -16461,7 +16461,7 @@
         <v/>
       </c>
       <c r="CB65" s="6">
-        <f>IF(AND(BQ65&gt;$CB$12,BS65&lt;$CB$13),E64,"")</f>
+        <f>IF(AND(BQ65&gt;$CB$12,BR65&lt;$CB$13),E64,"")</f>
         <v/>
       </c>
       <c r="CC65" s="6">
@@ -16678,24 +16678,24 @@
         <f>IF(COUNT(BA66:BA67)=2,ROUND((BA66/BA67-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR66" s="5" t="inlineStr"/>
-      <c r="BS66" s="6">
+      <c r="BR66" s="6">
         <f>IF(COUNT(BH66:BH67)=2,ROUND((BH66/BH67-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT66" s="5" t="inlineStr"/>
-      <c r="BU66" s="5" t="n">
+      <c r="BS66" s="5" t="inlineStr"/>
+      <c r="BT66" s="5" t="n">
         <v>16.76</v>
       </c>
-      <c r="BV66" s="6">
-        <f>IF(COUNT(BU66:BU67)=2,ROUND((BU66/BU67-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW66" s="6" t="n">
+      <c r="BU66" s="6">
+        <f>IF(COUNT(BT66:BT67)=2,ROUND((BT66/BT67-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV66" s="6" t="n">
         <v>-3.8991</v>
       </c>
+      <c r="BW66" s="5" t="inlineStr"/>
       <c r="BX66" s="6">
-        <f>IF(AND(BW66&gt;$BX$12,D66&lt;=$BX$13),D65,"")</f>
+        <f>IF(AND(BV66&gt;$BX$12,D66&lt;=$BX$13),D65,"")</f>
         <v/>
       </c>
       <c r="BY66" s="6">
@@ -16711,7 +16711,7 @@
         <v/>
       </c>
       <c r="CB66" s="6">
-        <f>IF(AND(BQ66&gt;$CB$12,BS66&lt;$CB$13),E65,"")</f>
+        <f>IF(AND(BQ66&gt;$CB$12,BR66&lt;$CB$13),E65,"")</f>
         <v/>
       </c>
       <c r="CC66" s="6">
@@ -16928,24 +16928,24 @@
         <f>IF(COUNT(BA67:BA68)=2,ROUND((BA67/BA68-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR67" s="5" t="inlineStr"/>
-      <c r="BS67" s="6">
+      <c r="BR67" s="6">
         <f>IF(COUNT(BH67:BH68)=2,ROUND((BH67/BH68-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT67" s="5" t="inlineStr"/>
-      <c r="BU67" s="5" t="n">
+      <c r="BS67" s="5" t="inlineStr"/>
+      <c r="BT67" s="5" t="n">
         <v>17.44</v>
       </c>
-      <c r="BV67" s="6">
-        <f>IF(COUNT(BU67:BU68)=2,ROUND((BU67/BU68-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW67" s="6" t="n">
+      <c r="BU67" s="6">
+        <f>IF(COUNT(BT67:BT68)=2,ROUND((BT67/BT68-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV67" s="6" t="n">
         <v>-3.433</v>
       </c>
+      <c r="BW67" s="5" t="inlineStr"/>
       <c r="BX67" s="6">
-        <f>IF(AND(BW67&gt;$BX$12,D67&lt;=$BX$13),D66,"")</f>
+        <f>IF(AND(BV67&gt;$BX$12,D67&lt;=$BX$13),D66,"")</f>
         <v/>
       </c>
       <c r="BY67" s="6">
@@ -16961,7 +16961,7 @@
         <v/>
       </c>
       <c r="CB67" s="6">
-        <f>IF(AND(BQ67&gt;$CB$12,BS67&lt;$CB$13),E66,"")</f>
+        <f>IF(AND(BQ67&gt;$CB$12,BR67&lt;$CB$13),E66,"")</f>
         <v/>
       </c>
       <c r="CC67" s="6">
@@ -17178,24 +17178,24 @@
         <f>IF(COUNT(BA68:BA69)=2,ROUND((BA68/BA69-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR68" s="5" t="inlineStr"/>
-      <c r="BS68" s="6">
+      <c r="BR68" s="6">
         <f>IF(COUNT(BH68:BH69)=2,ROUND((BH68/BH69-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT68" s="5" t="inlineStr"/>
-      <c r="BU68" s="5" t="n">
+      <c r="BS68" s="5" t="inlineStr"/>
+      <c r="BT68" s="5" t="n">
         <v>18.06</v>
       </c>
-      <c r="BV68" s="6">
-        <f>IF(COUNT(BU68:BU69)=2,ROUND((BU68/BU69-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW68" s="6" t="n">
+      <c r="BU68" s="6">
+        <f>IF(COUNT(BT68:BT69)=2,ROUND((BT68/BT69-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV68" s="6" t="n">
         <v>1.3468</v>
       </c>
+      <c r="BW68" s="5" t="inlineStr"/>
       <c r="BX68" s="6">
-        <f>IF(AND(BW68&gt;$BX$12,D68&lt;=$BX$13),D67,"")</f>
+        <f>IF(AND(BV68&gt;$BX$12,D68&lt;=$BX$13),D67,"")</f>
         <v/>
       </c>
       <c r="BY68" s="6">
@@ -17211,7 +17211,7 @@
         <v/>
       </c>
       <c r="CB68" s="6">
-        <f>IF(AND(BQ68&gt;$CB$12,BS68&lt;$CB$13),E67,"")</f>
+        <f>IF(AND(BQ68&gt;$CB$12,BR68&lt;$CB$13),E67,"")</f>
         <v/>
       </c>
       <c r="CC68" s="6">
@@ -17428,24 +17428,24 @@
         <f>IF(COUNT(BA69:BA70)=2,ROUND((BA69/BA70-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR69" s="5" t="inlineStr"/>
-      <c r="BS69" s="6">
+      <c r="BR69" s="6">
         <f>IF(COUNT(BH69:BH70)=2,ROUND((BH69/BH70-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT69" s="5" t="inlineStr"/>
-      <c r="BU69" s="5" t="n">
+      <c r="BS69" s="5" t="inlineStr"/>
+      <c r="BT69" s="5" t="n">
         <v>17.82</v>
       </c>
-      <c r="BV69" s="6">
-        <f>IF(COUNT(BU69:BU70)=2,ROUND((BU69/BU70-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW69" s="6" t="n">
+      <c r="BU69" s="6">
+        <f>IF(COUNT(BT69:BT70)=2,ROUND((BT69/BT70-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV69" s="6" t="n">
         <v>-3.3098</v>
       </c>
+      <c r="BW69" s="5" t="inlineStr"/>
       <c r="BX69" s="6">
-        <f>IF(AND(BW69&gt;$BX$12,D69&lt;=$BX$13),D68,"")</f>
+        <f>IF(AND(BV69&gt;$BX$12,D69&lt;=$BX$13),D68,"")</f>
         <v/>
       </c>
       <c r="BY69" s="6">
@@ -17461,7 +17461,7 @@
         <v/>
       </c>
       <c r="CB69" s="6">
-        <f>IF(AND(BQ69&gt;$CB$12,BS69&lt;$CB$13),E68,"")</f>
+        <f>IF(AND(BQ69&gt;$CB$12,BR69&lt;$CB$13),E68,"")</f>
         <v/>
       </c>
       <c r="CC69" s="6">
@@ -17678,24 +17678,24 @@
         <f>IF(COUNT(BA70:BA71)=2,ROUND((BA70/BA71-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR70" s="5" t="inlineStr"/>
-      <c r="BS70" s="6">
+      <c r="BR70" s="6">
         <f>IF(COUNT(BH70:BH71)=2,ROUND((BH70/BH71-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT70" s="5" t="inlineStr"/>
-      <c r="BU70" s="5" t="n">
+      <c r="BS70" s="5" t="inlineStr"/>
+      <c r="BT70" s="5" t="n">
         <v>18.43</v>
       </c>
-      <c r="BV70" s="6">
-        <f>IF(COUNT(BU70:BU71)=2,ROUND((BU70/BU71-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW70" s="6" t="n">
+      <c r="BU70" s="6">
+        <f>IF(COUNT(BT70:BT71)=2,ROUND((BT70/BT71-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV70" s="6" t="n">
         <v>6.7787</v>
       </c>
+      <c r="BW70" s="5" t="inlineStr"/>
       <c r="BX70" s="6">
-        <f>IF(AND(BW70&gt;$BX$12,D70&lt;=$BX$13),D69,"")</f>
+        <f>IF(AND(BV70&gt;$BX$12,D70&lt;=$BX$13),D69,"")</f>
         <v/>
       </c>
       <c r="BY70" s="6">
@@ -17711,7 +17711,7 @@
         <v/>
       </c>
       <c r="CB70" s="6">
-        <f>IF(AND(BQ70&gt;$CB$12,BS70&lt;$CB$13),E69,"")</f>
+        <f>IF(AND(BQ70&gt;$CB$12,BR70&lt;$CB$13),E69,"")</f>
         <v/>
       </c>
       <c r="CC70" s="6">
@@ -17928,24 +17928,24 @@
         <f>IF(COUNT(BA71:BA72)=2,ROUND((BA71/BA72-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR71" s="5" t="inlineStr"/>
-      <c r="BS71" s="6">
+      <c r="BR71" s="6">
         <f>IF(COUNT(BH71:BH72)=2,ROUND((BH71/BH72-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT71" s="5" t="inlineStr"/>
-      <c r="BU71" s="5" t="n">
+      <c r="BS71" s="5" t="inlineStr"/>
+      <c r="BT71" s="5" t="n">
         <v>17.26</v>
       </c>
-      <c r="BV71" s="6">
-        <f>IF(COUNT(BU71:BU72)=2,ROUND((BU71/BU72-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW71" s="6" t="n">
+      <c r="BU71" s="6">
+        <f>IF(COUNT(BT71:BT72)=2,ROUND((BT71/BT72-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV71" s="6" t="n">
         <v>-3.4135</v>
       </c>
+      <c r="BW71" s="5" t="inlineStr"/>
       <c r="BX71" s="6">
-        <f>IF(AND(BW71&gt;$BX$12,D71&lt;=$BX$13),D70,"")</f>
+        <f>IF(AND(BV71&gt;$BX$12,D71&lt;=$BX$13),D70,"")</f>
         <v/>
       </c>
       <c r="BY71" s="6">
@@ -17961,7 +17961,7 @@
         <v/>
       </c>
       <c r="CB71" s="6">
-        <f>IF(AND(BQ71&gt;$CB$12,BS71&lt;$CB$13),E70,"")</f>
+        <f>IF(AND(BQ71&gt;$CB$12,BR71&lt;$CB$13),E70,"")</f>
         <v/>
       </c>
       <c r="CC71" s="6">
@@ -18178,24 +18178,24 @@
         <f>IF(COUNT(BA72:BA73)=2,ROUND((BA72/BA73-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR72" s="5" t="inlineStr"/>
-      <c r="BS72" s="6">
+      <c r="BR72" s="6">
         <f>IF(COUNT(BH72:BH73)=2,ROUND((BH72/BH73-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT72" s="5" t="inlineStr"/>
-      <c r="BU72" s="5" t="n">
+      <c r="BS72" s="5" t="inlineStr"/>
+      <c r="BT72" s="5" t="n">
         <v>17.87</v>
       </c>
-      <c r="BV72" s="6">
-        <f>IF(COUNT(BU72:BU73)=2,ROUND((BU72/BU73-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW72" s="6" t="n">
+      <c r="BU72" s="6">
+        <f>IF(COUNT(BT72:BT73)=2,ROUND((BT72/BT73-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV72" s="6" t="n">
         <v>-0.667</v>
       </c>
+      <c r="BW72" s="5" t="inlineStr"/>
       <c r="BX72" s="6">
-        <f>IF(AND(BW72&gt;$BX$12,D72&lt;=$BX$13),D71,"")</f>
+        <f>IF(AND(BV72&gt;$BX$12,D72&lt;=$BX$13),D71,"")</f>
         <v/>
       </c>
       <c r="BY72" s="6">
@@ -18211,7 +18211,7 @@
         <v/>
       </c>
       <c r="CB72" s="6">
-        <f>IF(AND(BQ72&gt;$CB$12,BS72&lt;$CB$13),E71,"")</f>
+        <f>IF(AND(BQ72&gt;$CB$12,BR72&lt;$CB$13),E71,"")</f>
         <v/>
       </c>
       <c r="CC72" s="6">
@@ -18428,24 +18428,24 @@
         <f>IF(COUNT(BA73:BA74)=2,ROUND((BA73/BA74-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR73" s="5" t="inlineStr"/>
-      <c r="BS73" s="6">
+      <c r="BR73" s="6">
         <f>IF(COUNT(BH73:BH74)=2,ROUND((BH73/BH74-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT73" s="5" t="inlineStr"/>
-      <c r="BU73" s="5" t="n">
+      <c r="BS73" s="5" t="inlineStr"/>
+      <c r="BT73" s="5" t="n">
         <v>17.99</v>
       </c>
-      <c r="BV73" s="6">
-        <f>IF(COUNT(BU73:BU74)=2,ROUND((BU73/BU74-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW73" s="6" t="n">
+      <c r="BU73" s="6">
+        <f>IF(COUNT(BT73:BT74)=2,ROUND((BT73/BT74-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV73" s="6" t="n">
         <v>-2.1219</v>
       </c>
+      <c r="BW73" s="5" t="inlineStr"/>
       <c r="BX73" s="6">
-        <f>IF(AND(BW73&gt;$BX$12,D73&lt;=$BX$13),D72,"")</f>
+        <f>IF(AND(BV73&gt;$BX$12,D73&lt;=$BX$13),D72,"")</f>
         <v/>
       </c>
       <c r="BY73" s="6">
@@ -18461,7 +18461,7 @@
         <v/>
       </c>
       <c r="CB73" s="6">
-        <f>IF(AND(BQ73&gt;$CB$12,BS73&lt;$CB$13),E72,"")</f>
+        <f>IF(AND(BQ73&gt;$CB$12,BR73&lt;$CB$13),E72,"")</f>
         <v/>
       </c>
       <c r="CC73" s="6">
@@ -18678,24 +18678,24 @@
         <f>IF(COUNT(BA74:BA75)=2,ROUND((BA74/BA75-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BR74" s="5" t="inlineStr"/>
-      <c r="BS74" s="6">
+      <c r="BR74" s="6">
         <f>IF(COUNT(BH74:BH75)=2,ROUND((BH74/BH75-1)*100,4),"")</f>
         <v/>
       </c>
-      <c r="BT74" s="5" t="inlineStr"/>
-      <c r="BU74" s="5" t="n">
+      <c r="BS74" s="5" t="inlineStr"/>
+      <c r="BT74" s="5" t="n">
         <v>18.38</v>
       </c>
-      <c r="BV74" s="6">
-        <f>IF(COUNT(BU74:BU75)=2,ROUND((BU74/BU75-1)*100,4),"")</f>
-        <v/>
-      </c>
-      <c r="BW74" s="6" t="n">
+      <c r="BU74" s="6">
+        <f>IF(COUNT(BT74:BT75)=2,ROUND((BT74/BT75-1)*100,4),"")</f>
+        <v/>
+      </c>
+      <c r="BV74" s="6" t="n">
         <v>6.9226</v>
       </c>
+      <c r="BW74" s="5" t="inlineStr"/>
       <c r="BX74" s="6">
-        <f>IF(AND(BW74&gt;$BX$12,D74&lt;=$BX$13),D73,"")</f>
+        <f>IF(AND(BV74&gt;$BX$12,D74&lt;=$BX$13),D73,"")</f>
         <v/>
       </c>
       <c r="BY74" s="6">
@@ -18711,7 +18711,7 @@
         <v/>
       </c>
       <c r="CB74" s="6">
-        <f>IF(AND(BQ74&gt;$CB$12,BS74&lt;$CB$13),E73,"")</f>
+        <f>IF(AND(BQ74&gt;$CB$12,BR74&lt;$CB$13),E73,"")</f>
         <v/>
       </c>
       <c r="CC74" s="6">
@@ -18901,18 +18901,18 @@
       <c r="BO75" s="6" t="inlineStr"/>
       <c r="BP75" s="6" t="inlineStr"/>
       <c r="BQ75" s="6" t="inlineStr"/>
-      <c r="BR75" s="5" t="inlineStr"/>
-      <c r="BS75" s="6" t="inlineStr"/>
-      <c r="BT75" s="5" t="inlineStr"/>
-      <c r="BU75" s="5" t="n">
+      <c r="BR75" s="6" t="inlineStr"/>
+      <c r="BS75" s="5" t="inlineStr"/>
+      <c r="BT75" s="5" t="n">
         <v>17.19</v>
       </c>
-      <c r="BV75" s="6" t="inlineStr"/>
-      <c r="BW75" s="6" t="n">
+      <c r="BU75" s="6" t="inlineStr"/>
+      <c r="BV75" s="6" t="n">
         <v>0.644</v>
       </c>
+      <c r="BW75" s="5" t="inlineStr"/>
       <c r="BX75" s="6">
-        <f>IF(AND(BW75&gt;$BX$12,D75&lt;=$BX$13),D74,"")</f>
+        <f>IF(AND(BV75&gt;$BX$12,D75&lt;=$BX$13),D74,"")</f>
         <v/>
       </c>
       <c r="BY75" s="6">
@@ -18928,7 +18928,7 @@
         <v/>
       </c>
       <c r="CB75" s="6">
-        <f>IF(AND(BQ75&gt;$CB$12,BS75&lt;$CB$13),E74,"")</f>
+        <f>IF(AND(BQ75&gt;$CB$12,BR75&lt;$CB$13),E74,"")</f>
         <v/>
       </c>
       <c r="CC75" s="6">

</xml_diff>